<commit_message>
Ergänzung Heatpump in Datenbank
</commit_message>
<xml_diff>
--- a/Methanol_DAC_Greenfield_Patagonien/Datenbank.xlsx
+++ b/Methanol_DAC_Greenfield_Patagonien/Datenbank.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\01-Arbeit\06-FENES\09-P2X3\FENES_P2X\Methanol_DAC_Greenfield_Patagonien\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E76ECB87-727C-4C09-BD07-57DEE6B16246}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15E961C6-683D-4E50-A982-1085A77723A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Datenauswahl" sheetId="1" r:id="rId1"/>
     <sheet name="Ergebnisse" sheetId="5" r:id="rId2"/>
-    <sheet name="DAC Quelle" sheetId="6" r:id="rId3"/>
+    <sheet name="Quelle" sheetId="6" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,6 +42,8 @@
   <authors>
     <author>tc={AFE4F70E-4F68-4601-B8CF-DFA896FC8A62}</author>
     <author>tc={50E20A73-76EE-480B-AC2B-85B9568229B3}</author>
+    <author>tc={A66B6FDD-7E3A-402B-8E6B-7073C79B9436}</author>
+    <author>tc={5F7F21A6-9267-43AB-9E2F-857C43A6B051}</author>
     <author>tc={87F94307-F9C1-413A-A184-19A69689A8AF}</author>
     <author>tc={011C4874-472E-423F-9F9E-1A44747EBF50}</author>
     <author>Timon Geiß</author>
@@ -64,7 +66,23 @@
     Die Methanol-Synthese benötigt 1,375 kg CO₂ pro kg Methanol (CH₃OH) unter idealen stöchiometrischen Bedingungen. Dies ergibt sich aus der Reaktionsgleichung der CO₂-Hydrierung </t>
       </text>
     </comment>
-    <comment ref="E24" authorId="2" shapeId="0" xr:uid="{87F94307-F9C1-413A-A184-19A69689A8AF}">
+    <comment ref="E18" authorId="2" shapeId="0" xr:uid="{A66B6FDD-7E3A-402B-8E6B-7073C79B9436}">
+      <text>
+        <t xml:space="preserve">[Kommentarthread]
+Ihre Version von Excel gestattet Ihnen das Lesen dieses Kommentarthreads. Jegliche Bearbeitungen daran werden jedoch entfernt, wenn die Datei in einer neueren Version von Excel geöffnet wird. Weitere Informationen: https://go.microsoft.com/fwlink/?linkid=870924.
+Kommentar:
+    0,7 * 10^6 /1000 </t>
+      </text>
+    </comment>
+    <comment ref="E23" authorId="3" shapeId="0" xr:uid="{5F7F21A6-9267-43AB-9E2F-857C43A6B051}">
+      <text>
+        <t>[Kommentarthread]
+Ihre Version von Excel gestattet Ihnen das Lesen dieses Kommentarthreads. Jegliche Bearbeitungen daran werden jedoch entfernt, wenn die Datei in einer neueren Version von Excel geöffnet wird. Weitere Informationen: https://go.microsoft.com/fwlink/?linkid=870924.
+Kommentar:
+    1750 kWh_th/t durch 1000</t>
+      </text>
+    </comment>
+    <comment ref="E24" authorId="4" shapeId="0" xr:uid="{87F94307-F9C1-413A-A184-19A69689A8AF}">
       <text>
         <t>[Kommentarthread]
 Ihre Version von Excel gestattet Ihnen das Lesen dieses Kommentarthreads. Jegliche Bearbeitungen daran werden jedoch entfernt, wenn die Datei in einer neueren Version von Excel geöffnet wird. Weitere Informationen: https://go.microsoft.com/fwlink/?linkid=870924.
@@ -72,7 +90,7 @@
     800 €/t*a * 8760 h/a / 1000 kg/t = €/kg *h</t>
       </text>
     </comment>
-    <comment ref="E25" authorId="3" shapeId="0" xr:uid="{011C4874-472E-423F-9F9E-1A44747EBF50}">
+    <comment ref="E25" authorId="5" shapeId="0" xr:uid="{011C4874-472E-423F-9F9E-1A44747EBF50}">
       <text>
         <t>[Kommentarthread]
 Ihre Version von Excel gestattet Ihnen das Lesen dieses Kommentarthreads. Jegliche Bearbeitungen daran werden jedoch entfernt, wenn die Datei in einer neueren Version von Excel geöffnet wird. Weitere Informationen: https://go.microsoft.com/fwlink/?linkid=870924.
@@ -80,7 +98,7 @@
     ~ 40 opex/ 800 capex</t>
       </text>
     </comment>
-    <comment ref="E42" authorId="4" shapeId="0" xr:uid="{22946658-3822-4C9A-8007-CC034FA9B8AB}">
+    <comment ref="E42" authorId="6" shapeId="0" xr:uid="{22946658-3822-4C9A-8007-CC034FA9B8AB}">
       <text>
         <r>
           <rPr>
@@ -104,7 +122,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E43" authorId="4" shapeId="0" xr:uid="{426A9046-86EB-4AF9-8A2D-1FEFC7B6C4A3}">
+    <comment ref="E43" authorId="6" shapeId="0" xr:uid="{426A9046-86EB-4AF9-8A2D-1FEFC7B6C4A3}">
       <text>
         <r>
           <rPr>
@@ -128,7 +146,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E44" authorId="4" shapeId="0" xr:uid="{360FC6EE-8AD3-4EF7-B2BF-00DD1029DCAF}">
+    <comment ref="E44" authorId="6" shapeId="0" xr:uid="{360FC6EE-8AD3-4EF7-B2BF-00DD1029DCAF}">
       <text>
         <r>
           <rPr>
@@ -152,7 +170,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E64" authorId="5" shapeId="0" xr:uid="{24965C23-66A2-443D-B1F3-FDFF8EFF87E6}">
+    <comment ref="E64" authorId="7" shapeId="0" xr:uid="{24965C23-66A2-443D-B1F3-FDFF8EFF87E6}">
       <text>
         <t>[Kommentarthread]
 Ihre Version von Excel gestattet Ihnen das Lesen dieses Kommentarthreads. Jegliche Bearbeitungen daran werden jedoch entfernt, wenn die Datei in einer neueren Version von Excel geöffnet wird. Weitere Informationen: https://go.microsoft.com/fwlink/?linkid=870924.
@@ -165,7 +183,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="513" uniqueCount="305">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="565" uniqueCount="331">
   <si>
     <t>PEM Elektrolyse</t>
   </si>
@@ -937,9 +955,6 @@
     <t>annuity_ms</t>
   </si>
   <si>
-    <t>result_ms_flowsum_nh3out</t>
-  </si>
-  <si>
     <t>result_ms_flowsum_h2in</t>
   </si>
   <si>
@@ -985,9 +1000,6 @@
     <t>result_dac_flowsum_elin</t>
   </si>
   <si>
-    <t>result_dac_flowsum_n2out</t>
-  </si>
-  <si>
     <t>calc_gesamtinvest_dac</t>
   </si>
   <si>
@@ -1082,6 +1094,90 @@
   </si>
   <si>
     <t>€/kg_CH3OH</t>
+  </si>
+  <si>
+    <t>eta_hp</t>
+  </si>
+  <si>
+    <t>strombedarf_hp</t>
+  </si>
+  <si>
+    <t>capex_hp</t>
+  </si>
+  <si>
+    <t>opex_hp</t>
+  </si>
+  <si>
+    <t>lebensdauer_hp</t>
+  </si>
+  <si>
+    <t>zinssatz_hp</t>
+  </si>
+  <si>
+    <t>kWh_el/kWh_th</t>
+  </si>
+  <si>
+    <t>€/kW_th</t>
+  </si>
+  <si>
+    <t>Wärmebedarf</t>
+  </si>
+  <si>
+    <t>waerme_bedarf_dac</t>
+  </si>
+  <si>
+    <t>kWh_th/kg_CO2</t>
+  </si>
+  <si>
+    <t>annuity_hp</t>
+  </si>
+  <si>
+    <t>result_hp_leistung</t>
+  </si>
+  <si>
+    <t>result_hp_flowsum_elin</t>
+  </si>
+  <si>
+    <t>calc_gesamtinvest_hp</t>
+  </si>
+  <si>
+    <t>calc_opex_fix_hp</t>
+  </si>
+  <si>
+    <t>calc_annuity_hp</t>
+  </si>
+  <si>
+    <t>calc_verzinstinvest_hp</t>
+  </si>
+  <si>
+    <t>calc_cost_hp</t>
+  </si>
+  <si>
+    <t>€/ kW_th a</t>
+  </si>
+  <si>
+    <t>kW_th</t>
+  </si>
+  <si>
+    <t>MWh_th/a</t>
+  </si>
+  <si>
+    <t>Waermeproduktion</t>
+  </si>
+  <si>
+    <t>result_hp_flowsum_qout</t>
+  </si>
+  <si>
+    <t>MWh_el/a</t>
+  </si>
+  <si>
+    <t>result_dac_flowsum_co2out</t>
+  </si>
+  <si>
+    <t>result_dac_flowsum_qin</t>
+  </si>
+  <si>
+    <t>result_ms_flowsum_ch3ohout</t>
   </si>
 </sst>
 </file>
@@ -1094,7 +1190,7 @@
     <numFmt numFmtId="165" formatCode="0.000"/>
     <numFmt numFmtId="166" formatCode="0.00000"/>
   </numFmts>
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1188,6 +1284,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1269,7 +1372,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="103">
+  <cellXfs count="107">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -1399,13 +1502,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1414,38 +1511,50 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1900,6 +2009,12 @@
   <threadedComment ref="E13" dT="2025-03-14T08:20:33.73" personId="{7B1A26D8-2D09-4CF3-BDB9-5A9185883024}" id="{50E20A73-76EE-480B-AC2B-85B9568229B3}">
     <text xml:space="preserve">Die Methanol-Synthese benötigt 1,375 kg CO₂ pro kg Methanol (CH₃OH) unter idealen stöchiometrischen Bedingungen. Dies ergibt sich aus der Reaktionsgleichung der CO₂-Hydrierung </text>
   </threadedComment>
+  <threadedComment ref="E18" dT="2025-03-18T08:08:24.46" personId="{7B1A26D8-2D09-4CF3-BDB9-5A9185883024}" id="{A66B6FDD-7E3A-402B-8E6B-7073C79B9436}">
+    <text xml:space="preserve">0,7 * 10^6 /1000 </text>
+  </threadedComment>
+  <threadedComment ref="E23" dT="2025-03-18T08:05:52.08" personId="{7B1A26D8-2D09-4CF3-BDB9-5A9185883024}" id="{5F7F21A6-9267-43AB-9E2F-857C43A6B051}">
+    <text>1750 kWh_th/t durch 1000</text>
+  </threadedComment>
   <threadedComment ref="E24" dT="2025-03-14T09:24:29.74" personId="{7B1A26D8-2D09-4CF3-BDB9-5A9185883024}" id="{87F94307-F9C1-413A-A184-19A69689A8AF}">
     <text>800 €/t*a * 8760 h/a / 1000 kg/t = €/kg *h</text>
   </threadedComment>
@@ -2190,77 +2305,133 @@
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="72"/>
       <c r="B16" s="83" t="s">
-        <v>302</v>
-      </c>
-      <c r="C16" s="36"/>
-      <c r="D16" s="36"/>
-      <c r="E16" s="41"/>
-      <c r="F16" s="36"/>
+        <v>300</v>
+      </c>
+      <c r="C16" s="36" t="s">
+        <v>8</v>
+      </c>
+      <c r="D16" s="36" t="s">
+        <v>303</v>
+      </c>
+      <c r="E16" s="103">
+        <v>3.7</v>
+      </c>
+      <c r="F16" s="36" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="72"/>
-      <c r="B17" s="99"/>
-      <c r="C17" s="53"/>
-      <c r="D17" s="53"/>
-      <c r="E17" s="54"/>
-      <c r="F17" s="53"/>
+      <c r="B17" s="87"/>
+      <c r="C17" s="53" t="s">
+        <v>85</v>
+      </c>
+      <c r="D17" s="53" t="s">
+        <v>304</v>
+      </c>
+      <c r="E17" s="104">
+        <v>0.27</v>
+      </c>
+      <c r="F17" s="53" t="s">
+        <v>309</v>
+      </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="72"/>
-      <c r="B18" s="99"/>
-      <c r="C18" s="53"/>
-      <c r="D18" s="53"/>
-      <c r="E18" s="54"/>
-      <c r="F18" s="53"/>
+      <c r="B18" s="87"/>
+      <c r="C18" s="53" t="s">
+        <v>10</v>
+      </c>
+      <c r="D18" s="53" t="s">
+        <v>305</v>
+      </c>
+      <c r="E18" s="104">
+        <v>700</v>
+      </c>
+      <c r="F18" s="53" t="s">
+        <v>310</v>
+      </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="72"/>
-      <c r="B19" s="99"/>
-      <c r="C19" s="53"/>
-      <c r="D19" s="53"/>
-      <c r="E19" s="54"/>
-      <c r="F19" s="53"/>
+      <c r="B19" s="87"/>
+      <c r="C19" s="53" t="s">
+        <v>11</v>
+      </c>
+      <c r="D19" s="53" t="s">
+        <v>306</v>
+      </c>
+      <c r="E19" s="104">
+        <v>0.02</v>
+      </c>
+      <c r="F19" s="53" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="72"/>
-      <c r="B20" s="99"/>
-      <c r="C20" s="53"/>
-      <c r="D20" s="53"/>
-      <c r="E20" s="54"/>
-      <c r="F20" s="53"/>
+      <c r="B20" s="87"/>
+      <c r="C20" s="53" t="s">
+        <v>13</v>
+      </c>
+      <c r="D20" s="53" t="s">
+        <v>307</v>
+      </c>
+      <c r="E20" s="104">
+        <v>20</v>
+      </c>
+      <c r="F20" s="53" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="72"/>
-      <c r="B21" s="99"/>
-      <c r="C21" s="53"/>
-      <c r="D21" s="53"/>
-      <c r="E21" s="54"/>
-      <c r="F21" s="53"/>
+      <c r="B21" s="85"/>
+      <c r="C21" s="38" t="s">
+        <v>15</v>
+      </c>
+      <c r="D21" s="38" t="s">
+        <v>308</v>
+      </c>
+      <c r="E21" s="105">
+        <v>0.05</v>
+      </c>
+      <c r="F21" s="38" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="72"/>
-      <c r="B22" s="85"/>
-      <c r="C22" s="38"/>
-      <c r="D22" s="38"/>
-      <c r="E22" s="39"/>
-      <c r="F22" s="38"/>
+      <c r="B22" s="86" t="s">
+        <v>233</v>
+      </c>
+      <c r="C22" s="46" t="s">
+        <v>85</v>
+      </c>
+      <c r="D22" s="46" t="s">
+        <v>247</v>
+      </c>
+      <c r="E22" s="55">
+        <v>0.5</v>
+      </c>
+      <c r="F22" s="46" t="s">
+        <v>252</v>
+      </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="72"/>
-      <c r="B23" s="86" t="s">
-        <v>233</v>
-      </c>
+      <c r="B23" s="86"/>
       <c r="C23" s="46" t="s">
-        <v>85</v>
+        <v>311</v>
       </c>
       <c r="D23" s="46" t="s">
-        <v>247</v>
+        <v>312</v>
       </c>
       <c r="E23" s="55">
-        <v>0.5</v>
+        <v>1.75</v>
       </c>
       <c r="F23" s="46" t="s">
-        <v>252</v>
+        <v>313</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
@@ -2927,19 +3098,19 @@
     <row r="64" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A64" s="73"/>
       <c r="B64" s="1" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="C64" s="15" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="D64" s="15" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="E64" s="16">
         <v>-0.6</v>
       </c>
       <c r="F64" s="15" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
     </row>
   </sheetData>
@@ -2954,8 +3125,8 @@
     <mergeCell ref="B36:B46"/>
     <mergeCell ref="B2:B7"/>
     <mergeCell ref="B8:B15"/>
-    <mergeCell ref="B23:B27"/>
-    <mergeCell ref="B16:B22"/>
+    <mergeCell ref="B22:B27"/>
+    <mergeCell ref="B16:B21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -2965,7 +3136,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83AB2E79-6F94-41B5-A552-C40EC4890194}">
-  <dimension ref="A1:F109"/>
+  <dimension ref="A1:F120"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.5546875" style="13" customWidth="1"/>
@@ -2998,10 +3169,10 @@
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="87" t="s">
+      <c r="A2" s="92" t="s">
         <v>71</v>
       </c>
-      <c r="B2" s="89" t="s">
+      <c r="B2" s="91" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="27" t="s">
@@ -3016,7 +3187,7 @@
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="88"/>
+      <c r="A3" s="94"/>
       <c r="B3" s="84"/>
       <c r="C3" s="13" t="s">
         <v>109</v>
@@ -3030,7 +3201,7 @@
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="88"/>
+      <c r="A4" s="94"/>
       <c r="B4" s="84"/>
       <c r="C4" s="13" t="s">
         <v>85</v>
@@ -3044,7 +3215,7 @@
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="88"/>
+      <c r="A5" s="94"/>
       <c r="B5" s="84"/>
       <c r="C5" s="13" t="s">
         <v>140</v>
@@ -3058,7 +3229,7 @@
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="88"/>
+      <c r="A6" s="94"/>
       <c r="B6" s="84"/>
       <c r="C6" s="13" t="s">
         <v>143</v>
@@ -3072,7 +3243,7 @@
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="88"/>
+      <c r="A7" s="94"/>
       <c r="B7" s="84"/>
       <c r="C7" s="13" t="s">
         <v>157</v>
@@ -3086,7 +3257,7 @@
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="88"/>
+      <c r="A8" s="94"/>
       <c r="B8" s="84"/>
       <c r="C8" s="13" t="s">
         <v>200</v>
@@ -3100,7 +3271,7 @@
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="88"/>
+      <c r="A9" s="94"/>
       <c r="B9" s="84"/>
       <c r="C9" s="13" t="s">
         <v>169</v>
@@ -3114,7 +3285,7 @@
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="88"/>
+      <c r="A10" s="94"/>
       <c r="B10" s="84"/>
       <c r="C10" s="13" t="s">
         <v>192</v>
@@ -3128,13 +3299,13 @@
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" s="88"/>
+      <c r="A11" s="94"/>
       <c r="B11" s="84"/>
       <c r="E11" s="34"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="88"/>
-      <c r="B12" s="90" t="s">
+      <c r="A12" s="94"/>
+      <c r="B12" s="88" t="s">
         <v>234</v>
       </c>
       <c r="C12" s="56" t="s">
@@ -3149,27 +3320,27 @@
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="88"/>
-      <c r="B13" s="91"/>
+      <c r="A13" s="94"/>
+      <c r="B13" s="89"/>
       <c r="C13" s="46" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D13" s="46" t="s">
-        <v>256</v>
+        <v>330</v>
       </c>
       <c r="E13" s="55"/>
       <c r="F13" s="46" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" s="88"/>
-      <c r="B14" s="91"/>
+      <c r="A14" s="94"/>
+      <c r="B14" s="89"/>
       <c r="C14" s="46" t="s">
         <v>141</v>
       </c>
       <c r="D14" s="46" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="E14" s="55"/>
       <c r="F14" s="55" t="s">
@@ -3177,27 +3348,27 @@
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" s="88"/>
-      <c r="B15" s="91"/>
+      <c r="A15" s="94"/>
+      <c r="B15" s="89"/>
       <c r="C15" s="46" t="s">
+        <v>264</v>
+      </c>
+      <c r="D15" s="46" t="s">
         <v>265</v>
-      </c>
-      <c r="D15" s="46" t="s">
-        <v>266</v>
       </c>
       <c r="E15" s="58"/>
       <c r="F15" s="46" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" s="88"/>
-      <c r="B16" s="91"/>
+      <c r="A16" s="94"/>
+      <c r="B16" s="89"/>
       <c r="C16" s="46" t="s">
         <v>85</v>
       </c>
       <c r="D16" s="46" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="E16" s="55"/>
       <c r="F16" s="46" t="s">
@@ -3205,13 +3376,13 @@
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" s="88"/>
-      <c r="B17" s="91"/>
+      <c r="A17" s="94"/>
+      <c r="B17" s="89"/>
       <c r="C17" s="46" t="s">
         <v>143</v>
       </c>
       <c r="D17" s="46" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E17" s="55"/>
       <c r="F17" s="46" t="s">
@@ -3219,13 +3390,13 @@
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" s="88"/>
-      <c r="B18" s="91"/>
+      <c r="A18" s="94"/>
+      <c r="B18" s="89"/>
       <c r="C18" s="46" t="s">
         <v>157</v>
       </c>
       <c r="D18" s="46" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="E18" s="59"/>
       <c r="F18" s="46" t="s">
@@ -3233,13 +3404,13 @@
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" s="88"/>
-      <c r="B19" s="91"/>
+      <c r="A19" s="94"/>
+      <c r="B19" s="89"/>
       <c r="C19" s="46" t="s">
         <v>200</v>
       </c>
       <c r="D19" s="46" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="E19" s="59"/>
       <c r="F19" s="46" t="s">
@@ -3247,13 +3418,13 @@
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" s="88"/>
-      <c r="B20" s="91"/>
+      <c r="A20" s="94"/>
+      <c r="B20" s="89"/>
       <c r="C20" s="46" t="s">
         <v>169</v>
       </c>
       <c r="D20" s="46" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E20" s="59"/>
       <c r="F20" s="46" t="s">
@@ -3261,13 +3432,13 @@
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A21" s="88"/>
-      <c r="B21" s="91"/>
+      <c r="A21" s="94"/>
+      <c r="B21" s="89"/>
       <c r="C21" s="46" t="s">
         <v>192</v>
       </c>
       <c r="D21" s="46" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="E21" s="59"/>
       <c r="F21" s="46" t="s">
@@ -3275,79 +3446,79 @@
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A22" s="88"/>
-      <c r="B22" s="92"/>
+      <c r="A22" s="94"/>
+      <c r="B22" s="99"/>
       <c r="C22" s="60"/>
       <c r="D22" s="60"/>
       <c r="E22" s="61"/>
       <c r="F22" s="60"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" s="88"/>
-      <c r="B23" s="93" t="s">
-        <v>233</v>
+      <c r="A23" s="94"/>
+      <c r="B23" s="88" t="s">
+        <v>300</v>
       </c>
       <c r="C23" s="46" t="s">
         <v>98</v>
       </c>
       <c r="D23" s="46" t="s">
-        <v>269</v>
+        <v>314</v>
       </c>
       <c r="E23" s="55"/>
       <c r="F23" s="46" t="s">
-        <v>106</v>
+        <v>322</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" s="88"/>
-      <c r="B24" s="93"/>
+      <c r="A24" s="94"/>
+      <c r="B24" s="106"/>
       <c r="C24" s="46" t="s">
         <v>109</v>
       </c>
       <c r="D24" s="46" t="s">
-        <v>270</v>
+        <v>315</v>
       </c>
       <c r="E24" s="55"/>
       <c r="F24" s="46" t="s">
-        <v>189</v>
+        <v>323</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25" s="88"/>
-      <c r="B25" s="93"/>
+      <c r="A25" s="94"/>
+      <c r="B25" s="106"/>
       <c r="C25" s="46" t="s">
         <v>85</v>
       </c>
       <c r="D25" s="46" t="s">
-        <v>271</v>
+        <v>316</v>
       </c>
       <c r="E25" s="58"/>
       <c r="F25" s="46" t="s">
-        <v>120</v>
+        <v>327</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26" s="88"/>
-      <c r="B26" s="93"/>
+      <c r="A26" s="94"/>
+      <c r="B26" s="106"/>
       <c r="C26" s="46" t="s">
-        <v>278</v>
+        <v>325</v>
       </c>
       <c r="D26" s="46" t="s">
-        <v>272</v>
+        <v>326</v>
       </c>
       <c r="E26" s="59"/>
       <c r="F26" s="46" t="s">
-        <v>268</v>
+        <v>324</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A27" s="88"/>
-      <c r="B27" s="93"/>
+      <c r="A27" s="94"/>
+      <c r="B27" s="106"/>
       <c r="C27" s="46" t="s">
         <v>143</v>
       </c>
       <c r="D27" s="46" t="s">
-        <v>273</v>
+        <v>317</v>
       </c>
       <c r="E27" s="59"/>
       <c r="F27" s="46" t="s">
@@ -3355,13 +3526,13 @@
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A28" s="88"/>
-      <c r="B28" s="93"/>
+      <c r="A28" s="94"/>
+      <c r="B28" s="106"/>
       <c r="C28" s="46" t="s">
         <v>157</v>
       </c>
       <c r="D28" s="46" t="s">
-        <v>274</v>
+        <v>318</v>
       </c>
       <c r="E28" s="59"/>
       <c r="F28" s="46" t="s">
@@ -3369,13 +3540,13 @@
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A29" s="88"/>
-      <c r="B29" s="93"/>
+      <c r="A29" s="94"/>
+      <c r="B29" s="106"/>
       <c r="C29" s="46" t="s">
         <v>200</v>
       </c>
       <c r="D29" s="46" t="s">
-        <v>275</v>
+        <v>319</v>
       </c>
       <c r="E29" s="59"/>
       <c r="F29" s="46" t="s">
@@ -3383,13 +3554,13 @@
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A30" s="88"/>
-      <c r="B30" s="93"/>
+      <c r="A30" s="94"/>
+      <c r="B30" s="106"/>
       <c r="C30" s="46" t="s">
         <v>169</v>
       </c>
       <c r="D30" s="46" t="s">
-        <v>276</v>
+        <v>320</v>
       </c>
       <c r="E30" s="58"/>
       <c r="F30" s="46" t="s">
@@ -3397,270 +3568,273 @@
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A31" s="88"/>
-      <c r="B31" s="93"/>
+      <c r="A31" s="94"/>
+      <c r="B31" s="106"/>
       <c r="C31" s="46" t="s">
         <v>192</v>
       </c>
       <c r="D31" s="46" t="s">
-        <v>277</v>
+        <v>321</v>
       </c>
       <c r="E31" s="58"/>
       <c r="F31" s="46" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="32" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="88"/>
-      <c r="B32" s="93"/>
-      <c r="C32" s="46"/>
-      <c r="D32" s="46"/>
-      <c r="E32" s="58"/>
-      <c r="F32" s="46"/>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A32" s="94"/>
+      <c r="B32" s="99"/>
+      <c r="C32" s="60"/>
+      <c r="D32" s="60"/>
+      <c r="E32" s="61"/>
+      <c r="F32" s="60"/>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A33" s="87" t="s">
+      <c r="A33" s="94"/>
+      <c r="B33" s="100" t="s">
+        <v>233</v>
+      </c>
+      <c r="C33" s="46" t="s">
+        <v>98</v>
+      </c>
+      <c r="D33" s="46" t="s">
+        <v>268</v>
+      </c>
+      <c r="E33" s="55"/>
+      <c r="F33" s="46" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A34" s="94"/>
+      <c r="B34" s="100"/>
+      <c r="C34" s="46" t="s">
+        <v>109</v>
+      </c>
+      <c r="D34" s="46" t="s">
+        <v>269</v>
+      </c>
+      <c r="E34" s="55"/>
+      <c r="F34" s="46" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A35" s="94"/>
+      <c r="B35" s="100"/>
+      <c r="C35" s="46" t="s">
+        <v>85</v>
+      </c>
+      <c r="D35" s="46" t="s">
+        <v>270</v>
+      </c>
+      <c r="E35" s="58"/>
+      <c r="F35" s="46" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A36" s="94"/>
+      <c r="B36" s="100"/>
+      <c r="C36" s="46" t="s">
+        <v>311</v>
+      </c>
+      <c r="D36" s="46" t="s">
+        <v>329</v>
+      </c>
+      <c r="E36" s="58"/>
+      <c r="F36" s="46" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A37" s="94"/>
+      <c r="B37" s="100"/>
+      <c r="C37" s="46" t="s">
+        <v>276</v>
+      </c>
+      <c r="D37" s="46" t="s">
+        <v>328</v>
+      </c>
+      <c r="E37" s="59"/>
+      <c r="F37" s="46" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A38" s="94"/>
+      <c r="B38" s="100"/>
+      <c r="C38" s="46" t="s">
+        <v>143</v>
+      </c>
+      <c r="D38" s="46" t="s">
+        <v>271</v>
+      </c>
+      <c r="E38" s="59"/>
+      <c r="F38" s="46" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A39" s="94"/>
+      <c r="B39" s="100"/>
+      <c r="C39" s="46" t="s">
+        <v>157</v>
+      </c>
+      <c r="D39" s="46" t="s">
+        <v>272</v>
+      </c>
+      <c r="E39" s="59"/>
+      <c r="F39" s="46" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A40" s="94"/>
+      <c r="B40" s="100"/>
+      <c r="C40" s="46" t="s">
+        <v>200</v>
+      </c>
+      <c r="D40" s="46" t="s">
+        <v>273</v>
+      </c>
+      <c r="E40" s="59"/>
+      <c r="F40" s="46" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A41" s="94"/>
+      <c r="B41" s="100"/>
+      <c r="C41" s="46" t="s">
+        <v>169</v>
+      </c>
+      <c r="D41" s="46" t="s">
+        <v>274</v>
+      </c>
+      <c r="E41" s="58"/>
+      <c r="F41" s="46" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A42" s="94"/>
+      <c r="B42" s="100"/>
+      <c r="C42" s="46" t="s">
+        <v>192</v>
+      </c>
+      <c r="D42" s="46" t="s">
+        <v>275</v>
+      </c>
+      <c r="E42" s="58"/>
+      <c r="F42" s="46" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A43" s="94"/>
+      <c r="B43" s="100"/>
+      <c r="C43" s="46"/>
+      <c r="D43" s="46"/>
+      <c r="E43" s="58"/>
+      <c r="F43" s="46"/>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A44" s="92" t="s">
         <v>72</v>
       </c>
-      <c r="B33" s="95" t="s">
+      <c r="B44" s="101" t="s">
         <v>3</v>
       </c>
-      <c r="C33" s="27" t="s">
+      <c r="C44" s="27" t="s">
         <v>115</v>
       </c>
-      <c r="D33" s="27" t="s">
+      <c r="D44" s="27" t="s">
         <v>105</v>
       </c>
-      <c r="E33" s="40"/>
-      <c r="F33" s="62" t="s">
+      <c r="E44" s="40"/>
+      <c r="F44" s="62" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A34" s="88"/>
-      <c r="B34" s="86"/>
-      <c r="C34" s="13" t="s">
-        <v>113</v>
-      </c>
-      <c r="D34" s="13" t="s">
-        <v>112</v>
-      </c>
-      <c r="E34" s="34"/>
-      <c r="F34" s="63" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A35" s="88"/>
-      <c r="B35" s="86"/>
-      <c r="C35" s="13" t="s">
-        <v>137</v>
-      </c>
-      <c r="D35" s="13" t="s">
-        <v>135</v>
-      </c>
-      <c r="E35" s="35"/>
-      <c r="F35" s="13" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A36" s="88"/>
-      <c r="B36" s="86"/>
-      <c r="C36" s="13" t="s">
-        <v>138</v>
-      </c>
-      <c r="D36" s="13" t="s">
-        <v>136</v>
-      </c>
-      <c r="E36" s="34"/>
-      <c r="F36" s="13" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A37" s="88"/>
-      <c r="B37" s="86"/>
-      <c r="C37" s="13" t="s">
-        <v>143</v>
-      </c>
-      <c r="D37" s="13" t="s">
-        <v>148</v>
-      </c>
-      <c r="E37" s="34"/>
-      <c r="F37" s="13" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A38" s="88"/>
-      <c r="B38" s="86"/>
-      <c r="C38" s="13" t="s">
-        <v>157</v>
-      </c>
-      <c r="D38" s="13" t="s">
-        <v>161</v>
-      </c>
-      <c r="E38" s="34"/>
-      <c r="F38" s="13" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A39" s="88"/>
-      <c r="B39" s="86"/>
-      <c r="C39" s="13" t="s">
-        <v>200</v>
-      </c>
-      <c r="D39" s="13" t="s">
-        <v>203</v>
-      </c>
-      <c r="E39" s="34"/>
-      <c r="F39" s="13" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A40" s="88"/>
-      <c r="B40" s="86"/>
-      <c r="C40" s="13" t="s">
-        <v>169</v>
-      </c>
-      <c r="D40" s="13" t="s">
-        <v>173</v>
-      </c>
-      <c r="E40" s="34"/>
-      <c r="F40" s="13" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A41" s="88"/>
-      <c r="B41" s="86"/>
-      <c r="C41" s="13" t="s">
-        <v>192</v>
-      </c>
-      <c r="D41" s="13" t="s">
-        <v>197</v>
-      </c>
-      <c r="E41" s="34"/>
-      <c r="F41" s="13" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A42" s="88"/>
-      <c r="B42" s="86"/>
-      <c r="E42" s="34"/>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A43" s="88"/>
-      <c r="B43" s="96" t="s">
-        <v>6</v>
-      </c>
-      <c r="C43" s="36" t="s">
-        <v>98</v>
-      </c>
-      <c r="D43" s="36" t="s">
-        <v>102</v>
-      </c>
-      <c r="E43" s="41"/>
-      <c r="F43" s="36" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A44" s="88"/>
-      <c r="B44" s="86"/>
-      <c r="C44" s="13" t="s">
-        <v>115</v>
-      </c>
-      <c r="D44" s="13" t="s">
-        <v>104</v>
-      </c>
-      <c r="E44" s="34"/>
-      <c r="F44" s="13" t="s">
-        <v>107</v>
-      </c>
-    </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A45" s="88"/>
-      <c r="B45" s="84"/>
+      <c r="A45" s="94"/>
+      <c r="B45" s="86"/>
       <c r="C45" s="13" t="s">
         <v>113</v>
       </c>
       <c r="D45" s="13" t="s">
-        <v>114</v>
-      </c>
-      <c r="E45" s="32"/>
-      <c r="F45" s="13" t="s">
-        <v>116</v>
+        <v>112</v>
+      </c>
+      <c r="E45" s="34"/>
+      <c r="F45" s="63" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A46" s="88"/>
-      <c r="B46" s="84"/>
+      <c r="A46" s="94"/>
+      <c r="B46" s="86"/>
       <c r="C46" s="13" t="s">
-        <v>109</v>
+        <v>137</v>
       </c>
       <c r="D46" s="13" t="s">
-        <v>188</v>
-      </c>
-      <c r="E46" s="32"/>
+        <v>135</v>
+      </c>
+      <c r="E46" s="35"/>
       <c r="F46" s="13" t="s">
-        <v>67</v>
+        <v>134</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A47" s="88"/>
-      <c r="B47" s="84"/>
+      <c r="A47" s="94"/>
+      <c r="B47" s="86"/>
       <c r="C47" s="13" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="D47" s="13" t="s">
-        <v>126</v>
-      </c>
-      <c r="E47" s="32"/>
+        <v>136</v>
+      </c>
+      <c r="E47" s="34"/>
       <c r="F47" s="13" t="s">
-        <v>120</v>
+        <v>134</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A48" s="88"/>
-      <c r="B48" s="84"/>
+      <c r="A48" s="94"/>
+      <c r="B48" s="86"/>
       <c r="C48" s="13" t="s">
-        <v>129</v>
+        <v>143</v>
       </c>
       <c r="D48" s="13" t="s">
-        <v>127</v>
+        <v>148</v>
       </c>
       <c r="E48" s="34"/>
       <c r="F48" s="13" t="s">
-        <v>120</v>
+        <v>142</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A49" s="88"/>
-      <c r="B49" s="84"/>
+      <c r="A49" s="94"/>
+      <c r="B49" s="86"/>
       <c r="C49" s="13" t="s">
-        <v>143</v>
+        <v>157</v>
       </c>
       <c r="D49" s="13" t="s">
-        <v>147</v>
-      </c>
-      <c r="E49" s="32"/>
+        <v>161</v>
+      </c>
+      <c r="E49" s="34"/>
       <c r="F49" s="13" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A50" s="88"/>
-      <c r="B50" s="84"/>
+      <c r="A50" s="94"/>
+      <c r="B50" s="86"/>
       <c r="C50" s="13" t="s">
-        <v>157</v>
+        <v>200</v>
       </c>
       <c r="D50" s="13" t="s">
-        <v>159</v>
+        <v>203</v>
       </c>
       <c r="E50" s="34"/>
       <c r="F50" s="13" t="s">
@@ -3668,810 +3842,958 @@
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A51" s="88"/>
-      <c r="B51" s="84"/>
+      <c r="A51" s="94"/>
+      <c r="B51" s="86"/>
       <c r="C51" s="13" t="s">
-        <v>200</v>
+        <v>169</v>
       </c>
       <c r="D51" s="13" t="s">
-        <v>204</v>
+        <v>173</v>
       </c>
       <c r="E51" s="34"/>
       <c r="F51" s="13" t="s">
-        <v>151</v>
+        <v>142</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A52" s="88"/>
-      <c r="B52" s="84"/>
+      <c r="A52" s="94"/>
+      <c r="B52" s="86"/>
       <c r="C52" s="13" t="s">
-        <v>169</v>
+        <v>192</v>
       </c>
       <c r="D52" s="13" t="s">
-        <v>172</v>
+        <v>197</v>
       </c>
       <c r="E52" s="34"/>
       <c r="F52" s="13" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A53" s="88"/>
-      <c r="B53" s="84"/>
-      <c r="C53" s="13" t="s">
-        <v>192</v>
-      </c>
-      <c r="D53" s="13" t="s">
-        <v>196</v>
-      </c>
+      <c r="A53" s="94"/>
+      <c r="B53" s="86"/>
       <c r="E53" s="34"/>
-      <c r="F53" s="13" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A54" s="94"/>
-      <c r="B54" s="97"/>
-      <c r="C54" s="42"/>
-      <c r="D54" s="42"/>
-      <c r="E54" s="43"/>
-      <c r="F54" s="42"/>
+      <c r="B54" s="96" t="s">
+        <v>6</v>
+      </c>
+      <c r="C54" s="36" t="s">
+        <v>98</v>
+      </c>
+      <c r="D54" s="36" t="s">
+        <v>102</v>
+      </c>
+      <c r="E54" s="41"/>
+      <c r="F54" s="36" t="s">
+        <v>100</v>
+      </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A55" s="87" t="s">
-        <v>73</v>
-      </c>
-      <c r="B55" s="89" t="s">
-        <v>74</v>
-      </c>
-      <c r="C55" s="27" t="s">
-        <v>119</v>
-      </c>
-      <c r="D55" s="27" t="s">
-        <v>118</v>
-      </c>
-      <c r="E55" s="40"/>
-      <c r="F55" s="27" t="s">
-        <v>120</v>
+      <c r="A55" s="94"/>
+      <c r="B55" s="86"/>
+      <c r="C55" s="13" t="s">
+        <v>115</v>
+      </c>
+      <c r="D55" s="13" t="s">
+        <v>104</v>
+      </c>
+      <c r="E55" s="34"/>
+      <c r="F55" s="13" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A56" s="88"/>
+      <c r="A56" s="94"/>
       <c r="B56" s="84"/>
       <c r="C56" s="13" t="s">
-        <v>155</v>
+        <v>113</v>
       </c>
       <c r="D56" s="13" t="s">
-        <v>154</v>
+        <v>114</v>
       </c>
       <c r="E56" s="32"/>
       <c r="F56" s="13" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A57" s="94"/>
+      <c r="B57" s="84"/>
+      <c r="C57" s="13" t="s">
+        <v>109</v>
+      </c>
+      <c r="D57" s="13" t="s">
+        <v>188</v>
+      </c>
+      <c r="E57" s="32"/>
+      <c r="F57" s="13" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A58" s="94"/>
+      <c r="B58" s="84"/>
+      <c r="C58" s="13" t="s">
+        <v>128</v>
+      </c>
+      <c r="D58" s="13" t="s">
+        <v>126</v>
+      </c>
+      <c r="E58" s="32"/>
+      <c r="F58" s="13" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A59" s="94"/>
+      <c r="B59" s="84"/>
+      <c r="C59" s="13" t="s">
+        <v>129</v>
+      </c>
+      <c r="D59" s="13" t="s">
+        <v>127</v>
+      </c>
+      <c r="E59" s="34"/>
+      <c r="F59" s="13" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A60" s="94"/>
+      <c r="B60" s="84"/>
+      <c r="C60" s="13" t="s">
+        <v>143</v>
+      </c>
+      <c r="D60" s="13" t="s">
+        <v>147</v>
+      </c>
+      <c r="E60" s="32"/>
+      <c r="F60" s="13" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A61" s="94"/>
+      <c r="B61" s="84"/>
+      <c r="C61" s="13" t="s">
+        <v>157</v>
+      </c>
+      <c r="D61" s="13" t="s">
+        <v>159</v>
+      </c>
+      <c r="E61" s="34"/>
+      <c r="F61" s="13" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A57" s="88"/>
-      <c r="B57" s="85"/>
-      <c r="E57" s="32"/>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A58" s="88"/>
-      <c r="B58" s="96" t="s">
-        <v>4</v>
-      </c>
-      <c r="C58" s="36" t="s">
-        <v>98</v>
-      </c>
-      <c r="D58" s="36" t="s">
-        <v>101</v>
-      </c>
-      <c r="E58" s="41"/>
-      <c r="F58" s="36" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A59" s="88"/>
-      <c r="B59" s="86"/>
-      <c r="C59" s="13" t="s">
-        <v>109</v>
-      </c>
-      <c r="D59" s="13" t="s">
-        <v>111</v>
-      </c>
-      <c r="E59" s="44"/>
-      <c r="F59" s="13" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A60" s="88"/>
-      <c r="B60" s="86"/>
-      <c r="C60" s="13" t="s">
-        <v>124</v>
-      </c>
-      <c r="D60" s="13" t="s">
-        <v>123</v>
-      </c>
-      <c r="E60" s="44"/>
-      <c r="F60" s="13" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A61" s="88"/>
-      <c r="B61" s="86"/>
-      <c r="C61" s="13" t="s">
-        <v>143</v>
-      </c>
-      <c r="D61" s="13" t="s">
-        <v>146</v>
-      </c>
-      <c r="E61" s="32"/>
-      <c r="F61" s="13" t="s">
-        <v>142</v>
-      </c>
-    </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A62" s="88"/>
-      <c r="B62" s="86"/>
+      <c r="A62" s="94"/>
+      <c r="B62" s="84"/>
       <c r="C62" s="13" t="s">
-        <v>157</v>
+        <v>200</v>
       </c>
       <c r="D62" s="13" t="s">
-        <v>158</v>
-      </c>
-      <c r="E62" s="35"/>
+        <v>204</v>
+      </c>
+      <c r="E62" s="34"/>
       <c r="F62" s="13" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A63" s="88"/>
-      <c r="B63" s="86"/>
+      <c r="A63" s="94"/>
+      <c r="B63" s="84"/>
       <c r="C63" s="13" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="D63" s="13" t="s">
-        <v>164</v>
-      </c>
-      <c r="E63" s="32"/>
+        <v>172</v>
+      </c>
+      <c r="E63" s="34"/>
       <c r="F63" s="13" t="s">
-        <v>151</v>
+        <v>142</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A64" s="88"/>
-      <c r="B64" s="86"/>
+      <c r="A64" s="94"/>
+      <c r="B64" s="84"/>
       <c r="C64" s="13" t="s">
-        <v>200</v>
+        <v>192</v>
       </c>
       <c r="D64" s="13" t="s">
-        <v>202</v>
-      </c>
-      <c r="E64" s="32"/>
+        <v>196</v>
+      </c>
+      <c r="E64" s="34"/>
       <c r="F64" s="13" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A65" s="88"/>
-      <c r="B65" s="86"/>
-      <c r="C65" s="13" t="s">
-        <v>169</v>
-      </c>
-      <c r="D65" s="13" t="s">
-        <v>171</v>
-      </c>
-      <c r="E65" s="34"/>
-      <c r="F65" s="13" t="s">
-        <v>142</v>
-      </c>
+    <row r="65" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A65" s="95"/>
+      <c r="B65" s="102"/>
+      <c r="C65" s="42"/>
+      <c r="D65" s="42"/>
+      <c r="E65" s="43"/>
+      <c r="F65" s="42"/>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A66" s="88"/>
-      <c r="B66" s="86"/>
-      <c r="C66" s="13" t="s">
-        <v>192</v>
-      </c>
-      <c r="D66" s="13" t="s">
-        <v>194</v>
-      </c>
-      <c r="E66" s="34"/>
-      <c r="F66" s="13" t="s">
+      <c r="A66" s="92" t="s">
+        <v>73</v>
+      </c>
+      <c r="B66" s="91" t="s">
+        <v>74</v>
+      </c>
+      <c r="C66" s="27" t="s">
+        <v>119</v>
+      </c>
+      <c r="D66" s="27" t="s">
+        <v>118</v>
+      </c>
+      <c r="E66" s="40"/>
+      <c r="F66" s="27" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A67" s="94"/>
+      <c r="B67" s="84"/>
+      <c r="C67" s="13" t="s">
+        <v>155</v>
+      </c>
+      <c r="D67" s="13" t="s">
+        <v>154</v>
+      </c>
+      <c r="E67" s="32"/>
+      <c r="F67" s="13" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A67" s="88"/>
-      <c r="B67" s="101"/>
-    </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A68" s="88"/>
-      <c r="B68" s="96" t="s">
-        <v>5</v>
-      </c>
-      <c r="C68" s="36" t="s">
+      <c r="A68" s="94"/>
+      <c r="B68" s="85"/>
+      <c r="E68" s="32"/>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A69" s="94"/>
+      <c r="B69" s="96" t="s">
+        <v>4</v>
+      </c>
+      <c r="C69" s="36" t="s">
         <v>98</v>
       </c>
-      <c r="D68" s="36" t="s">
-        <v>103</v>
-      </c>
-      <c r="E68" s="41"/>
-      <c r="F68" s="36" t="s">
+      <c r="D69" s="36" t="s">
+        <v>101</v>
+      </c>
+      <c r="E69" s="41"/>
+      <c r="F69" s="36" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A69" s="88"/>
-      <c r="B69" s="86"/>
-      <c r="C69" s="13" t="s">
-        <v>110</v>
-      </c>
-      <c r="D69" s="13" t="s">
-        <v>108</v>
-      </c>
-      <c r="E69" s="44"/>
-      <c r="F69" s="13" t="s">
-        <v>67</v>
-      </c>
-    </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A70" s="88"/>
+      <c r="A70" s="94"/>
       <c r="B70" s="86"/>
       <c r="C70" s="13" t="s">
-        <v>122</v>
+        <v>109</v>
       </c>
       <c r="D70" s="13" t="s">
-        <v>121</v>
+        <v>111</v>
       </c>
       <c r="E70" s="44"/>
       <c r="F70" s="13" t="s">
-        <v>120</v>
+        <v>67</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A71" s="88"/>
+      <c r="A71" s="94"/>
       <c r="B71" s="86"/>
       <c r="C71" s="13" t="s">
-        <v>143</v>
+        <v>124</v>
       </c>
       <c r="D71" s="13" t="s">
-        <v>144</v>
+        <v>123</v>
       </c>
       <c r="E71" s="44"/>
       <c r="F71" s="13" t="s">
-        <v>142</v>
+        <v>120</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A72" s="88"/>
+      <c r="A72" s="94"/>
       <c r="B72" s="86"/>
       <c r="C72" s="13" t="s">
-        <v>157</v>
+        <v>143</v>
       </c>
       <c r="D72" s="13" t="s">
-        <v>156</v>
-      </c>
-      <c r="E72" s="35"/>
+        <v>146</v>
+      </c>
+      <c r="E72" s="32"/>
       <c r="F72" s="13" t="s">
-        <v>151</v>
+        <v>142</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A73" s="88"/>
+      <c r="A73" s="94"/>
       <c r="B73" s="86"/>
       <c r="C73" s="13" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="D73" s="13" t="s">
-        <v>162</v>
-      </c>
-      <c r="E73" s="45"/>
+        <v>158</v>
+      </c>
+      <c r="E73" s="35"/>
       <c r="F73" s="13" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A74" s="88"/>
+      <c r="A74" s="94"/>
       <c r="B74" s="86"/>
       <c r="C74" s="13" t="s">
-        <v>200</v>
+        <v>163</v>
       </c>
       <c r="D74" s="13" t="s">
-        <v>201</v>
-      </c>
-      <c r="E74" s="45"/>
+        <v>164</v>
+      </c>
+      <c r="E74" s="32"/>
       <c r="F74" s="13" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A75" s="88"/>
+      <c r="A75" s="94"/>
       <c r="B75" s="86"/>
       <c r="C75" s="13" t="s">
-        <v>169</v>
+        <v>200</v>
       </c>
       <c r="D75" s="13" t="s">
-        <v>170</v>
-      </c>
-      <c r="E75" s="34"/>
+        <v>202</v>
+      </c>
+      <c r="E75" s="32"/>
       <c r="F75" s="13" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A76" s="88"/>
+      <c r="A76" s="94"/>
       <c r="B76" s="86"/>
       <c r="C76" s="13" t="s">
-        <v>192</v>
+        <v>169</v>
       </c>
       <c r="D76" s="13" t="s">
-        <v>193</v>
+        <v>171</v>
       </c>
       <c r="E76" s="34"/>
       <c r="F76" s="13" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A77" s="94"/>
+      <c r="B77" s="86"/>
+      <c r="C77" s="13" t="s">
+        <v>192</v>
+      </c>
+      <c r="D77" s="13" t="s">
+        <v>194</v>
+      </c>
+      <c r="E77" s="34"/>
+      <c r="F77" s="13" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="77" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A77" s="94"/>
-      <c r="B77" s="102"/>
-    </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A78" s="87" t="s">
-        <v>77</v>
-      </c>
-      <c r="B78" s="89" t="s">
-        <v>74</v>
-      </c>
-      <c r="C78" s="27" t="s">
-        <v>131</v>
-      </c>
-      <c r="D78" s="27" t="s">
-        <v>130</v>
-      </c>
-      <c r="E78" s="31"/>
-      <c r="F78" s="27" t="s">
+      <c r="A78" s="94"/>
+      <c r="B78" s="97"/>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A79" s="94"/>
+      <c r="B79" s="96" t="s">
+        <v>5</v>
+      </c>
+      <c r="C79" s="36" t="s">
+        <v>98</v>
+      </c>
+      <c r="D79" s="36" t="s">
+        <v>103</v>
+      </c>
+      <c r="E79" s="41"/>
+      <c r="F79" s="36" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A80" s="94"/>
+      <c r="B80" s="86"/>
+      <c r="C80" s="13" t="s">
+        <v>110</v>
+      </c>
+      <c r="D80" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="E80" s="44"/>
+      <c r="F80" s="13" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A81" s="94"/>
+      <c r="B81" s="86"/>
+      <c r="C81" s="13" t="s">
+        <v>122</v>
+      </c>
+      <c r="D81" s="13" t="s">
+        <v>121</v>
+      </c>
+      <c r="E81" s="44"/>
+      <c r="F81" s="13" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A79" s="100"/>
-      <c r="B79" s="99"/>
-      <c r="C79" s="53" t="s">
-        <v>232</v>
-      </c>
-      <c r="D79" s="53" t="s">
-        <v>231</v>
-      </c>
-      <c r="E79" s="54"/>
-      <c r="F79" s="53" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A80" s="88"/>
-      <c r="B80" s="84"/>
-      <c r="C80" s="13" t="s">
-        <v>152</v>
-      </c>
-      <c r="D80" s="13" t="s">
-        <v>149</v>
-      </c>
-      <c r="E80" s="34"/>
-      <c r="F80" s="13" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A81" s="88"/>
-      <c r="B81" s="85"/>
-      <c r="E81" s="34"/>
-    </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A82" s="88"/>
-      <c r="B82" s="83" t="s">
-        <v>80</v>
-      </c>
-      <c r="C82" s="36" t="s">
-        <v>133</v>
-      </c>
-      <c r="D82" s="36" t="s">
-        <v>132</v>
-      </c>
-      <c r="E82" s="41"/>
-      <c r="F82" s="36" t="s">
-        <v>134</v>
+      <c r="A82" s="94"/>
+      <c r="B82" s="86"/>
+      <c r="C82" s="13" t="s">
+        <v>143</v>
+      </c>
+      <c r="D82" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E82" s="44"/>
+      <c r="F82" s="13" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A83" s="88"/>
-      <c r="B83" s="84"/>
+      <c r="A83" s="94"/>
+      <c r="B83" s="86"/>
       <c r="C83" s="13" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D83" s="13" t="s">
-        <v>150</v>
-      </c>
-      <c r="E83" s="34"/>
+        <v>156</v>
+      </c>
+      <c r="E83" s="35"/>
       <c r="F83" s="13" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A84" s="88"/>
-      <c r="B84" s="85"/>
-      <c r="C84" s="38"/>
-      <c r="D84" s="38"/>
-      <c r="E84" s="39"/>
-      <c r="F84" s="38"/>
+      <c r="A84" s="94"/>
+      <c r="B84" s="86"/>
+      <c r="C84" s="13" t="s">
+        <v>163</v>
+      </c>
+      <c r="D84" s="13" t="s">
+        <v>162</v>
+      </c>
+      <c r="E84" s="45"/>
+      <c r="F84" s="13" t="s">
+        <v>151</v>
+      </c>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A85" s="88"/>
-      <c r="B85" s="90" t="s">
-        <v>280</v>
-      </c>
-      <c r="C85" s="46" t="s">
-        <v>279</v>
-      </c>
-      <c r="D85" s="46" t="s">
-        <v>282</v>
-      </c>
-      <c r="E85" s="58"/>
-      <c r="F85" s="46" t="s">
-        <v>267</v>
+      <c r="A85" s="94"/>
+      <c r="B85" s="86"/>
+      <c r="C85" s="13" t="s">
+        <v>200</v>
+      </c>
+      <c r="D85" s="13" t="s">
+        <v>201</v>
+      </c>
+      <c r="E85" s="45"/>
+      <c r="F85" s="13" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A86" s="88"/>
-      <c r="B86" s="91"/>
-      <c r="C86" s="46" t="s">
-        <v>281</v>
-      </c>
-      <c r="D86" s="46" t="s">
-        <v>283</v>
-      </c>
-      <c r="E86" s="58"/>
-      <c r="F86" s="46" t="s">
+      <c r="A86" s="94"/>
+      <c r="B86" s="86"/>
+      <c r="C86" s="13" t="s">
+        <v>169</v>
+      </c>
+      <c r="D86" s="13" t="s">
+        <v>170</v>
+      </c>
+      <c r="E86" s="34"/>
+      <c r="F86" s="13" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A87" s="94"/>
+      <c r="B87" s="86"/>
+      <c r="C87" s="13" t="s">
+        <v>192</v>
+      </c>
+      <c r="D87" s="13" t="s">
+        <v>193</v>
+      </c>
+      <c r="E87" s="34"/>
+      <c r="F87" s="13" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="87" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A87" s="94"/>
-      <c r="B87" s="98"/>
-      <c r="C87" s="64"/>
-      <c r="D87" s="64"/>
-      <c r="E87" s="65"/>
-      <c r="F87" s="64"/>
-    </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A88" s="87" t="s">
-        <v>165</v>
-      </c>
-      <c r="B88" s="89" t="s">
-        <v>13</v>
-      </c>
-      <c r="C88" s="27" t="s">
-        <v>175</v>
-      </c>
-      <c r="D88" s="27" t="s">
-        <v>174</v>
-      </c>
-      <c r="E88" s="27"/>
-      <c r="F88" s="27" t="s">
-        <v>142</v>
-      </c>
+    <row r="88" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A88" s="95"/>
+      <c r="B88" s="98"/>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A89" s="100"/>
-      <c r="B89" s="84"/>
-      <c r="C89" s="13" t="s">
-        <v>176</v>
-      </c>
-      <c r="D89" s="13" t="s">
-        <v>177</v>
-      </c>
-      <c r="F89" s="13" t="s">
-        <v>142</v>
+      <c r="A89" s="92" t="s">
+        <v>77</v>
+      </c>
+      <c r="B89" s="91" t="s">
+        <v>74</v>
+      </c>
+      <c r="C89" s="27" t="s">
+        <v>131</v>
+      </c>
+      <c r="D89" s="27" t="s">
+        <v>130</v>
+      </c>
+      <c r="E89" s="31"/>
+      <c r="F89" s="27" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A90" s="100"/>
-      <c r="B90" s="85"/>
-      <c r="C90" s="38"/>
-      <c r="D90" s="38"/>
-      <c r="E90" s="38"/>
-      <c r="F90" s="38"/>
+      <c r="A90" s="93"/>
+      <c r="B90" s="87"/>
+      <c r="C90" s="53" t="s">
+        <v>232</v>
+      </c>
+      <c r="D90" s="53" t="s">
+        <v>231</v>
+      </c>
+      <c r="E90" s="54"/>
+      <c r="F90" s="53" t="s">
+        <v>151</v>
+      </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A91" s="100"/>
-      <c r="B91" s="83" t="s">
-        <v>186</v>
-      </c>
+      <c r="A91" s="94"/>
+      <c r="B91" s="84"/>
       <c r="C91" s="13" t="s">
-        <v>167</v>
+        <v>152</v>
       </c>
       <c r="D91" s="13" t="s">
-        <v>166</v>
-      </c>
+        <v>149</v>
+      </c>
+      <c r="E91" s="34"/>
       <c r="F91" s="13" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A92" s="100"/>
-      <c r="B92" s="84"/>
-      <c r="C92" s="13" t="s">
-        <v>184</v>
-      </c>
-      <c r="D92" s="13" t="s">
-        <v>178</v>
-      </c>
-      <c r="F92" s="13" t="s">
-        <v>151</v>
-      </c>
+      <c r="A92" s="94"/>
+      <c r="B92" s="85"/>
+      <c r="E92" s="34"/>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A93" s="100"/>
-      <c r="B93" s="84"/>
-      <c r="C93" s="13" t="s">
-        <v>180</v>
-      </c>
-      <c r="D93" s="13" t="s">
-        <v>179</v>
-      </c>
-      <c r="F93" s="13" t="s">
-        <v>151</v>
+      <c r="A93" s="94"/>
+      <c r="B93" s="83" t="s">
+        <v>80</v>
+      </c>
+      <c r="C93" s="36" t="s">
+        <v>133</v>
+      </c>
+      <c r="D93" s="36" t="s">
+        <v>132</v>
+      </c>
+      <c r="E93" s="41"/>
+      <c r="F93" s="36" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A94" s="100"/>
+      <c r="A94" s="94"/>
       <c r="B94" s="84"/>
       <c r="C94" s="13" t="s">
-        <v>182</v>
+        <v>153</v>
       </c>
       <c r="D94" s="13" t="s">
-        <v>181</v>
-      </c>
+        <v>150</v>
+      </c>
+      <c r="E94" s="34"/>
       <c r="F94" s="13" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A95" s="100"/>
-      <c r="B95" s="84"/>
-      <c r="C95" s="13" t="s">
+      <c r="A95" s="94"/>
+      <c r="B95" s="85"/>
+      <c r="C95" s="38"/>
+      <c r="D95" s="38"/>
+      <c r="E95" s="39"/>
+      <c r="F95" s="38"/>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A96" s="94"/>
+      <c r="B96" s="88" t="s">
+        <v>278</v>
+      </c>
+      <c r="C96" s="46" t="s">
+        <v>277</v>
+      </c>
+      <c r="D96" s="46" t="s">
+        <v>280</v>
+      </c>
+      <c r="E96" s="58"/>
+      <c r="F96" s="46" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A97" s="94"/>
+      <c r="B97" s="89"/>
+      <c r="C97" s="46" t="s">
+        <v>279</v>
+      </c>
+      <c r="D97" s="46" t="s">
+        <v>281</v>
+      </c>
+      <c r="E97" s="58"/>
+      <c r="F97" s="46" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A98" s="95"/>
+      <c r="B98" s="90"/>
+      <c r="C98" s="64"/>
+      <c r="D98" s="64"/>
+      <c r="E98" s="65"/>
+      <c r="F98" s="64"/>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A99" s="92" t="s">
+        <v>165</v>
+      </c>
+      <c r="B99" s="91" t="s">
+        <v>13</v>
+      </c>
+      <c r="C99" s="27" t="s">
+        <v>175</v>
+      </c>
+      <c r="D99" s="27" t="s">
+        <v>174</v>
+      </c>
+      <c r="E99" s="27"/>
+      <c r="F99" s="27" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A100" s="93"/>
+      <c r="B100" s="84"/>
+      <c r="C100" s="13" t="s">
+        <v>176</v>
+      </c>
+      <c r="D100" s="13" t="s">
+        <v>177</v>
+      </c>
+      <c r="F100" s="13" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A101" s="93"/>
+      <c r="B101" s="85"/>
+      <c r="C101" s="38"/>
+      <c r="D101" s="38"/>
+      <c r="E101" s="38"/>
+      <c r="F101" s="38"/>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A102" s="93"/>
+      <c r="B102" s="83" t="s">
+        <v>186</v>
+      </c>
+      <c r="C102" s="13" t="s">
+        <v>167</v>
+      </c>
+      <c r="D102" s="13" t="s">
+        <v>166</v>
+      </c>
+      <c r="F102" s="13" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A103" s="93"/>
+      <c r="B103" s="84"/>
+      <c r="C103" s="13" t="s">
+        <v>184</v>
+      </c>
+      <c r="D103" s="13" t="s">
+        <v>178</v>
+      </c>
+      <c r="F103" s="13" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A104" s="93"/>
+      <c r="B104" s="84"/>
+      <c r="C104" s="13" t="s">
+        <v>180</v>
+      </c>
+      <c r="D104" s="13" t="s">
+        <v>179</v>
+      </c>
+      <c r="F104" s="13" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A105" s="93"/>
+      <c r="B105" s="84"/>
+      <c r="C105" s="13" t="s">
+        <v>182</v>
+      </c>
+      <c r="D105" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="F105" s="13" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A106" s="93"/>
+      <c r="B106" s="84"/>
+      <c r="C106" s="13" t="s">
         <v>185</v>
       </c>
-      <c r="D95" s="13" t="s">
+      <c r="D106" s="13" t="s">
         <v>183</v>
       </c>
-      <c r="F95" s="13" t="s">
+      <c r="F106" s="13" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A96" s="100"/>
-      <c r="B96" s="84"/>
-      <c r="C96" s="13" t="s">
+    <row r="107" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A107" s="93"/>
+      <c r="B107" s="84"/>
+      <c r="C107" s="13" t="s">
         <v>195</v>
       </c>
-      <c r="D96" s="13" t="s">
+      <c r="D107" s="13" t="s">
         <v>191</v>
       </c>
-      <c r="F96" s="13" t="s">
+      <c r="F107" s="13" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A97" s="100"/>
-      <c r="B97" s="83" t="s">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A108" s="93"/>
+      <c r="B108" s="83" t="s">
         <v>210</v>
       </c>
-      <c r="C97" s="36" t="s">
+      <c r="C108" s="36" t="s">
         <v>207</v>
       </c>
-      <c r="D97" s="36" t="s">
+      <c r="D108" s="36" t="s">
         <v>211</v>
       </c>
-      <c r="E97" s="36"/>
-      <c r="F97" s="36" t="s">
+      <c r="E108" s="36"/>
+      <c r="F108" s="36" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A98" s="100"/>
-      <c r="B98" s="99"/>
-      <c r="C98" s="53" t="s">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A109" s="93"/>
+      <c r="B109" s="87"/>
+      <c r="C109" s="53" t="s">
         <v>208</v>
       </c>
-      <c r="D98" s="53" t="s">
+      <c r="D109" s="53" t="s">
         <v>214</v>
       </c>
-      <c r="E98" s="53"/>
-      <c r="F98" s="53" t="s">
+      <c r="E109" s="53"/>
+      <c r="F109" s="53" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A99" s="100"/>
-      <c r="B99" s="99"/>
-      <c r="C99" s="53" t="s">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A110" s="93"/>
+      <c r="B110" s="87"/>
+      <c r="C110" s="53" t="s">
         <v>219</v>
       </c>
-      <c r="D99" s="53" t="s">
+      <c r="D110" s="53" t="s">
         <v>218</v>
       </c>
-      <c r="E99" s="53"/>
-      <c r="F99" s="53" t="s">
+      <c r="E110" s="53"/>
+      <c r="F110" s="53" t="s">
         <v>223</v>
       </c>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A100" s="100"/>
-      <c r="B100" s="99"/>
-      <c r="C100" s="53" t="s">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A111" s="93"/>
+      <c r="B111" s="87"/>
+      <c r="C111" s="53" t="s">
         <v>209</v>
       </c>
-      <c r="D100" s="53" t="s">
+      <c r="D111" s="53" t="s">
         <v>213</v>
       </c>
-      <c r="E100" s="53"/>
-      <c r="F100" s="53" t="s">
+      <c r="E111" s="53"/>
+      <c r="F111" s="53" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A101" s="100"/>
-      <c r="B101" s="99"/>
-      <c r="C101" s="53" t="s">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A112" s="93"/>
+      <c r="B112" s="87"/>
+      <c r="C112" s="53" t="s">
         <v>221</v>
       </c>
-      <c r="D101" s="53" t="s">
+      <c r="D112" s="53" t="s">
         <v>220</v>
       </c>
-      <c r="E101" s="53"/>
-      <c r="F101" s="53" t="s">
+      <c r="E112" s="53"/>
+      <c r="F112" s="53" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A102" s="100"/>
-      <c r="B102" s="99"/>
-      <c r="C102" s="53" t="s">
+    <row r="113" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A113" s="93"/>
+      <c r="B113" s="87"/>
+      <c r="C113" s="53" t="s">
         <v>225</v>
       </c>
-      <c r="D102" s="53" t="s">
+      <c r="D113" s="53" t="s">
         <v>215</v>
       </c>
-      <c r="E102" s="53"/>
-      <c r="F102" s="53" t="s">
+      <c r="E113" s="53"/>
+      <c r="F113" s="53" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A103" s="100"/>
-      <c r="B103" s="99"/>
-      <c r="C103" s="53" t="s">
+    <row r="114" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A114" s="93"/>
+      <c r="B114" s="87"/>
+      <c r="C114" s="53" t="s">
         <v>206</v>
       </c>
-      <c r="D103" s="13" t="s">
+      <c r="D114" s="13" t="s">
         <v>224</v>
       </c>
-      <c r="E103" s="53"/>
-      <c r="F103" s="53" t="s">
+      <c r="E114" s="53"/>
+      <c r="F114" s="53" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A104" s="100"/>
-      <c r="B104" s="99"/>
-      <c r="C104" s="66" t="s">
+    <row r="115" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A115" s="93"/>
+      <c r="B115" s="87"/>
+      <c r="C115" s="66" t="s">
+        <v>282</v>
+      </c>
+      <c r="D115" s="66" t="s">
+        <v>283</v>
+      </c>
+      <c r="E115" s="66"/>
+      <c r="F115" s="46" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A116" s="93"/>
+      <c r="B116" s="87"/>
+      <c r="C116" s="66" t="s">
+        <v>285</v>
+      </c>
+      <c r="D116" s="66" t="s">
         <v>284</v>
       </c>
-      <c r="D104" s="66" t="s">
-        <v>285</v>
-      </c>
-      <c r="E104" s="66"/>
-      <c r="F104" s="46" t="s">
+      <c r="E116" s="66"/>
+      <c r="F116" s="66" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A117" s="93"/>
+      <c r="B117" s="83" t="s">
+        <v>226</v>
+      </c>
+      <c r="C117" s="36" t="s">
+        <v>228</v>
+      </c>
+      <c r="D117" s="36" t="s">
+        <v>227</v>
+      </c>
+      <c r="E117" s="36"/>
+      <c r="F117" s="36" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A118" s="93"/>
+      <c r="B118" s="87"/>
+      <c r="C118" s="53" t="s">
+        <v>229</v>
+      </c>
+      <c r="D118" s="53" t="s">
+        <v>230</v>
+      </c>
+      <c r="E118" s="53"/>
+      <c r="F118" s="53" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A105" s="100"/>
-      <c r="B105" s="99"/>
-      <c r="C105" s="66" t="s">
+    <row r="119" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A119" s="93"/>
+      <c r="B119" s="87"/>
+      <c r="C119" s="66" t="s">
+        <v>286</v>
+      </c>
+      <c r="D119" s="66" t="s">
         <v>287</v>
       </c>
-      <c r="D105" s="66" t="s">
-        <v>286</v>
-      </c>
-      <c r="E105" s="66"/>
-      <c r="F105" s="66" t="s">
+      <c r="E119" s="66"/>
+      <c r="F119" s="66" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A120" s="93"/>
+      <c r="B120" s="87"/>
+      <c r="C120" s="46" t="s">
+        <v>288</v>
+      </c>
+      <c r="D120" s="46" t="s">
+        <v>289</v>
+      </c>
+      <c r="E120" s="46"/>
+      <c r="F120" s="46" t="s">
         <v>217</v>
       </c>
     </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A106" s="100"/>
-      <c r="B106" s="83" t="s">
-        <v>226</v>
-      </c>
-      <c r="C106" s="36" t="s">
-        <v>228</v>
-      </c>
-      <c r="D106" s="36" t="s">
-        <v>227</v>
-      </c>
-      <c r="E106" s="36"/>
-      <c r="F106" s="36" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A107" s="100"/>
-      <c r="B107" s="99"/>
-      <c r="C107" s="53" t="s">
-        <v>229</v>
-      </c>
-      <c r="D107" s="53" t="s">
-        <v>230</v>
-      </c>
-      <c r="E107" s="53"/>
-      <c r="F107" s="53" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A108" s="100"/>
-      <c r="B108" s="99"/>
-      <c r="C108" s="66" t="s">
-        <v>288</v>
-      </c>
-      <c r="D108" s="66" t="s">
-        <v>289</v>
-      </c>
-      <c r="E108" s="66"/>
-      <c r="F108" s="66" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A109" s="100"/>
-      <c r="B109" s="99"/>
-      <c r="C109" s="46" t="s">
-        <v>290</v>
-      </c>
-      <c r="D109" s="46" t="s">
-        <v>291</v>
-      </c>
-      <c r="E109" s="46"/>
-      <c r="F109" s="46" t="s">
-        <v>217</v>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="20">
-    <mergeCell ref="B85:B87"/>
-    <mergeCell ref="B55:B57"/>
-    <mergeCell ref="B91:B96"/>
-    <mergeCell ref="B106:B109"/>
-    <mergeCell ref="A88:A109"/>
-    <mergeCell ref="B97:B105"/>
-    <mergeCell ref="B88:B90"/>
-    <mergeCell ref="A55:A77"/>
-    <mergeCell ref="B58:B67"/>
-    <mergeCell ref="B68:B77"/>
-    <mergeCell ref="A78:A87"/>
-    <mergeCell ref="B78:B81"/>
-    <mergeCell ref="B82:B84"/>
-    <mergeCell ref="A2:A32"/>
+  <mergeCells count="21">
+    <mergeCell ref="A2:A43"/>
     <mergeCell ref="B2:B11"/>
     <mergeCell ref="B12:B22"/>
+    <mergeCell ref="B33:B43"/>
+    <mergeCell ref="A44:A65"/>
+    <mergeCell ref="B44:B53"/>
+    <mergeCell ref="B54:B65"/>
     <mergeCell ref="B23:B32"/>
-    <mergeCell ref="A33:A54"/>
-    <mergeCell ref="B33:B42"/>
-    <mergeCell ref="B43:B54"/>
+    <mergeCell ref="B96:B98"/>
+    <mergeCell ref="B66:B68"/>
+    <mergeCell ref="B102:B107"/>
+    <mergeCell ref="B117:B120"/>
+    <mergeCell ref="A99:A120"/>
+    <mergeCell ref="B108:B116"/>
+    <mergeCell ref="B99:B101"/>
+    <mergeCell ref="A66:A88"/>
+    <mergeCell ref="B69:B78"/>
+    <mergeCell ref="B79:B88"/>
+    <mergeCell ref="A89:A98"/>
+    <mergeCell ref="B89:B92"/>
+    <mergeCell ref="B93:B95"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -4488,47 +4810,47 @@
   <sheetData>
     <row r="1" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B1" s="67" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="2" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B2" s="67" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
     </row>
     <row r="22" spans="2:2" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B22" s="70" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
     </row>
     <row r="24" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B24" s="67" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
     </row>
     <row r="26" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B26" s="67" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
     </row>
     <row r="27" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B27" s="67" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
     </row>
     <row r="28" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B28" s="67" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
     </row>
     <row r="29" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B29" s="68" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
     </row>
     <row r="30" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B30" s="69" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
     </row>
     <row r="31" spans="2:2" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Initial Push Methanol Greenfield Patagonien Push
Modellvorschlag Methanol Greenfield Patagonien:
ASU durch DAC ersetzt
HB durch MS ersetzt
HP und Q hinzugefügt
Datenbank angepasst und Literaturvorschlag eingefügt
</commit_message>
<xml_diff>
--- a/Methanol_DAC_Greenfield_Patagonien/Datenbank.xlsx
+++ b/Methanol_DAC_Greenfield_Patagonien/Datenbank.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\01-Arbeit\06-FENES\09-P2X3\FENES_P2X\Methanol_DAC_Greenfield_Patagonien\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15E961C6-683D-4E50-A982-1085A77723A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{908D3A3D-CD06-467F-9C9A-476F00F703A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -170,7 +170,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E64" authorId="7" shapeId="0" xr:uid="{24965C23-66A2-443D-B1F3-FDFF8EFF87E6}">
+    <comment ref="E65" authorId="7" shapeId="0" xr:uid="{24965C23-66A2-443D-B1F3-FDFF8EFF87E6}">
       <text>
         <t>[Kommentarthread]
 Ihre Version von Excel gestattet Ihnen das Lesen dieses Kommentarthreads. Jegliche Bearbeitungen daran werden jedoch entfernt, wenn die Datei in einer neueren Version von Excel geöffnet wird. Weitere Informationen: https://go.microsoft.com/fwlink/?linkid=870924.
@@ -183,7 +183,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="565" uniqueCount="331">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="586" uniqueCount="346">
   <si>
     <t>PEM Elektrolyse</t>
   </si>
@@ -1054,9 +1054,6 @@
     <t>Gesamtkosten pro t Methanol</t>
   </si>
   <si>
-    <t>calc_cost_co3oh</t>
-  </si>
-  <si>
     <t>https://epub.wupperinst.org/frontdoor/deliver/index/docId/7944/file/WSA25_Block.pdf</t>
   </si>
   <si>
@@ -1114,9 +1111,6 @@
     <t>zinssatz_hp</t>
   </si>
   <si>
-    <t>kWh_el/kWh_th</t>
-  </si>
-  <si>
     <t>€/kW_th</t>
   </si>
   <si>
@@ -1156,9 +1150,6 @@
     <t>€/ kW_th a</t>
   </si>
   <si>
-    <t>kW_th</t>
-  </si>
-  <si>
     <t>MWh_th/a</t>
   </si>
   <si>
@@ -1178,6 +1169,60 @@
   </si>
   <si>
     <t>result_ms_flowsum_ch3ohout</t>
+  </si>
+  <si>
+    <t>Wärme Verkauf</t>
+  </si>
+  <si>
+    <t>Waerme Verkaufspreis</t>
+  </si>
+  <si>
+    <t>waermeerloes</t>
+  </si>
+  <si>
+    <t>kW_el/kW_th</t>
+  </si>
+  <si>
+    <t>Waerme Verkauf</t>
+  </si>
+  <si>
+    <t>Waermeverkauf</t>
+  </si>
+  <si>
+    <t>result_qverkauf_flowsum</t>
+  </si>
+  <si>
+    <t>calc_einnahmen_qverkauf_schattenvariable</t>
+  </si>
+  <si>
+    <t>calc_einnnahmen_qverkauf</t>
+  </si>
+  <si>
+    <t>Schattenvariable Einnahmen Wärmeverkauf</t>
+  </si>
+  <si>
+    <t>Einnahmen aus Wärmeverkauf</t>
+  </si>
+  <si>
+    <t>calc_cost_ch3oh</t>
+  </si>
+  <si>
+    <t>calc_annuity_gesamt</t>
+  </si>
+  <si>
+    <t>Levelized Cost of Heatpump</t>
+  </si>
+  <si>
+    <t>calc_lcoh_hp</t>
+  </si>
+  <si>
+    <t>Gesamtkosten pro kWh thermisch</t>
+  </si>
+  <si>
+    <t>calc_cost_q</t>
+  </si>
+  <si>
+    <t>ct/kWh_th</t>
   </si>
 </sst>
 </file>
@@ -1300,7 +1345,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -1366,13 +1411,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="107">
+  <cellXfs count="113">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -1392,7 +1448,6 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -1454,6 +1509,15 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1461,6 +1525,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1505,38 +1572,20 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -1544,17 +1593,32 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -2021,7 +2085,7 @@
   <threadedComment ref="E25" dT="2025-03-14T09:25:24.78" personId="{7B1A26D8-2D09-4CF3-BDB9-5A9185883024}" id="{011C4874-472E-423F-9F9E-1A44747EBF50}">
     <text>~ 40 opex/ 800 capex</text>
   </threadedComment>
-  <threadedComment ref="E64" dT="2025-03-18T07:43:27.70" personId="{7B1A26D8-2D09-4CF3-BDB9-5A9185883024}" id="{24965C23-66A2-443D-B1F3-FDFF8EFF87E6}">
+  <threadedComment ref="E65" dT="2025-03-18T07:43:27.70" personId="{7B1A26D8-2D09-4CF3-BDB9-5A9185883024}" id="{24965C23-66A2-443D-B1F3-FDFF8EFF87E6}">
     <text>https://de.statista.com/statistik/daten/studie/730823/umfrage/durchschnittlicher-preis-fuer-methanol-auf-dem-europaeischen-markt/</text>
     <extLst>
       <x:ext xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" uri="{F7C98A9C-CBB3-438F-8F68-D28B6AF4A901}">
@@ -2035,7 +2099,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G64"/>
+  <dimension ref="A1:G65"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.88671875" customWidth="1"/>
@@ -2073,10 +2137,10 @@
       <c r="G1" s="6"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="71" t="s">
+      <c r="A2" s="79" t="s">
         <v>71</v>
       </c>
-      <c r="B2" s="81" t="s">
+      <c r="B2" s="90" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="2" t="s">
@@ -2093,8 +2157,8 @@
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="72"/>
-      <c r="B3" s="82"/>
+      <c r="A3" s="80"/>
+      <c r="B3" s="91"/>
       <c r="C3" t="s">
         <v>85</v>
       </c>
@@ -2109,15 +2173,15 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="72"/>
-      <c r="B4" s="82"/>
+      <c r="A4" s="80"/>
+      <c r="B4" s="91"/>
       <c r="C4" t="s">
         <v>10</v>
       </c>
       <c r="D4" t="s">
         <v>26</v>
       </c>
-      <c r="E4" s="21">
+      <c r="E4" s="20">
         <v>1000</v>
       </c>
       <c r="F4" t="s">
@@ -2125,8 +2189,8 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="72"/>
-      <c r="B5" s="82"/>
+      <c r="A5" s="80"/>
+      <c r="B5" s="91"/>
       <c r="C5" t="s">
         <v>11</v>
       </c>
@@ -2141,15 +2205,15 @@
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="72"/>
-      <c r="B6" s="82"/>
+      <c r="A6" s="80"/>
+      <c r="B6" s="91"/>
       <c r="C6" t="s">
         <v>13</v>
       </c>
       <c r="D6" t="s">
         <v>28</v>
       </c>
-      <c r="E6" s="22">
+      <c r="E6" s="21">
         <v>20</v>
       </c>
       <c r="F6" t="s">
@@ -2157,8 +2221,8 @@
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="72"/>
-      <c r="B7" s="82"/>
+      <c r="A7" s="80"/>
+      <c r="B7" s="91"/>
       <c r="C7" t="s">
         <v>15</v>
       </c>
@@ -2173,65 +2237,65 @@
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="72"/>
-      <c r="B8" s="83" t="s">
+      <c r="A8" s="80"/>
+      <c r="B8" s="92" t="s">
         <v>234</v>
       </c>
-      <c r="C8" s="36" t="s">
+      <c r="C8" s="35" t="s">
         <v>85</v>
       </c>
-      <c r="D8" s="36" t="s">
+      <c r="D8" s="35" t="s">
         <v>236</v>
       </c>
-      <c r="E8" s="37">
+      <c r="E8" s="36">
         <v>1.5</v>
       </c>
-      <c r="F8" s="36" t="s">
+      <c r="F8" s="35" t="s">
         <v>235</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="72"/>
-      <c r="B9" s="84"/>
-      <c r="C9" s="46" t="s">
+      <c r="A9" s="80"/>
+      <c r="B9" s="93"/>
+      <c r="C9" s="45" t="s">
         <v>86</v>
       </c>
-      <c r="D9" s="46" t="s">
+      <c r="D9" s="45" t="s">
         <v>237</v>
       </c>
-      <c r="E9" s="55">
+      <c r="E9" s="54">
         <v>285.39999999999998</v>
       </c>
-      <c r="F9" s="46" t="s">
+      <c r="F9" s="45" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" s="72"/>
-      <c r="B10" s="84"/>
+      <c r="A10" s="80"/>
+      <c r="B10" s="93"/>
       <c r="C10" s="13" t="s">
         <v>10</v>
       </c>
       <c r="D10" s="13" t="s">
         <v>238</v>
       </c>
-      <c r="E10" s="32">
+      <c r="E10" s="31">
         <v>5000</v>
       </c>
-      <c r="F10" s="32" t="s">
+      <c r="F10" s="31" t="s">
         <v>243</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="72"/>
-      <c r="B11" s="84"/>
+      <c r="A11" s="80"/>
+      <c r="B11" s="93"/>
       <c r="C11" s="13" t="s">
         <v>11</v>
       </c>
       <c r="D11" s="13" t="s">
         <v>239</v>
       </c>
-      <c r="E11" s="34">
+      <c r="E11" s="33">
         <v>0.05</v>
       </c>
       <c r="F11" s="13" t="s">
@@ -2239,15 +2303,15 @@
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" s="72"/>
-      <c r="B12" s="84"/>
+      <c r="A12" s="80"/>
+      <c r="B12" s="93"/>
       <c r="C12" s="13" t="s">
         <v>87</v>
       </c>
       <c r="D12" s="13" t="s">
         <v>240</v>
       </c>
-      <c r="E12" s="32">
+      <c r="E12" s="31">
         <v>0.189</v>
       </c>
       <c r="F12" s="13" t="s">
@@ -2255,31 +2319,31 @@
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" s="72"/>
-      <c r="B13" s="84"/>
-      <c r="C13" s="46" t="s">
+      <c r="A13" s="80"/>
+      <c r="B13" s="93"/>
+      <c r="C13" s="45" t="s">
         <v>254</v>
       </c>
-      <c r="D13" s="46" t="s">
+      <c r="D13" s="45" t="s">
         <v>245</v>
       </c>
-      <c r="E13" s="55">
+      <c r="E13" s="54">
         <v>1.375</v>
       </c>
-      <c r="F13" s="46" t="s">
+      <c r="F13" s="45" t="s">
         <v>246</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" s="72"/>
-      <c r="B14" s="84"/>
+      <c r="A14" s="80"/>
+      <c r="B14" s="93"/>
       <c r="C14" s="13" t="s">
         <v>13</v>
       </c>
       <c r="D14" s="13" t="s">
         <v>241</v>
       </c>
-      <c r="E14" s="35">
+      <c r="E14" s="34">
         <v>25</v>
       </c>
       <c r="F14" s="13" t="s">
@@ -2287,222 +2351,222 @@
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A15" s="72"/>
-      <c r="B15" s="85"/>
-      <c r="C15" s="38" t="s">
+      <c r="A15" s="80"/>
+      <c r="B15" s="94"/>
+      <c r="C15" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="D15" s="38" t="s">
+      <c r="D15" s="37" t="s">
         <v>242</v>
       </c>
-      <c r="E15" s="39">
+      <c r="E15" s="38">
         <v>0.08</v>
       </c>
-      <c r="F15" s="38" t="s">
+      <c r="F15" s="37" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A16" s="72"/>
-      <c r="B16" s="83" t="s">
-        <v>300</v>
-      </c>
-      <c r="C16" s="36" t="s">
+      <c r="A16" s="80"/>
+      <c r="B16" s="92" t="s">
+        <v>299</v>
+      </c>
+      <c r="C16" s="35" t="s">
         <v>8</v>
       </c>
-      <c r="D16" s="36" t="s">
+      <c r="D16" s="35" t="s">
+        <v>302</v>
+      </c>
+      <c r="E16" s="70">
+        <v>3.7</v>
+      </c>
+      <c r="F16" s="35" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" s="80"/>
+      <c r="B17" s="96"/>
+      <c r="C17" s="52" t="s">
+        <v>85</v>
+      </c>
+      <c r="D17" s="52" t="s">
         <v>303</v>
       </c>
-      <c r="E16" s="103">
-        <v>3.7</v>
-      </c>
-      <c r="F16" s="36" t="s">
+      <c r="E17" s="71">
+        <v>0.27</v>
+      </c>
+      <c r="F17" s="78" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" s="80"/>
+      <c r="B18" s="96"/>
+      <c r="C18" s="52" t="s">
+        <v>10</v>
+      </c>
+      <c r="D18" s="52" t="s">
+        <v>304</v>
+      </c>
+      <c r="E18" s="71">
+        <v>700</v>
+      </c>
+      <c r="F18" s="52" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" s="80"/>
+      <c r="B19" s="96"/>
+      <c r="C19" s="52" t="s">
+        <v>11</v>
+      </c>
+      <c r="D19" s="52" t="s">
+        <v>305</v>
+      </c>
+      <c r="E19" s="71">
+        <v>0.02</v>
+      </c>
+      <c r="F19" s="52" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20" s="80"/>
+      <c r="B20" s="96"/>
+      <c r="C20" s="52" t="s">
+        <v>13</v>
+      </c>
+      <c r="D20" s="52" t="s">
+        <v>306</v>
+      </c>
+      <c r="E20" s="71">
+        <v>20</v>
+      </c>
+      <c r="F20" s="52" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A21" s="80"/>
+      <c r="B21" s="94"/>
+      <c r="C21" s="37" t="s">
+        <v>15</v>
+      </c>
+      <c r="D21" s="37" t="s">
+        <v>307</v>
+      </c>
+      <c r="E21" s="72">
+        <v>0.05</v>
+      </c>
+      <c r="F21" s="37" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" s="72"/>
-      <c r="B17" s="87"/>
-      <c r="C17" s="53" t="s">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A22" s="80"/>
+      <c r="B22" s="95" t="s">
+        <v>233</v>
+      </c>
+      <c r="C22" s="45" t="s">
         <v>85</v>
       </c>
-      <c r="D17" s="53" t="s">
-        <v>304</v>
-      </c>
-      <c r="E17" s="104">
-        <v>0.27</v>
-      </c>
-      <c r="F17" s="53" t="s">
+      <c r="D22" s="45" t="s">
+        <v>247</v>
+      </c>
+      <c r="E22" s="54">
+        <v>0.5</v>
+      </c>
+      <c r="F22" s="45" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A23" s="80"/>
+      <c r="B23" s="95"/>
+      <c r="C23" s="45" t="s">
         <v>309</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" s="72"/>
-      <c r="B18" s="87"/>
-      <c r="C18" s="53" t="s">
+      <c r="D23" s="45" t="s">
+        <v>310</v>
+      </c>
+      <c r="E23" s="54">
+        <v>1.75</v>
+      </c>
+      <c r="F23" s="45" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A24" s="80"/>
+      <c r="B24" s="95"/>
+      <c r="C24" s="45" t="s">
         <v>10</v>
       </c>
-      <c r="D18" s="53" t="s">
-        <v>305</v>
-      </c>
-      <c r="E18" s="104">
-        <v>700</v>
-      </c>
-      <c r="F18" s="53" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" s="72"/>
-      <c r="B19" s="87"/>
-      <c r="C19" s="53" t="s">
+      <c r="D24" s="45" t="s">
+        <v>248</v>
+      </c>
+      <c r="E24" s="54">
+        <v>7000</v>
+      </c>
+      <c r="F24" s="45" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A25" s="80"/>
+      <c r="B25" s="95"/>
+      <c r="C25" s="45" t="s">
         <v>11</v>
       </c>
-      <c r="D19" s="53" t="s">
-        <v>306</v>
-      </c>
-      <c r="E19" s="104">
-        <v>0.02</v>
-      </c>
-      <c r="F19" s="53" t="s">
+      <c r="D25" s="45" t="s">
+        <v>249</v>
+      </c>
+      <c r="E25" s="57">
+        <v>0.05</v>
+      </c>
+      <c r="F25" s="45" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" s="72"/>
-      <c r="B20" s="87"/>
-      <c r="C20" s="53" t="s">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A26" s="80"/>
+      <c r="B26" s="95"/>
+      <c r="C26" s="45" t="s">
         <v>13</v>
       </c>
-      <c r="D20" s="53" t="s">
-        <v>307</v>
-      </c>
-      <c r="E20" s="104">
-        <v>20</v>
-      </c>
-      <c r="F20" s="53" t="s">
+      <c r="D26" s="45" t="s">
+        <v>250</v>
+      </c>
+      <c r="E26" s="58">
+        <v>15</v>
+      </c>
+      <c r="F26" s="45" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A21" s="72"/>
-      <c r="B21" s="85"/>
-      <c r="C21" s="38" t="s">
+    <row r="27" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="80"/>
+      <c r="B27" s="95"/>
+      <c r="C27" s="45" t="s">
         <v>15</v>
       </c>
-      <c r="D21" s="38" t="s">
-        <v>308</v>
-      </c>
-      <c r="E21" s="105">
-        <v>0.05</v>
-      </c>
-      <c r="F21" s="38" t="s">
+      <c r="D27" s="45" t="s">
+        <v>251</v>
+      </c>
+      <c r="E27" s="57">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="F27" s="45" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A22" s="72"/>
-      <c r="B22" s="86" t="s">
-        <v>233</v>
-      </c>
-      <c r="C22" s="46" t="s">
-        <v>85</v>
-      </c>
-      <c r="D22" s="46" t="s">
-        <v>247</v>
-      </c>
-      <c r="E22" s="55">
-        <v>0.5</v>
-      </c>
-      <c r="F22" s="46" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" s="72"/>
-      <c r="B23" s="86"/>
-      <c r="C23" s="46" t="s">
-        <v>311</v>
-      </c>
-      <c r="D23" s="46" t="s">
-        <v>312</v>
-      </c>
-      <c r="E23" s="55">
-        <v>1.75</v>
-      </c>
-      <c r="F23" s="46" t="s">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" s="72"/>
-      <c r="B24" s="86"/>
-      <c r="C24" s="46" t="s">
-        <v>10</v>
-      </c>
-      <c r="D24" s="46" t="s">
-        <v>248</v>
-      </c>
-      <c r="E24" s="55">
-        <v>7000</v>
-      </c>
-      <c r="F24" s="46" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25" s="72"/>
-      <c r="B25" s="86"/>
-      <c r="C25" s="46" t="s">
-        <v>11</v>
-      </c>
-      <c r="D25" s="46" t="s">
-        <v>249</v>
-      </c>
-      <c r="E25" s="58">
-        <v>0.05</v>
-      </c>
-      <c r="F25" s="46" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26" s="72"/>
-      <c r="B26" s="86"/>
-      <c r="C26" s="46" t="s">
-        <v>13</v>
-      </c>
-      <c r="D26" s="46" t="s">
-        <v>250</v>
-      </c>
-      <c r="E26" s="59">
-        <v>15</v>
-      </c>
-      <c r="F26" s="46" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="72"/>
-      <c r="B27" s="86"/>
-      <c r="C27" s="46" t="s">
-        <v>15</v>
-      </c>
-      <c r="D27" s="46" t="s">
-        <v>251</v>
-      </c>
-      <c r="E27" s="58">
-        <v>7.0000000000000007E-2</v>
-      </c>
-      <c r="F27" s="46" t="s">
-        <v>22</v>
-      </c>
-    </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A28" s="71" t="s">
+      <c r="A28" s="79" t="s">
         <v>72</v>
       </c>
-      <c r="B28" s="74" t="s">
+      <c r="B28" s="83" t="s">
         <v>3</v>
       </c>
       <c r="C28" s="2" t="s">
@@ -2511,16 +2575,16 @@
       <c r="D28" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="E28" s="23">
+      <c r="E28" s="22">
         <v>490</v>
       </c>
-      <c r="F28" s="27" t="s">
+      <c r="F28" s="26" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A29" s="72"/>
-      <c r="B29" s="75"/>
+      <c r="A29" s="80"/>
+      <c r="B29" s="84"/>
       <c r="C29" t="s">
         <v>11</v>
       </c>
@@ -2535,15 +2599,15 @@
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A30" s="72"/>
-      <c r="B30" s="75"/>
+      <c r="A30" s="80"/>
+      <c r="B30" s="84"/>
       <c r="C30" t="s">
         <v>13</v>
       </c>
       <c r="D30" t="s">
         <v>32</v>
       </c>
-      <c r="E30" s="22">
+      <c r="E30" s="21">
         <v>20</v>
       </c>
       <c r="F30" t="s">
@@ -2551,15 +2615,15 @@
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A31" s="72"/>
-      <c r="B31" s="75"/>
+      <c r="A31" s="80"/>
+      <c r="B31" s="84"/>
       <c r="C31" t="s">
         <v>20</v>
       </c>
       <c r="D31" t="s">
         <v>34</v>
       </c>
-      <c r="E31" s="48">
+      <c r="E31" s="47">
         <v>1.0000000000000001E-5</v>
       </c>
       <c r="F31" s="13" t="s">
@@ -2567,8 +2631,8 @@
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A32" s="72"/>
-      <c r="B32" s="75"/>
+      <c r="A32" s="80"/>
+      <c r="B32" s="84"/>
       <c r="C32" t="s">
         <v>35</v>
       </c>
@@ -2583,8 +2647,8 @@
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A33" s="72"/>
-      <c r="B33" s="75"/>
+      <c r="A33" s="80"/>
+      <c r="B33" s="84"/>
       <c r="C33" t="s">
         <v>36</v>
       </c>
@@ -2599,8 +2663,8 @@
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A34" s="72"/>
-      <c r="B34" s="75"/>
+      <c r="A34" s="80"/>
+      <c r="B34" s="84"/>
       <c r="C34" t="s">
         <v>15</v>
       </c>
@@ -2615,8 +2679,8 @@
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A35" s="72"/>
-      <c r="B35" s="75"/>
+      <c r="A35" s="80"/>
+      <c r="B35" s="84"/>
       <c r="C35" t="s">
         <v>89</v>
       </c>
@@ -2631,8 +2695,8 @@
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A36" s="72"/>
-      <c r="B36" s="76" t="s">
+      <c r="A36" s="80"/>
+      <c r="B36" s="85" t="s">
         <v>205</v>
       </c>
       <c r="C36" s="4" t="s">
@@ -2649,153 +2713,153 @@
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A37" s="72"/>
-      <c r="B37" s="79"/>
-      <c r="C37" s="49" t="s">
+      <c r="A37" s="80"/>
+      <c r="B37" s="88"/>
+      <c r="C37" s="48" t="s">
         <v>21</v>
       </c>
-      <c r="D37" s="49" t="s">
+      <c r="D37" s="48" t="s">
         <v>55</v>
       </c>
-      <c r="E37" s="50">
+      <c r="E37" s="49">
         <f>E38*4</f>
         <v>424</v>
       </c>
-      <c r="F37" s="49" t="s">
+      <c r="F37" s="48" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A38" s="72"/>
-      <c r="B38" s="79"/>
-      <c r="C38" s="49" t="s">
+      <c r="A38" s="80"/>
+      <c r="B38" s="88"/>
+      <c r="C38" s="48" t="s">
         <v>16</v>
       </c>
-      <c r="D38" s="49" t="s">
+      <c r="D38" s="48" t="s">
         <v>56</v>
       </c>
-      <c r="E38" s="50">
+      <c r="E38" s="49">
         <v>106</v>
       </c>
-      <c r="F38" s="49" t="s">
+      <c r="F38" s="48" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A39" s="72"/>
-      <c r="B39" s="79"/>
-      <c r="C39" s="49" t="s">
+      <c r="A39" s="80"/>
+      <c r="B39" s="88"/>
+      <c r="C39" s="48" t="s">
         <v>17</v>
       </c>
-      <c r="D39" s="49" t="s">
+      <c r="D39" s="48" t="s">
         <v>57</v>
       </c>
-      <c r="E39" s="51">
+      <c r="E39" s="50">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="F39" s="49" t="s">
+      <c r="F39" s="48" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A40" s="72"/>
-      <c r="B40" s="79"/>
-      <c r="C40" s="49" t="s">
+      <c r="A40" s="80"/>
+      <c r="B40" s="88"/>
+      <c r="C40" s="48" t="s">
         <v>18</v>
       </c>
-      <c r="D40" s="49" t="s">
+      <c r="D40" s="48" t="s">
         <v>58</v>
       </c>
-      <c r="E40" s="50">
+      <c r="E40" s="49">
         <v>0</v>
       </c>
-      <c r="F40" s="53" t="s">
+      <c r="F40" s="52" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A41" s="72"/>
-      <c r="B41" s="79"/>
-      <c r="C41" s="49" t="s">
+      <c r="A41" s="80"/>
+      <c r="B41" s="88"/>
+      <c r="C41" s="48" t="s">
         <v>35</v>
       </c>
-      <c r="D41" s="49" t="s">
+      <c r="D41" s="48" t="s">
         <v>60</v>
       </c>
-      <c r="E41" s="51">
+      <c r="E41" s="50">
         <v>0.93500000000000005</v>
       </c>
-      <c r="F41" s="49" t="s">
+      <c r="F41" s="48" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A42" s="72"/>
-      <c r="B42" s="79"/>
-      <c r="C42" s="49" t="s">
+      <c r="A42" s="80"/>
+      <c r="B42" s="88"/>
+      <c r="C42" s="48" t="s">
         <v>36</v>
       </c>
-      <c r="D42" s="49" t="s">
+      <c r="D42" s="48" t="s">
         <v>61</v>
       </c>
-      <c r="E42" s="51">
+      <c r="E42" s="50">
         <v>0.93500000000000005</v>
       </c>
-      <c r="F42" s="49" t="s">
+      <c r="F42" s="48" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A43" s="72"/>
-      <c r="B43" s="79"/>
-      <c r="C43" s="49" t="s">
+      <c r="A43" s="80"/>
+      <c r="B43" s="88"/>
+      <c r="C43" s="48" t="s">
         <v>90</v>
       </c>
-      <c r="D43" s="49" t="s">
+      <c r="D43" s="48" t="s">
         <v>59</v>
       </c>
-      <c r="E43" s="50">
+      <c r="E43" s="49">
         <v>0.25</v>
       </c>
-      <c r="F43" s="49" t="s">
+      <c r="F43" s="48" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A44" s="72"/>
-      <c r="B44" s="79"/>
-      <c r="C44" s="49" t="s">
+      <c r="A44" s="80"/>
+      <c r="B44" s="88"/>
+      <c r="C44" s="48" t="s">
         <v>89</v>
       </c>
-      <c r="D44" s="49" t="s">
+      <c r="D44" s="48" t="s">
         <v>62</v>
       </c>
-      <c r="E44" s="51">
+      <c r="E44" s="50">
         <v>0</v>
       </c>
-      <c r="F44" s="49" t="s">
+      <c r="F44" s="48" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A45" s="72"/>
-      <c r="B45" s="79"/>
-      <c r="C45" s="49" t="s">
+      <c r="A45" s="80"/>
+      <c r="B45" s="88"/>
+      <c r="C45" s="48" t="s">
         <v>13</v>
       </c>
-      <c r="D45" s="49" t="s">
+      <c r="D45" s="48" t="s">
         <v>54</v>
       </c>
-      <c r="E45" s="52">
+      <c r="E45" s="51">
         <v>15</v>
       </c>
-      <c r="F45" s="49" t="s">
+      <c r="F45" s="48" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="46" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A46" s="73"/>
-      <c r="B46" s="80"/>
+      <c r="A46" s="81"/>
+      <c r="B46" s="89"/>
       <c r="C46" s="15" t="s">
         <v>15</v>
       </c>
@@ -2810,7 +2874,7 @@
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A47" s="71" t="s">
+      <c r="A47" s="79" t="s">
         <v>73</v>
       </c>
       <c r="B47" s="11" t="s">
@@ -2822,7 +2886,7 @@
       <c r="D47" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="E47" s="23">
+      <c r="E47" s="22">
         <v>2000</v>
       </c>
       <c r="F47" s="2" t="s">
@@ -2830,8 +2894,8 @@
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A48" s="72"/>
-      <c r="B48" s="76" t="s">
+      <c r="A48" s="80"/>
+      <c r="B48" s="85" t="s">
         <v>4</v>
       </c>
       <c r="C48" s="4" t="s">
@@ -2848,15 +2912,15 @@
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A49" s="72"/>
-      <c r="B49" s="75"/>
+      <c r="A49" s="80"/>
+      <c r="B49" s="84"/>
       <c r="C49" t="s">
         <v>10</v>
       </c>
       <c r="D49" t="s">
         <v>43</v>
       </c>
-      <c r="E49" s="24">
+      <c r="E49" s="23">
         <v>1100</v>
       </c>
       <c r="F49" t="s">
@@ -2864,15 +2928,15 @@
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A50" s="72"/>
-      <c r="B50" s="75"/>
+      <c r="A50" s="80"/>
+      <c r="B50" s="84"/>
       <c r="C50" t="s">
         <v>17</v>
       </c>
       <c r="D50" t="s">
         <v>44</v>
       </c>
-      <c r="E50" s="24">
+      <c r="E50" s="23">
         <v>17.84</v>
       </c>
       <c r="F50" t="s">
@@ -2880,8 +2944,8 @@
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A51" s="72"/>
-      <c r="B51" s="75"/>
+      <c r="A51" s="80"/>
+      <c r="B51" s="84"/>
       <c r="C51" t="s">
         <v>18</v>
       </c>
@@ -2896,15 +2960,15 @@
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A52" s="72"/>
-      <c r="B52" s="75"/>
+      <c r="A52" s="80"/>
+      <c r="B52" s="84"/>
       <c r="C52" t="s">
         <v>13</v>
       </c>
       <c r="D52" t="s">
         <v>42</v>
       </c>
-      <c r="E52" s="22">
+      <c r="E52" s="21">
         <v>25</v>
       </c>
       <c r="F52" t="s">
@@ -2912,8 +2976,8 @@
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A53" s="72"/>
-      <c r="B53" s="75"/>
+      <c r="A53" s="80"/>
+      <c r="B53" s="84"/>
       <c r="C53" t="s">
         <v>69</v>
       </c>
@@ -2928,8 +2992,8 @@
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A54" s="72"/>
-      <c r="B54" s="77"/>
+      <c r="A54" s="80"/>
+      <c r="B54" s="86"/>
       <c r="C54" s="5" t="s">
         <v>15</v>
       </c>
@@ -2944,8 +3008,8 @@
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A55" s="72"/>
-      <c r="B55" s="76" t="s">
+      <c r="A55" s="80"/>
+      <c r="B55" s="85" t="s">
         <v>5</v>
       </c>
       <c r="C55" s="4" t="s">
@@ -2962,15 +3026,15 @@
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A56" s="72"/>
-      <c r="B56" s="75"/>
+      <c r="A56" s="80"/>
+      <c r="B56" s="84"/>
       <c r="C56" t="s">
         <v>10</v>
       </c>
       <c r="D56" t="s">
         <v>48</v>
       </c>
-      <c r="E56" s="24">
+      <c r="E56" s="23">
         <v>1080</v>
       </c>
       <c r="F56" t="s">
@@ -2978,31 +3042,31 @@
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A57" s="72"/>
-      <c r="B57" s="75"/>
+      <c r="A57" s="80"/>
+      <c r="B57" s="84"/>
       <c r="C57" t="s">
         <v>17</v>
       </c>
       <c r="D57" t="s">
         <v>52</v>
       </c>
-      <c r="E57" s="44">
+      <c r="E57" s="43">
         <v>12.68</v>
       </c>
-      <c r="F57" s="25" t="s">
+      <c r="F57" s="24" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A58" s="72"/>
-      <c r="B58" s="75"/>
+      <c r="A58" s="80"/>
+      <c r="B58" s="84"/>
       <c r="C58" t="s">
         <v>18</v>
       </c>
       <c r="D58" t="s">
         <v>49</v>
       </c>
-      <c r="E58" s="47">
+      <c r="E58" s="46">
         <v>5.0000000000000001E-3</v>
       </c>
       <c r="F58" t="s">
@@ -3010,15 +3074,15 @@
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A59" s="72"/>
-      <c r="B59" s="75"/>
+      <c r="A59" s="80"/>
+      <c r="B59" s="84"/>
       <c r="C59" t="s">
         <v>13</v>
       </c>
       <c r="D59" t="s">
         <v>50</v>
       </c>
-      <c r="E59" s="22">
+      <c r="E59" s="21">
         <v>25</v>
       </c>
       <c r="F59" t="s">
@@ -3026,15 +3090,15 @@
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A60" s="72"/>
-      <c r="B60" s="75"/>
+      <c r="A60" s="80"/>
+      <c r="B60" s="84"/>
       <c r="C60" t="s">
         <v>69</v>
       </c>
       <c r="D60" t="s">
         <v>66</v>
       </c>
-      <c r="E60" s="26">
+      <c r="E60" s="25">
         <v>1000000</v>
       </c>
       <c r="F60" t="s">
@@ -3042,8 +3106,8 @@
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A61" s="73"/>
-      <c r="B61" s="78"/>
+      <c r="A61" s="81"/>
+      <c r="B61" s="87"/>
       <c r="C61" s="15" t="s">
         <v>15</v>
       </c>
@@ -3058,59 +3122,77 @@
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A62" s="71" t="s">
+      <c r="A62" s="79" t="s">
         <v>77</v>
       </c>
-      <c r="B62" s="17" t="s">
+      <c r="B62" s="74" t="s">
         <v>74</v>
       </c>
-      <c r="C62" s="2" t="s">
+      <c r="C62" s="75" t="s">
         <v>78</v>
       </c>
-      <c r="D62" s="2" t="s">
+      <c r="D62" s="75" t="s">
         <v>79</v>
       </c>
-      <c r="E62" s="3">
+      <c r="E62" s="76">
         <v>-1E-4</v>
       </c>
-      <c r="F62" s="2" t="s">
+      <c r="F62" s="75" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A63" s="72"/>
-      <c r="B63" s="18" t="s">
+      <c r="A63" s="82"/>
+      <c r="B63" s="73" t="s">
+        <v>328</v>
+      </c>
+      <c r="C63" s="77" t="s">
+        <v>329</v>
+      </c>
+      <c r="D63" s="77" t="s">
+        <v>330</v>
+      </c>
+      <c r="E63" s="50">
+        <v>-1E-4</v>
+      </c>
+      <c r="F63" s="77" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A64" s="80"/>
+      <c r="B64" s="17" t="s">
         <v>80</v>
       </c>
-      <c r="C63" s="19" t="s">
+      <c r="C64" s="18" t="s">
         <v>81</v>
       </c>
-      <c r="D63" s="19" t="s">
+      <c r="D64" s="18" t="s">
         <v>82</v>
       </c>
-      <c r="E63" s="20">
+      <c r="E64" s="19">
         <v>-1.5</v>
       </c>
-      <c r="F63" s="19" t="s">
+      <c r="F64" s="18" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A64" s="73"/>
-      <c r="B64" s="1" t="s">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A65" s="81"/>
+      <c r="B65" s="1" t="s">
         <v>278</v>
       </c>
-      <c r="C64" s="15" t="s">
+      <c r="C65" s="15" t="s">
+        <v>300</v>
+      </c>
+      <c r="D65" s="15" t="s">
+        <v>298</v>
+      </c>
+      <c r="E65" s="16">
+        <v>-0.6</v>
+      </c>
+      <c r="F65" s="15" t="s">
         <v>301</v>
-      </c>
-      <c r="D64" s="15" t="s">
-        <v>299</v>
-      </c>
-      <c r="E64" s="16">
-        <v>-0.6</v>
-      </c>
-      <c r="F64" s="15" t="s">
-        <v>302</v>
       </c>
     </row>
   </sheetData>
@@ -3118,7 +3200,7 @@
     <mergeCell ref="A2:A27"/>
     <mergeCell ref="A28:A46"/>
     <mergeCell ref="A47:A61"/>
-    <mergeCell ref="A62:A64"/>
+    <mergeCell ref="A62:A65"/>
     <mergeCell ref="B28:B35"/>
     <mergeCell ref="B48:B54"/>
     <mergeCell ref="B55:B61"/>
@@ -3136,12 +3218,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83AB2E79-6F94-41B5-A552-C40EC4890194}">
-  <dimension ref="A1:F120"/>
+  <dimension ref="A1:F127"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.5546875" style="13" customWidth="1"/>
     <col min="2" max="2" width="30.33203125" style="13" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="37.109375" style="13" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="38.5546875" style="13" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="50.77734375" style="13" customWidth="1"/>
     <col min="5" max="5" width="46.109375" style="13" customWidth="1"/>
     <col min="6" max="6" width="37.5546875" style="13" customWidth="1"/>
@@ -3149,1630 +3231,1731 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="27" t="s">
         <v>70</v>
       </c>
-      <c r="B1" s="29" t="s">
+      <c r="B1" s="28" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="29" t="s">
+      <c r="C1" s="28" t="s">
         <v>24</v>
       </c>
-      <c r="D1" s="29" t="s">
+      <c r="D1" s="28" t="s">
         <v>23</v>
       </c>
-      <c r="E1" s="30" t="s">
+      <c r="E1" s="29" t="s">
         <v>7</v>
       </c>
-      <c r="F1" s="29" t="s">
+      <c r="F1" s="28" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="92" t="s">
+      <c r="A2" s="97" t="s">
         <v>71</v>
       </c>
-      <c r="B2" s="91" t="s">
+      <c r="B2" s="99" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="27" t="s">
+      <c r="C2" s="26" t="s">
         <v>98</v>
       </c>
-      <c r="D2" s="27" t="s">
+      <c r="D2" s="26" t="s">
         <v>99</v>
       </c>
-      <c r="E2" s="31"/>
-      <c r="F2" s="27" t="s">
+      <c r="E2" s="30"/>
+      <c r="F2" s="26" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="94"/>
-      <c r="B3" s="84"/>
+      <c r="A3" s="98"/>
+      <c r="B3" s="93"/>
       <c r="C3" s="13" t="s">
         <v>109</v>
       </c>
       <c r="D3" s="13" t="s">
         <v>117</v>
       </c>
-      <c r="E3" s="32"/>
+      <c r="E3" s="31"/>
       <c r="F3" s="13" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="94"/>
-      <c r="B4" s="84"/>
+      <c r="A4" s="98"/>
+      <c r="B4" s="93"/>
       <c r="C4" s="13" t="s">
         <v>85</v>
       </c>
       <c r="D4" s="13" t="s">
         <v>125</v>
       </c>
-      <c r="E4" s="33"/>
+      <c r="E4" s="32"/>
       <c r="F4" s="13" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="94"/>
-      <c r="B5" s="84"/>
+      <c r="A5" s="98"/>
+      <c r="B5" s="93"/>
       <c r="C5" s="13" t="s">
         <v>140</v>
       </c>
       <c r="D5" s="13" t="s">
         <v>139</v>
       </c>
-      <c r="E5" s="34"/>
+      <c r="E5" s="33"/>
       <c r="F5" s="13" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="94"/>
-      <c r="B6" s="84"/>
+      <c r="A6" s="98"/>
+      <c r="B6" s="93"/>
       <c r="C6" s="13" t="s">
         <v>143</v>
       </c>
       <c r="D6" s="13" t="s">
         <v>145</v>
       </c>
-      <c r="E6" s="35"/>
+      <c r="E6" s="34"/>
       <c r="F6" s="13" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="94"/>
-      <c r="B7" s="84"/>
+      <c r="A7" s="98"/>
+      <c r="B7" s="93"/>
       <c r="C7" s="13" t="s">
         <v>157</v>
       </c>
       <c r="D7" s="13" t="s">
         <v>160</v>
       </c>
-      <c r="E7" s="35"/>
+      <c r="E7" s="34"/>
       <c r="F7" s="13" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="94"/>
-      <c r="B8" s="84"/>
+      <c r="A8" s="98"/>
+      <c r="B8" s="93"/>
       <c r="C8" s="13" t="s">
         <v>200</v>
       </c>
       <c r="D8" s="13" t="s">
         <v>199</v>
       </c>
-      <c r="E8" s="35"/>
+      <c r="E8" s="34"/>
       <c r="F8" s="13" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="94"/>
-      <c r="B9" s="84"/>
+      <c r="A9" s="98"/>
+      <c r="B9" s="93"/>
       <c r="C9" s="13" t="s">
         <v>169</v>
       </c>
       <c r="D9" s="13" t="s">
         <v>168</v>
       </c>
-      <c r="E9" s="35"/>
+      <c r="E9" s="34"/>
       <c r="F9" s="13" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="94"/>
-      <c r="B10" s="84"/>
+      <c r="A10" s="98"/>
+      <c r="B10" s="93"/>
       <c r="C10" s="13" t="s">
         <v>192</v>
       </c>
       <c r="D10" s="13" t="s">
         <v>198</v>
       </c>
-      <c r="E10" s="35"/>
+      <c r="E10" s="34"/>
       <c r="F10" s="13" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" s="94"/>
-      <c r="B11" s="84"/>
-      <c r="E11" s="34"/>
+      <c r="A11" s="98"/>
+      <c r="B11" s="93"/>
+      <c r="E11" s="33"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="94"/>
-      <c r="B12" s="88" t="s">
+      <c r="A12" s="98"/>
+      <c r="B12" s="100" t="s">
         <v>234</v>
       </c>
-      <c r="C12" s="56" t="s">
+      <c r="C12" s="55" t="s">
         <v>98</v>
       </c>
-      <c r="D12" s="56" t="s">
+      <c r="D12" s="55" t="s">
         <v>255</v>
       </c>
-      <c r="E12" s="57"/>
-      <c r="F12" s="56" t="s">
+      <c r="E12" s="56"/>
+      <c r="F12" s="55" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="94"/>
-      <c r="B13" s="89"/>
-      <c r="C13" s="46" t="s">
+      <c r="A13" s="98"/>
+      <c r="B13" s="101"/>
+      <c r="C13" s="45" t="s">
         <v>263</v>
       </c>
-      <c r="D13" s="46" t="s">
-        <v>330</v>
-      </c>
-      <c r="E13" s="55"/>
-      <c r="F13" s="46" t="s">
+      <c r="D13" s="45" t="s">
+        <v>327</v>
+      </c>
+      <c r="E13" s="54"/>
+      <c r="F13" s="45" t="s">
         <v>266</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" s="94"/>
-      <c r="B14" s="89"/>
-      <c r="C14" s="46" t="s">
+      <c r="A14" s="98"/>
+      <c r="B14" s="101"/>
+      <c r="C14" s="45" t="s">
         <v>141</v>
       </c>
-      <c r="D14" s="46" t="s">
+      <c r="D14" s="45" t="s">
         <v>256</v>
       </c>
-      <c r="E14" s="55"/>
-      <c r="F14" s="55" t="s">
+      <c r="E14" s="54"/>
+      <c r="F14" s="54" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" s="94"/>
-      <c r="B15" s="89"/>
-      <c r="C15" s="46" t="s">
+      <c r="A15" s="98"/>
+      <c r="B15" s="101"/>
+      <c r="C15" s="45" t="s">
         <v>264</v>
       </c>
-      <c r="D15" s="46" t="s">
+      <c r="D15" s="45" t="s">
         <v>265</v>
       </c>
-      <c r="E15" s="58"/>
-      <c r="F15" s="46" t="s">
+      <c r="E15" s="57"/>
+      <c r="F15" s="45" t="s">
         <v>267</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" s="94"/>
-      <c r="B16" s="89"/>
-      <c r="C16" s="46" t="s">
+      <c r="A16" s="98"/>
+      <c r="B16" s="101"/>
+      <c r="C16" s="45" t="s">
         <v>85</v>
       </c>
-      <c r="D16" s="46" t="s">
+      <c r="D16" s="45" t="s">
         <v>257</v>
       </c>
-      <c r="E16" s="55"/>
-      <c r="F16" s="46" t="s">
+      <c r="E16" s="54"/>
+      <c r="F16" s="45" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" s="94"/>
-      <c r="B17" s="89"/>
-      <c r="C17" s="46" t="s">
+      <c r="A17" s="98"/>
+      <c r="B17" s="101"/>
+      <c r="C17" s="45" t="s">
         <v>143</v>
       </c>
-      <c r="D17" s="46" t="s">
+      <c r="D17" s="45" t="s">
         <v>258</v>
       </c>
-      <c r="E17" s="55"/>
-      <c r="F17" s="46" t="s">
+      <c r="E17" s="54"/>
+      <c r="F17" s="45" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" s="94"/>
-      <c r="B18" s="89"/>
-      <c r="C18" s="46" t="s">
+      <c r="A18" s="98"/>
+      <c r="B18" s="101"/>
+      <c r="C18" s="45" t="s">
         <v>157</v>
       </c>
-      <c r="D18" s="46" t="s">
+      <c r="D18" s="45" t="s">
         <v>259</v>
       </c>
-      <c r="E18" s="59"/>
-      <c r="F18" s="46" t="s">
+      <c r="E18" s="58"/>
+      <c r="F18" s="45" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" s="94"/>
-      <c r="B19" s="89"/>
-      <c r="C19" s="46" t="s">
+      <c r="A19" s="98"/>
+      <c r="B19" s="101"/>
+      <c r="C19" s="45" t="s">
         <v>200</v>
       </c>
-      <c r="D19" s="46" t="s">
+      <c r="D19" s="45" t="s">
         <v>260</v>
       </c>
-      <c r="E19" s="59"/>
-      <c r="F19" s="46" t="s">
+      <c r="E19" s="58"/>
+      <c r="F19" s="45" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" s="94"/>
-      <c r="B20" s="89"/>
-      <c r="C20" s="46" t="s">
+      <c r="A20" s="98"/>
+      <c r="B20" s="101"/>
+      <c r="C20" s="45" t="s">
         <v>169</v>
       </c>
-      <c r="D20" s="46" t="s">
+      <c r="D20" s="45" t="s">
         <v>261</v>
       </c>
-      <c r="E20" s="59"/>
-      <c r="F20" s="46" t="s">
+      <c r="E20" s="58"/>
+      <c r="F20" s="45" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A21" s="94"/>
-      <c r="B21" s="89"/>
-      <c r="C21" s="46" t="s">
+      <c r="A21" s="98"/>
+      <c r="B21" s="101"/>
+      <c r="C21" s="45" t="s">
         <v>192</v>
       </c>
-      <c r="D21" s="46" t="s">
+      <c r="D21" s="45" t="s">
         <v>262</v>
       </c>
-      <c r="E21" s="59"/>
-      <c r="F21" s="46" t="s">
+      <c r="E21" s="58"/>
+      <c r="F21" s="45" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A22" s="94"/>
-      <c r="B22" s="99"/>
-      <c r="C22" s="60"/>
-      <c r="D22" s="60"/>
-      <c r="E22" s="61"/>
-      <c r="F22" s="60"/>
+      <c r="A22" s="98"/>
+      <c r="B22" s="102"/>
+      <c r="C22" s="59"/>
+      <c r="D22" s="59"/>
+      <c r="E22" s="60"/>
+      <c r="F22" s="59"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" s="94"/>
-      <c r="B23" s="88" t="s">
-        <v>300</v>
-      </c>
-      <c r="C23" s="46" t="s">
+      <c r="A23" s="98"/>
+      <c r="B23" s="100" t="s">
+        <v>299</v>
+      </c>
+      <c r="C23" s="45" t="s">
         <v>98</v>
       </c>
-      <c r="D23" s="46" t="s">
+      <c r="D23" s="45" t="s">
+        <v>312</v>
+      </c>
+      <c r="E23" s="54"/>
+      <c r="F23" s="45" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A24" s="98"/>
+      <c r="B24" s="108"/>
+      <c r="C24" s="45" t="s">
+        <v>109</v>
+      </c>
+      <c r="D24" s="45" t="s">
+        <v>313</v>
+      </c>
+      <c r="E24" s="54"/>
+      <c r="F24" s="45" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A25" s="98"/>
+      <c r="B25" s="108"/>
+      <c r="C25" s="45" t="s">
+        <v>85</v>
+      </c>
+      <c r="D25" s="45" t="s">
         <v>314</v>
       </c>
-      <c r="E23" s="55"/>
-      <c r="F23" s="46" t="s">
+      <c r="E25" s="57"/>
+      <c r="F25" s="45" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A26" s="98"/>
+      <c r="B26" s="108"/>
+      <c r="C26" s="45" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" s="94"/>
-      <c r="B24" s="106"/>
-      <c r="C24" s="46" t="s">
+      <c r="D26" s="45" t="s">
+        <v>323</v>
+      </c>
+      <c r="E26" s="58"/>
+      <c r="F26" s="45" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A27" s="98"/>
+      <c r="B27" s="108"/>
+      <c r="C27" s="45" t="s">
+        <v>143</v>
+      </c>
+      <c r="D27" s="45" t="s">
+        <v>315</v>
+      </c>
+      <c r="E27" s="58"/>
+      <c r="F27" s="45" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A28" s="98"/>
+      <c r="B28" s="108"/>
+      <c r="C28" s="45" t="s">
+        <v>157</v>
+      </c>
+      <c r="D28" s="45" t="s">
+        <v>316</v>
+      </c>
+      <c r="E28" s="58"/>
+      <c r="F28" s="45" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A29" s="98"/>
+      <c r="B29" s="108"/>
+      <c r="C29" s="45" t="s">
+        <v>200</v>
+      </c>
+      <c r="D29" s="45" t="s">
+        <v>317</v>
+      </c>
+      <c r="E29" s="58"/>
+      <c r="F29" s="45" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A30" s="98"/>
+      <c r="B30" s="108"/>
+      <c r="C30" s="45" t="s">
+        <v>169</v>
+      </c>
+      <c r="D30" s="45" t="s">
+        <v>318</v>
+      </c>
+      <c r="E30" s="57"/>
+      <c r="F30" s="45" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A31" s="98"/>
+      <c r="B31" s="108"/>
+      <c r="C31" s="45" t="s">
+        <v>192</v>
+      </c>
+      <c r="D31" s="45" t="s">
+        <v>319</v>
+      </c>
+      <c r="E31" s="57"/>
+      <c r="F31" s="45" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A32" s="98"/>
+      <c r="B32" s="102"/>
+      <c r="C32" s="59"/>
+      <c r="D32" s="59"/>
+      <c r="E32" s="60"/>
+      <c r="F32" s="59"/>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A33" s="98"/>
+      <c r="B33" s="103" t="s">
+        <v>233</v>
+      </c>
+      <c r="C33" s="45" t="s">
+        <v>98</v>
+      </c>
+      <c r="D33" s="45" t="s">
+        <v>268</v>
+      </c>
+      <c r="E33" s="54"/>
+      <c r="F33" s="45" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A34" s="98"/>
+      <c r="B34" s="103"/>
+      <c r="C34" s="45" t="s">
         <v>109</v>
       </c>
-      <c r="D24" s="46" t="s">
-        <v>315</v>
-      </c>
-      <c r="E24" s="55"/>
-      <c r="F24" s="46" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25" s="94"/>
-      <c r="B25" s="106"/>
-      <c r="C25" s="46" t="s">
+      <c r="D34" s="45" t="s">
+        <v>269</v>
+      </c>
+      <c r="E34" s="54"/>
+      <c r="F34" s="45" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A35" s="98"/>
+      <c r="B35" s="103"/>
+      <c r="C35" s="45" t="s">
         <v>85</v>
       </c>
-      <c r="D25" s="46" t="s">
-        <v>316</v>
-      </c>
-      <c r="E25" s="58"/>
-      <c r="F25" s="46" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26" s="94"/>
-      <c r="B26" s="106"/>
-      <c r="C26" s="46" t="s">
+      <c r="D35" s="45" t="s">
+        <v>270</v>
+      </c>
+      <c r="E35" s="57"/>
+      <c r="F35" s="45" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A36" s="98"/>
+      <c r="B36" s="103"/>
+      <c r="C36" s="45" t="s">
+        <v>309</v>
+      </c>
+      <c r="D36" s="45" t="s">
+        <v>326</v>
+      </c>
+      <c r="E36" s="57"/>
+      <c r="F36" s="45" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A37" s="98"/>
+      <c r="B37" s="103"/>
+      <c r="C37" s="45" t="s">
+        <v>276</v>
+      </c>
+      <c r="D37" s="45" t="s">
         <v>325</v>
       </c>
-      <c r="D26" s="46" t="s">
-        <v>326</v>
-      </c>
-      <c r="E26" s="59"/>
-      <c r="F26" s="46" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A27" s="94"/>
-      <c r="B27" s="106"/>
-      <c r="C27" s="46" t="s">
+      <c r="E37" s="58"/>
+      <c r="F37" s="45" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A38" s="98"/>
+      <c r="B38" s="103"/>
+      <c r="C38" s="45" t="s">
         <v>143</v>
       </c>
-      <c r="D27" s="46" t="s">
-        <v>317</v>
-      </c>
-      <c r="E27" s="59"/>
-      <c r="F27" s="46" t="s">
+      <c r="D38" s="45" t="s">
+        <v>271</v>
+      </c>
+      <c r="E38" s="58"/>
+      <c r="F38" s="45" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A28" s="94"/>
-      <c r="B28" s="106"/>
-      <c r="C28" s="46" t="s">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A39" s="98"/>
+      <c r="B39" s="103"/>
+      <c r="C39" s="45" t="s">
         <v>157</v>
       </c>
-      <c r="D28" s="46" t="s">
-        <v>318</v>
-      </c>
-      <c r="E28" s="59"/>
-      <c r="F28" s="46" t="s">
+      <c r="D39" s="45" t="s">
+        <v>272</v>
+      </c>
+      <c r="E39" s="58"/>
+      <c r="F39" s="45" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A29" s="94"/>
-      <c r="B29" s="106"/>
-      <c r="C29" s="46" t="s">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A40" s="98"/>
+      <c r="B40" s="103"/>
+      <c r="C40" s="45" t="s">
         <v>200</v>
       </c>
-      <c r="D29" s="46" t="s">
-        <v>319</v>
-      </c>
-      <c r="E29" s="59"/>
-      <c r="F29" s="46" t="s">
+      <c r="D40" s="45" t="s">
+        <v>273</v>
+      </c>
+      <c r="E40" s="58"/>
+      <c r="F40" s="45" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A30" s="94"/>
-      <c r="B30" s="106"/>
-      <c r="C30" s="46" t="s">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A41" s="98"/>
+      <c r="B41" s="103"/>
+      <c r="C41" s="45" t="s">
         <v>169</v>
       </c>
-      <c r="D30" s="46" t="s">
-        <v>320</v>
-      </c>
-      <c r="E30" s="58"/>
-      <c r="F30" s="46" t="s">
+      <c r="D41" s="45" t="s">
+        <v>274</v>
+      </c>
+      <c r="E41" s="57"/>
+      <c r="F41" s="45" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A31" s="94"/>
-      <c r="B31" s="106"/>
-      <c r="C31" s="46" t="s">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A42" s="98"/>
+      <c r="B42" s="103"/>
+      <c r="C42" s="45" t="s">
         <v>192</v>
       </c>
-      <c r="D31" s="46" t="s">
-        <v>321</v>
-      </c>
-      <c r="E31" s="58"/>
-      <c r="F31" s="46" t="s">
+      <c r="D42" s="45" t="s">
+        <v>275</v>
+      </c>
+      <c r="E42" s="57"/>
+      <c r="F42" s="45" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A32" s="94"/>
-      <c r="B32" s="99"/>
-      <c r="C32" s="60"/>
-      <c r="D32" s="60"/>
-      <c r="E32" s="61"/>
-      <c r="F32" s="60"/>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A33" s="94"/>
-      <c r="B33" s="100" t="s">
-        <v>233</v>
-      </c>
-      <c r="C33" s="46" t="s">
-        <v>98</v>
-      </c>
-      <c r="D33" s="46" t="s">
-        <v>268</v>
-      </c>
-      <c r="E33" s="55"/>
-      <c r="F33" s="46" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A34" s="94"/>
-      <c r="B34" s="100"/>
-      <c r="C34" s="46" t="s">
-        <v>109</v>
-      </c>
-      <c r="D34" s="46" t="s">
-        <v>269</v>
-      </c>
-      <c r="E34" s="55"/>
-      <c r="F34" s="46" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A35" s="94"/>
-      <c r="B35" s="100"/>
-      <c r="C35" s="46" t="s">
-        <v>85</v>
-      </c>
-      <c r="D35" s="46" t="s">
-        <v>270</v>
-      </c>
-      <c r="E35" s="58"/>
-      <c r="F35" s="46" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A36" s="94"/>
-      <c r="B36" s="100"/>
-      <c r="C36" s="46" t="s">
-        <v>311</v>
-      </c>
-      <c r="D36" s="46" t="s">
-        <v>329</v>
-      </c>
-      <c r="E36" s="58"/>
-      <c r="F36" s="46" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A37" s="94"/>
-      <c r="B37" s="100"/>
-      <c r="C37" s="46" t="s">
-        <v>276</v>
-      </c>
-      <c r="D37" s="46" t="s">
-        <v>328</v>
-      </c>
-      <c r="E37" s="59"/>
-      <c r="F37" s="46" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A38" s="94"/>
-      <c r="B38" s="100"/>
-      <c r="C38" s="46" t="s">
-        <v>143</v>
-      </c>
-      <c r="D38" s="46" t="s">
-        <v>271</v>
-      </c>
-      <c r="E38" s="59"/>
-      <c r="F38" s="46" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A39" s="94"/>
-      <c r="B39" s="100"/>
-      <c r="C39" s="46" t="s">
-        <v>157</v>
-      </c>
-      <c r="D39" s="46" t="s">
-        <v>272</v>
-      </c>
-      <c r="E39" s="59"/>
-      <c r="F39" s="46" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A40" s="94"/>
-      <c r="B40" s="100"/>
-      <c r="C40" s="46" t="s">
-        <v>200</v>
-      </c>
-      <c r="D40" s="46" t="s">
-        <v>273</v>
-      </c>
-      <c r="E40" s="59"/>
-      <c r="F40" s="46" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A41" s="94"/>
-      <c r="B41" s="100"/>
-      <c r="C41" s="46" t="s">
-        <v>169</v>
-      </c>
-      <c r="D41" s="46" t="s">
-        <v>274</v>
-      </c>
-      <c r="E41" s="58"/>
-      <c r="F41" s="46" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A42" s="94"/>
-      <c r="B42" s="100"/>
-      <c r="C42" s="46" t="s">
-        <v>192</v>
-      </c>
-      <c r="D42" s="46" t="s">
-        <v>275</v>
-      </c>
-      <c r="E42" s="58"/>
-      <c r="F42" s="46" t="s">
-        <v>151</v>
-      </c>
-    </row>
     <row r="43" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="94"/>
-      <c r="B43" s="100"/>
-      <c r="C43" s="46"/>
-      <c r="D43" s="46"/>
-      <c r="E43" s="58"/>
-      <c r="F43" s="46"/>
+      <c r="A43" s="98"/>
+      <c r="B43" s="103"/>
+      <c r="C43" s="45"/>
+      <c r="D43" s="45"/>
+      <c r="E43" s="57"/>
+      <c r="F43" s="45"/>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A44" s="92" t="s">
+      <c r="A44" s="97" t="s">
         <v>72</v>
       </c>
-      <c r="B44" s="101" t="s">
+      <c r="B44" s="105" t="s">
         <v>3</v>
       </c>
-      <c r="C44" s="27" t="s">
+      <c r="C44" s="26" t="s">
         <v>115</v>
       </c>
-      <c r="D44" s="27" t="s">
+      <c r="D44" s="26" t="s">
         <v>105</v>
       </c>
-      <c r="E44" s="40"/>
-      <c r="F44" s="62" t="s">
+      <c r="E44" s="39"/>
+      <c r="F44" s="61" t="s">
         <v>190</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A45" s="94"/>
-      <c r="B45" s="86"/>
+      <c r="A45" s="98"/>
+      <c r="B45" s="95"/>
       <c r="C45" s="13" t="s">
         <v>113</v>
       </c>
       <c r="D45" s="13" t="s">
         <v>112</v>
       </c>
-      <c r="E45" s="34"/>
-      <c r="F45" s="63" t="s">
+      <c r="E45" s="33"/>
+      <c r="F45" s="62" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A46" s="94"/>
-      <c r="B46" s="86"/>
+      <c r="A46" s="98"/>
+      <c r="B46" s="95"/>
       <c r="C46" s="13" t="s">
         <v>137</v>
       </c>
       <c r="D46" s="13" t="s">
         <v>135</v>
       </c>
-      <c r="E46" s="35"/>
+      <c r="E46" s="34"/>
       <c r="F46" s="13" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A47" s="94"/>
-      <c r="B47" s="86"/>
+      <c r="A47" s="98"/>
+      <c r="B47" s="95"/>
       <c r="C47" s="13" t="s">
         <v>138</v>
       </c>
       <c r="D47" s="13" t="s">
         <v>136</v>
       </c>
-      <c r="E47" s="34"/>
+      <c r="E47" s="33"/>
       <c r="F47" s="13" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A48" s="94"/>
-      <c r="B48" s="86"/>
+      <c r="A48" s="98"/>
+      <c r="B48" s="95"/>
       <c r="C48" s="13" t="s">
         <v>143</v>
       </c>
       <c r="D48" s="13" t="s">
         <v>148</v>
       </c>
-      <c r="E48" s="34"/>
+      <c r="E48" s="33"/>
       <c r="F48" s="13" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A49" s="94"/>
-      <c r="B49" s="86"/>
+      <c r="A49" s="98"/>
+      <c r="B49" s="95"/>
       <c r="C49" s="13" t="s">
         <v>157</v>
       </c>
       <c r="D49" s="13" t="s">
         <v>161</v>
       </c>
-      <c r="E49" s="34"/>
+      <c r="E49" s="33"/>
       <c r="F49" s="13" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A50" s="94"/>
-      <c r="B50" s="86"/>
+      <c r="A50" s="98"/>
+      <c r="B50" s="95"/>
       <c r="C50" s="13" t="s">
         <v>200</v>
       </c>
       <c r="D50" s="13" t="s">
         <v>203</v>
       </c>
-      <c r="E50" s="34"/>
+      <c r="E50" s="33"/>
       <c r="F50" s="13" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A51" s="94"/>
-      <c r="B51" s="86"/>
+      <c r="A51" s="98"/>
+      <c r="B51" s="95"/>
       <c r="C51" s="13" t="s">
         <v>169</v>
       </c>
       <c r="D51" s="13" t="s">
         <v>173</v>
       </c>
-      <c r="E51" s="34"/>
+      <c r="E51" s="33"/>
       <c r="F51" s="13" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A52" s="94"/>
-      <c r="B52" s="86"/>
+      <c r="A52" s="98"/>
+      <c r="B52" s="95"/>
       <c r="C52" s="13" t="s">
         <v>192</v>
       </c>
       <c r="D52" s="13" t="s">
         <v>197</v>
       </c>
-      <c r="E52" s="34"/>
+      <c r="E52" s="33"/>
       <c r="F52" s="13" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A53" s="94"/>
-      <c r="B53" s="86"/>
-      <c r="E53" s="34"/>
+      <c r="A53" s="98"/>
+      <c r="B53" s="95"/>
+      <c r="E53" s="33"/>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A54" s="94"/>
-      <c r="B54" s="96" t="s">
+      <c r="A54" s="98"/>
+      <c r="B54" s="106" t="s">
         <v>6</v>
       </c>
-      <c r="C54" s="36" t="s">
+      <c r="C54" s="35" t="s">
         <v>98</v>
       </c>
-      <c r="D54" s="36" t="s">
+      <c r="D54" s="35" t="s">
         <v>102</v>
       </c>
-      <c r="E54" s="41"/>
-      <c r="F54" s="36" t="s">
+      <c r="E54" s="40"/>
+      <c r="F54" s="35" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A55" s="94"/>
-      <c r="B55" s="86"/>
+      <c r="A55" s="98"/>
+      <c r="B55" s="95"/>
       <c r="C55" s="13" t="s">
         <v>115</v>
       </c>
       <c r="D55" s="13" t="s">
         <v>104</v>
       </c>
-      <c r="E55" s="34"/>
+      <c r="E55" s="33"/>
       <c r="F55" s="13" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A56" s="94"/>
-      <c r="B56" s="84"/>
+      <c r="A56" s="98"/>
+      <c r="B56" s="93"/>
       <c r="C56" s="13" t="s">
         <v>113</v>
       </c>
       <c r="D56" s="13" t="s">
         <v>114</v>
       </c>
-      <c r="E56" s="32"/>
+      <c r="E56" s="31"/>
       <c r="F56" s="13" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A57" s="94"/>
-      <c r="B57" s="84"/>
+      <c r="A57" s="98"/>
+      <c r="B57" s="93"/>
       <c r="C57" s="13" t="s">
         <v>109</v>
       </c>
       <c r="D57" s="13" t="s">
         <v>188</v>
       </c>
-      <c r="E57" s="32"/>
+      <c r="E57" s="31"/>
       <c r="F57" s="13" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A58" s="94"/>
-      <c r="B58" s="84"/>
+      <c r="A58" s="98"/>
+      <c r="B58" s="93"/>
       <c r="C58" s="13" t="s">
         <v>128</v>
       </c>
       <c r="D58" s="13" t="s">
         <v>126</v>
       </c>
-      <c r="E58" s="32"/>
+      <c r="E58" s="31"/>
       <c r="F58" s="13" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A59" s="94"/>
-      <c r="B59" s="84"/>
+      <c r="A59" s="98"/>
+      <c r="B59" s="93"/>
       <c r="C59" s="13" t="s">
         <v>129</v>
       </c>
       <c r="D59" s="13" t="s">
         <v>127</v>
       </c>
-      <c r="E59" s="34"/>
+      <c r="E59" s="33"/>
       <c r="F59" s="13" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A60" s="94"/>
-      <c r="B60" s="84"/>
+      <c r="A60" s="98"/>
+      <c r="B60" s="93"/>
       <c r="C60" s="13" t="s">
         <v>143</v>
       </c>
       <c r="D60" s="13" t="s">
         <v>147</v>
       </c>
-      <c r="E60" s="32"/>
+      <c r="E60" s="31"/>
       <c r="F60" s="13" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A61" s="94"/>
-      <c r="B61" s="84"/>
+      <c r="A61" s="98"/>
+      <c r="B61" s="93"/>
       <c r="C61" s="13" t="s">
         <v>157</v>
       </c>
       <c r="D61" s="13" t="s">
         <v>159</v>
       </c>
-      <c r="E61" s="34"/>
+      <c r="E61" s="33"/>
       <c r="F61" s="13" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A62" s="94"/>
-      <c r="B62" s="84"/>
+      <c r="A62" s="98"/>
+      <c r="B62" s="93"/>
       <c r="C62" s="13" t="s">
         <v>200</v>
       </c>
       <c r="D62" s="13" t="s">
         <v>204</v>
       </c>
-      <c r="E62" s="34"/>
+      <c r="E62" s="33"/>
       <c r="F62" s="13" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A63" s="94"/>
-      <c r="B63" s="84"/>
+      <c r="A63" s="98"/>
+      <c r="B63" s="93"/>
       <c r="C63" s="13" t="s">
         <v>169</v>
       </c>
       <c r="D63" s="13" t="s">
         <v>172</v>
       </c>
-      <c r="E63" s="34"/>
+      <c r="E63" s="33"/>
       <c r="F63" s="13" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A64" s="94"/>
-      <c r="B64" s="84"/>
+      <c r="A64" s="98"/>
+      <c r="B64" s="93"/>
       <c r="C64" s="13" t="s">
         <v>192</v>
       </c>
       <c r="D64" s="13" t="s">
         <v>196</v>
       </c>
-      <c r="E64" s="34"/>
+      <c r="E64" s="33"/>
       <c r="F64" s="13" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="65" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A65" s="95"/>
-      <c r="B65" s="102"/>
-      <c r="C65" s="42"/>
-      <c r="D65" s="42"/>
-      <c r="E65" s="43"/>
-      <c r="F65" s="42"/>
+      <c r="A65" s="104"/>
+      <c r="B65" s="107"/>
+      <c r="C65" s="41"/>
+      <c r="D65" s="41"/>
+      <c r="E65" s="42"/>
+      <c r="F65" s="41"/>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A66" s="92" t="s">
+      <c r="A66" s="97" t="s">
         <v>73</v>
       </c>
-      <c r="B66" s="91" t="s">
+      <c r="B66" s="99" t="s">
         <v>74</v>
       </c>
-      <c r="C66" s="27" t="s">
+      <c r="C66" s="26" t="s">
         <v>119</v>
       </c>
-      <c r="D66" s="27" t="s">
+      <c r="D66" s="26" t="s">
         <v>118</v>
       </c>
-      <c r="E66" s="40"/>
-      <c r="F66" s="27" t="s">
+      <c r="E66" s="39"/>
+      <c r="F66" s="26" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A67" s="94"/>
-      <c r="B67" s="84"/>
+      <c r="A67" s="98"/>
+      <c r="B67" s="93"/>
       <c r="C67" s="13" t="s">
         <v>155</v>
       </c>
       <c r="D67" s="13" t="s">
         <v>154</v>
       </c>
-      <c r="E67" s="32"/>
+      <c r="E67" s="31"/>
       <c r="F67" s="13" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A68" s="94"/>
-      <c r="B68" s="85"/>
-      <c r="E68" s="32"/>
+      <c r="A68" s="98"/>
+      <c r="B68" s="94"/>
+      <c r="E68" s="31"/>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A69" s="94"/>
-      <c r="B69" s="96" t="s">
+      <c r="A69" s="98"/>
+      <c r="B69" s="106" t="s">
         <v>4</v>
       </c>
-      <c r="C69" s="36" t="s">
+      <c r="C69" s="35" t="s">
         <v>98</v>
       </c>
-      <c r="D69" s="36" t="s">
+      <c r="D69" s="35" t="s">
         <v>101</v>
       </c>
-      <c r="E69" s="41"/>
-      <c r="F69" s="36" t="s">
+      <c r="E69" s="40"/>
+      <c r="F69" s="35" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A70" s="94"/>
-      <c r="B70" s="86"/>
+      <c r="A70" s="98"/>
+      <c r="B70" s="95"/>
       <c r="C70" s="13" t="s">
         <v>109</v>
       </c>
       <c r="D70" s="13" t="s">
         <v>111</v>
       </c>
-      <c r="E70" s="44"/>
+      <c r="E70" s="43"/>
       <c r="F70" s="13" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A71" s="94"/>
-      <c r="B71" s="86"/>
+      <c r="A71" s="98"/>
+      <c r="B71" s="95"/>
       <c r="C71" s="13" t="s">
         <v>124</v>
       </c>
       <c r="D71" s="13" t="s">
         <v>123</v>
       </c>
-      <c r="E71" s="44"/>
+      <c r="E71" s="43"/>
       <c r="F71" s="13" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A72" s="94"/>
-      <c r="B72" s="86"/>
+      <c r="A72" s="98"/>
+      <c r="B72" s="95"/>
       <c r="C72" s="13" t="s">
         <v>143</v>
       </c>
       <c r="D72" s="13" t="s">
         <v>146</v>
       </c>
-      <c r="E72" s="32"/>
+      <c r="E72" s="31"/>
       <c r="F72" s="13" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A73" s="94"/>
-      <c r="B73" s="86"/>
+      <c r="A73" s="98"/>
+      <c r="B73" s="95"/>
       <c r="C73" s="13" t="s">
         <v>157</v>
       </c>
       <c r="D73" s="13" t="s">
         <v>158</v>
       </c>
-      <c r="E73" s="35"/>
+      <c r="E73" s="34"/>
       <c r="F73" s="13" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A74" s="94"/>
-      <c r="B74" s="86"/>
+      <c r="A74" s="98"/>
+      <c r="B74" s="95"/>
       <c r="C74" s="13" t="s">
         <v>163</v>
       </c>
       <c r="D74" s="13" t="s">
         <v>164</v>
       </c>
-      <c r="E74" s="32"/>
+      <c r="E74" s="31"/>
       <c r="F74" s="13" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A75" s="94"/>
-      <c r="B75" s="86"/>
+      <c r="A75" s="98"/>
+      <c r="B75" s="95"/>
       <c r="C75" s="13" t="s">
         <v>200</v>
       </c>
       <c r="D75" s="13" t="s">
         <v>202</v>
       </c>
-      <c r="E75" s="32"/>
+      <c r="E75" s="31"/>
       <c r="F75" s="13" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A76" s="94"/>
-      <c r="B76" s="86"/>
+      <c r="A76" s="98"/>
+      <c r="B76" s="95"/>
       <c r="C76" s="13" t="s">
         <v>169</v>
       </c>
       <c r="D76" s="13" t="s">
         <v>171</v>
       </c>
-      <c r="E76" s="34"/>
+      <c r="E76" s="33"/>
       <c r="F76" s="13" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A77" s="94"/>
-      <c r="B77" s="86"/>
+      <c r="A77" s="98"/>
+      <c r="B77" s="95"/>
       <c r="C77" s="13" t="s">
         <v>192</v>
       </c>
       <c r="D77" s="13" t="s">
         <v>194</v>
       </c>
-      <c r="E77" s="34"/>
+      <c r="E77" s="33"/>
       <c r="F77" s="13" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A78" s="94"/>
-      <c r="B78" s="97"/>
+      <c r="A78" s="98"/>
+      <c r="B78" s="111"/>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A79" s="94"/>
-      <c r="B79" s="96" t="s">
+      <c r="A79" s="98"/>
+      <c r="B79" s="106" t="s">
         <v>5</v>
       </c>
-      <c r="C79" s="36" t="s">
+      <c r="C79" s="35" t="s">
         <v>98</v>
       </c>
-      <c r="D79" s="36" t="s">
+      <c r="D79" s="35" t="s">
         <v>103</v>
       </c>
-      <c r="E79" s="41"/>
-      <c r="F79" s="36" t="s">
+      <c r="E79" s="40"/>
+      <c r="F79" s="35" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A80" s="94"/>
-      <c r="B80" s="86"/>
+      <c r="A80" s="98"/>
+      <c r="B80" s="95"/>
       <c r="C80" s="13" t="s">
         <v>110</v>
       </c>
       <c r="D80" s="13" t="s">
         <v>108</v>
       </c>
-      <c r="E80" s="44"/>
+      <c r="E80" s="43"/>
       <c r="F80" s="13" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A81" s="94"/>
-      <c r="B81" s="86"/>
+      <c r="A81" s="98"/>
+      <c r="B81" s="95"/>
       <c r="C81" s="13" t="s">
         <v>122</v>
       </c>
       <c r="D81" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="E81" s="44"/>
+      <c r="E81" s="43"/>
       <c r="F81" s="13" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A82" s="94"/>
-      <c r="B82" s="86"/>
+      <c r="A82" s="98"/>
+      <c r="B82" s="95"/>
       <c r="C82" s="13" t="s">
         <v>143</v>
       </c>
       <c r="D82" s="13" t="s">
         <v>144</v>
       </c>
-      <c r="E82" s="44"/>
+      <c r="E82" s="43"/>
       <c r="F82" s="13" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A83" s="94"/>
-      <c r="B83" s="86"/>
+      <c r="A83" s="98"/>
+      <c r="B83" s="95"/>
       <c r="C83" s="13" t="s">
         <v>157</v>
       </c>
       <c r="D83" s="13" t="s">
         <v>156</v>
       </c>
-      <c r="E83" s="35"/>
+      <c r="E83" s="34"/>
       <c r="F83" s="13" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A84" s="94"/>
-      <c r="B84" s="86"/>
+      <c r="A84" s="98"/>
+      <c r="B84" s="95"/>
       <c r="C84" s="13" t="s">
         <v>163</v>
       </c>
       <c r="D84" s="13" t="s">
         <v>162</v>
       </c>
-      <c r="E84" s="45"/>
+      <c r="E84" s="44"/>
       <c r="F84" s="13" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A85" s="94"/>
-      <c r="B85" s="86"/>
+      <c r="A85" s="98"/>
+      <c r="B85" s="95"/>
       <c r="C85" s="13" t="s">
         <v>200</v>
       </c>
       <c r="D85" s="13" t="s">
         <v>201</v>
       </c>
-      <c r="E85" s="45"/>
+      <c r="E85" s="44"/>
       <c r="F85" s="13" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A86" s="94"/>
-      <c r="B86" s="86"/>
+      <c r="A86" s="98"/>
+      <c r="B86" s="95"/>
       <c r="C86" s="13" t="s">
         <v>169</v>
       </c>
       <c r="D86" s="13" t="s">
         <v>170</v>
       </c>
-      <c r="E86" s="34"/>
+      <c r="E86" s="33"/>
       <c r="F86" s="13" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A87" s="94"/>
-      <c r="B87" s="86"/>
+      <c r="A87" s="98"/>
+      <c r="B87" s="95"/>
       <c r="C87" s="13" t="s">
         <v>192</v>
       </c>
       <c r="D87" s="13" t="s">
         <v>193</v>
       </c>
-      <c r="E87" s="34"/>
+      <c r="E87" s="33"/>
       <c r="F87" s="13" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="88" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A88" s="95"/>
-      <c r="B88" s="98"/>
+      <c r="A88" s="104"/>
+      <c r="B88" s="112"/>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A89" s="92" t="s">
+      <c r="A89" s="97" t="s">
         <v>77</v>
       </c>
-      <c r="B89" s="91" t="s">
+      <c r="B89" s="99" t="s">
         <v>74</v>
       </c>
-      <c r="C89" s="27" t="s">
+      <c r="C89" s="26" t="s">
         <v>131</v>
       </c>
-      <c r="D89" s="27" t="s">
+      <c r="D89" s="26" t="s">
         <v>130</v>
       </c>
-      <c r="E89" s="31"/>
-      <c r="F89" s="27" t="s">
+      <c r="E89" s="30"/>
+      <c r="F89" s="26" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A90" s="93"/>
-      <c r="B90" s="87"/>
-      <c r="C90" s="53" t="s">
+      <c r="A90" s="110"/>
+      <c r="B90" s="96"/>
+      <c r="C90" s="52" t="s">
         <v>232</v>
       </c>
-      <c r="D90" s="53" t="s">
+      <c r="D90" s="52" t="s">
         <v>231</v>
       </c>
-      <c r="E90" s="54"/>
-      <c r="F90" s="53" t="s">
+      <c r="E90" s="53"/>
+      <c r="F90" s="52" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A91" s="94"/>
-      <c r="B91" s="84"/>
-      <c r="C91" s="13" t="s">
+      <c r="A91" s="98"/>
+      <c r="B91" s="96"/>
+      <c r="C91" s="52" t="s">
         <v>152</v>
       </c>
-      <c r="D91" s="13" t="s">
+      <c r="D91" s="52" t="s">
         <v>149</v>
       </c>
-      <c r="E91" s="34"/>
-      <c r="F91" s="13" t="s">
+      <c r="E91" s="53"/>
+      <c r="F91" s="52" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A92" s="94"/>
-      <c r="B92" s="85"/>
-      <c r="E92" s="34"/>
+      <c r="A92" s="98"/>
+      <c r="B92" s="94"/>
+      <c r="C92" s="37"/>
+      <c r="D92" s="37"/>
+      <c r="E92" s="38"/>
+      <c r="F92" s="37"/>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A93" s="94"/>
-      <c r="B93" s="83" t="s">
-        <v>80</v>
-      </c>
-      <c r="C93" s="36" t="s">
-        <v>133</v>
-      </c>
-      <c r="D93" s="36" t="s">
-        <v>132</v>
-      </c>
-      <c r="E93" s="41"/>
-      <c r="F93" s="36" t="s">
-        <v>134</v>
+      <c r="A93" s="98"/>
+      <c r="B93" s="92" t="s">
+        <v>332</v>
+      </c>
+      <c r="C93" s="13" t="s">
+        <v>333</v>
+      </c>
+      <c r="D93" s="13" t="s">
+        <v>334</v>
+      </c>
+      <c r="E93" s="33"/>
+      <c r="F93" s="13" t="s">
+        <v>321</v>
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A94" s="94"/>
-      <c r="B94" s="84"/>
+      <c r="A94" s="98"/>
+      <c r="B94" s="93"/>
       <c r="C94" s="13" t="s">
-        <v>153</v>
+        <v>337</v>
       </c>
       <c r="D94" s="13" t="s">
-        <v>150</v>
-      </c>
-      <c r="E94" s="34"/>
+        <v>335</v>
+      </c>
+      <c r="E94" s="33"/>
       <c r="F94" s="13" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A95" s="94"/>
-      <c r="B95" s="85"/>
-      <c r="C95" s="38"/>
-      <c r="D95" s="38"/>
-      <c r="E95" s="39"/>
-      <c r="F95" s="38"/>
+      <c r="A95" s="98"/>
+      <c r="B95" s="93"/>
+      <c r="C95" s="13" t="s">
+        <v>338</v>
+      </c>
+      <c r="D95" s="13" t="s">
+        <v>336</v>
+      </c>
+      <c r="E95" s="33"/>
+      <c r="F95" s="13" t="s">
+        <v>151</v>
+      </c>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A96" s="94"/>
-      <c r="B96" s="88" t="s">
+      <c r="A96" s="98"/>
+      <c r="B96" s="94"/>
+      <c r="E96" s="33"/>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A97" s="98"/>
+      <c r="B97" s="92" t="s">
+        <v>80</v>
+      </c>
+      <c r="C97" s="35" t="s">
+        <v>133</v>
+      </c>
+      <c r="D97" s="35" t="s">
+        <v>132</v>
+      </c>
+      <c r="E97" s="40"/>
+      <c r="F97" s="35" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A98" s="98"/>
+      <c r="B98" s="93"/>
+      <c r="C98" s="13" t="s">
+        <v>153</v>
+      </c>
+      <c r="D98" s="13" t="s">
+        <v>150</v>
+      </c>
+      <c r="E98" s="33"/>
+      <c r="F98" s="13" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A99" s="98"/>
+      <c r="B99" s="94"/>
+      <c r="C99" s="37"/>
+      <c r="D99" s="37"/>
+      <c r="E99" s="38"/>
+      <c r="F99" s="37"/>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A100" s="98"/>
+      <c r="B100" s="100" t="s">
         <v>278</v>
       </c>
-      <c r="C96" s="46" t="s">
+      <c r="C100" s="45" t="s">
         <v>277</v>
       </c>
-      <c r="D96" s="46" t="s">
+      <c r="D100" s="45" t="s">
         <v>280</v>
       </c>
-      <c r="E96" s="58"/>
-      <c r="F96" s="46" t="s">
+      <c r="E100" s="57"/>
+      <c r="F100" s="45" t="s">
         <v>266</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A97" s="94"/>
-      <c r="B97" s="89"/>
-      <c r="C97" s="46" t="s">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A101" s="98"/>
+      <c r="B101" s="101"/>
+      <c r="C101" s="45" t="s">
         <v>279</v>
       </c>
-      <c r="D97" s="46" t="s">
+      <c r="D101" s="45" t="s">
         <v>281</v>
       </c>
-      <c r="E97" s="58"/>
-      <c r="F97" s="46" t="s">
+      <c r="E101" s="57"/>
+      <c r="F101" s="45" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="98" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A98" s="95"/>
-      <c r="B98" s="90"/>
-      <c r="C98" s="64"/>
-      <c r="D98" s="64"/>
-      <c r="E98" s="65"/>
-      <c r="F98" s="64"/>
-    </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A99" s="92" t="s">
+    <row r="102" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A102" s="104"/>
+      <c r="B102" s="109"/>
+      <c r="C102" s="63"/>
+      <c r="D102" s="63"/>
+      <c r="E102" s="64"/>
+      <c r="F102" s="63"/>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A103" s="97" t="s">
         <v>165</v>
       </c>
-      <c r="B99" s="91" t="s">
+      <c r="B103" s="99" t="s">
         <v>13</v>
       </c>
-      <c r="C99" s="27" t="s">
+      <c r="C103" s="26" t="s">
         <v>175</v>
       </c>
-      <c r="D99" s="27" t="s">
+      <c r="D103" s="26" t="s">
         <v>174</v>
       </c>
-      <c r="E99" s="27"/>
-      <c r="F99" s="27" t="s">
+      <c r="E103" s="26"/>
+      <c r="F103" s="26" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A100" s="93"/>
-      <c r="B100" s="84"/>
-      <c r="C100" s="13" t="s">
+    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A104" s="110"/>
+      <c r="B104" s="93"/>
+      <c r="C104" s="13" t="s">
         <v>176</v>
       </c>
-      <c r="D100" s="13" t="s">
+      <c r="D104" s="13" t="s">
         <v>177</v>
       </c>
-      <c r="F100" s="13" t="s">
+      <c r="F104" s="13" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A101" s="93"/>
-      <c r="B101" s="85"/>
-      <c r="C101" s="38"/>
-      <c r="D101" s="38"/>
-      <c r="E101" s="38"/>
-      <c r="F101" s="38"/>
-    </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A102" s="93"/>
-      <c r="B102" s="83" t="s">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A105" s="110"/>
+      <c r="B105" s="94"/>
+      <c r="C105" s="37"/>
+      <c r="D105" s="37"/>
+      <c r="E105" s="37"/>
+      <c r="F105" s="37"/>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A106" s="110"/>
+      <c r="B106" s="92" t="s">
         <v>186</v>
       </c>
-      <c r="C102" s="13" t="s">
+      <c r="C106" s="13" t="s">
         <v>167</v>
       </c>
-      <c r="D102" s="13" t="s">
+      <c r="D106" s="13" t="s">
         <v>166</v>
-      </c>
-      <c r="F102" s="13" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A103" s="93"/>
-      <c r="B103" s="84"/>
-      <c r="C103" s="13" t="s">
-        <v>184</v>
-      </c>
-      <c r="D103" s="13" t="s">
-        <v>178</v>
-      </c>
-      <c r="F103" s="13" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A104" s="93"/>
-      <c r="B104" s="84"/>
-      <c r="C104" s="13" t="s">
-        <v>180</v>
-      </c>
-      <c r="D104" s="13" t="s">
-        <v>179</v>
-      </c>
-      <c r="F104" s="13" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A105" s="93"/>
-      <c r="B105" s="84"/>
-      <c r="C105" s="13" t="s">
-        <v>182</v>
-      </c>
-      <c r="D105" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="F105" s="13" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A106" s="93"/>
-      <c r="B106" s="84"/>
-      <c r="C106" s="13" t="s">
-        <v>185</v>
-      </c>
-      <c r="D106" s="13" t="s">
-        <v>183</v>
       </c>
       <c r="F106" s="13" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A107" s="93"/>
-      <c r="B107" s="84"/>
+      <c r="A107" s="110"/>
+      <c r="B107" s="93"/>
       <c r="C107" s="13" t="s">
-        <v>195</v>
+        <v>184</v>
       </c>
       <c r="D107" s="13" t="s">
-        <v>191</v>
+        <v>178</v>
       </c>
       <c r="F107" s="13" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A108" s="93"/>
-      <c r="B108" s="83" t="s">
+      <c r="A108" s="110"/>
+      <c r="B108" s="93"/>
+      <c r="D108" s="13" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A109" s="110"/>
+      <c r="B109" s="93"/>
+      <c r="C109" s="13" t="s">
+        <v>180</v>
+      </c>
+      <c r="D109" s="13" t="s">
+        <v>179</v>
+      </c>
+      <c r="F109" s="13" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A110" s="110"/>
+      <c r="B110" s="93"/>
+      <c r="C110" s="13" t="s">
+        <v>182</v>
+      </c>
+      <c r="D110" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="F110" s="13" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A111" s="110"/>
+      <c r="B111" s="93"/>
+      <c r="C111" s="13" t="s">
+        <v>185</v>
+      </c>
+      <c r="D111" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="F111" s="13" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A112" s="110"/>
+      <c r="B112" s="93"/>
+      <c r="C112" s="13" t="s">
+        <v>195</v>
+      </c>
+      <c r="D112" s="13" t="s">
+        <v>191</v>
+      </c>
+      <c r="F112" s="13" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A113" s="110"/>
+      <c r="B113" s="92" t="s">
         <v>210</v>
       </c>
-      <c r="C108" s="36" t="s">
+      <c r="C113" s="35" t="s">
         <v>207</v>
       </c>
-      <c r="D108" s="36" t="s">
+      <c r="D113" s="35" t="s">
         <v>211</v>
       </c>
-      <c r="E108" s="36"/>
-      <c r="F108" s="36" t="s">
+      <c r="E113" s="35"/>
+      <c r="F113" s="35" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A109" s="93"/>
-      <c r="B109" s="87"/>
-      <c r="C109" s="53" t="s">
+    <row r="114" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A114" s="110"/>
+      <c r="B114" s="96"/>
+      <c r="C114" s="52" t="s">
         <v>208</v>
       </c>
-      <c r="D109" s="53" t="s">
+      <c r="D114" s="52" t="s">
         <v>214</v>
       </c>
-      <c r="E109" s="53"/>
-      <c r="F109" s="53" t="s">
+      <c r="E114" s="52"/>
+      <c r="F114" s="52" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A110" s="93"/>
-      <c r="B110" s="87"/>
-      <c r="C110" s="53" t="s">
+    <row r="115" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A115" s="110"/>
+      <c r="B115" s="96"/>
+      <c r="C115" s="52" t="s">
         <v>219</v>
       </c>
-      <c r="D110" s="53" t="s">
+      <c r="D115" s="52" t="s">
         <v>218</v>
       </c>
-      <c r="E110" s="53"/>
-      <c r="F110" s="53" t="s">
+      <c r="E115" s="52"/>
+      <c r="F115" s="52" t="s">
         <v>223</v>
       </c>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A111" s="93"/>
-      <c r="B111" s="87"/>
-      <c r="C111" s="53" t="s">
+    <row r="116" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A116" s="110"/>
+      <c r="B116" s="96"/>
+      <c r="C116" s="52" t="s">
         <v>209</v>
       </c>
-      <c r="D111" s="53" t="s">
+      <c r="D116" s="52" t="s">
         <v>213</v>
       </c>
-      <c r="E111" s="53"/>
-      <c r="F111" s="53" t="s">
+      <c r="E116" s="52"/>
+      <c r="F116" s="52" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A112" s="93"/>
-      <c r="B112" s="87"/>
-      <c r="C112" s="53" t="s">
+    <row r="117" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A117" s="110"/>
+      <c r="B117" s="96"/>
+      <c r="C117" s="52" t="s">
+        <v>341</v>
+      </c>
+      <c r="D117" s="52" t="s">
+        <v>342</v>
+      </c>
+      <c r="E117" s="52"/>
+      <c r="F117" s="52" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A118" s="110"/>
+      <c r="B118" s="96"/>
+      <c r="C118" s="52" t="s">
         <v>221</v>
       </c>
-      <c r="D112" s="53" t="s">
+      <c r="D118" s="52" t="s">
         <v>220</v>
       </c>
-      <c r="E112" s="53"/>
-      <c r="F112" s="53" t="s">
+      <c r="E118" s="52"/>
+      <c r="F118" s="52" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A113" s="93"/>
-      <c r="B113" s="87"/>
-      <c r="C113" s="53" t="s">
+    <row r="119" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A119" s="110"/>
+      <c r="B119" s="96"/>
+      <c r="C119" s="52" t="s">
         <v>225</v>
       </c>
-      <c r="D113" s="53" t="s">
+      <c r="D119" s="52" t="s">
         <v>215</v>
       </c>
-      <c r="E113" s="53"/>
-      <c r="F113" s="53" t="s">
+      <c r="E119" s="52"/>
+      <c r="F119" s="52" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A114" s="93"/>
-      <c r="B114" s="87"/>
-      <c r="C114" s="53" t="s">
+    <row r="120" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A120" s="110"/>
+      <c r="B120" s="96"/>
+      <c r="C120" s="52" t="s">
         <v>206</v>
       </c>
-      <c r="D114" s="13" t="s">
+      <c r="D120" s="13" t="s">
         <v>224</v>
       </c>
-      <c r="E114" s="53"/>
-      <c r="F114" s="53" t="s">
+      <c r="E120" s="52"/>
+      <c r="F120" s="52" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A115" s="93"/>
-      <c r="B115" s="87"/>
-      <c r="C115" s="66" t="s">
+    <row r="121" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A121" s="110"/>
+      <c r="B121" s="96"/>
+      <c r="C121" s="65" t="s">
         <v>282</v>
       </c>
-      <c r="D115" s="66" t="s">
+      <c r="D121" s="65" t="s">
         <v>283</v>
       </c>
-      <c r="E115" s="66"/>
-      <c r="F115" s="46" t="s">
+      <c r="E121" s="65"/>
+      <c r="F121" s="45" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A116" s="93"/>
-      <c r="B116" s="87"/>
-      <c r="C116" s="66" t="s">
+    <row r="122" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A122" s="110"/>
+      <c r="B122" s="96"/>
+      <c r="C122" s="65" t="s">
         <v>285</v>
       </c>
-      <c r="D116" s="66" t="s">
+      <c r="D122" s="65" t="s">
         <v>284</v>
       </c>
-      <c r="E116" s="66"/>
-      <c r="F116" s="66" t="s">
+      <c r="E122" s="65"/>
+      <c r="F122" s="65" t="s">
         <v>217</v>
       </c>
     </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A117" s="93"/>
-      <c r="B117" s="83" t="s">
+    <row r="123" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A123" s="110"/>
+      <c r="B123" s="92" t="s">
         <v>226</v>
       </c>
-      <c r="C117" s="36" t="s">
+      <c r="C123" s="35" t="s">
         <v>228</v>
       </c>
-      <c r="D117" s="36" t="s">
+      <c r="D123" s="35" t="s">
         <v>227</v>
       </c>
-      <c r="E117" s="36"/>
-      <c r="F117" s="36" t="s">
+      <c r="E123" s="35"/>
+      <c r="F123" s="35" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A118" s="93"/>
-      <c r="B118" s="87"/>
-      <c r="C118" s="53" t="s">
+    <row r="124" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A124" s="110"/>
+      <c r="B124" s="96"/>
+      <c r="C124" s="52" t="s">
+        <v>343</v>
+      </c>
+      <c r="D124" s="52" t="s">
+        <v>344</v>
+      </c>
+      <c r="E124" s="52"/>
+      <c r="F124" s="52" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A125" s="110"/>
+      <c r="B125" s="96"/>
+      <c r="C125" s="52" t="s">
         <v>229</v>
       </c>
-      <c r="D118" s="53" t="s">
+      <c r="D125" s="52" t="s">
         <v>230</v>
       </c>
-      <c r="E118" s="53"/>
-      <c r="F118" s="53" t="s">
+      <c r="E125" s="52"/>
+      <c r="F125" s="52" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A119" s="93"/>
-      <c r="B119" s="87"/>
-      <c r="C119" s="66" t="s">
+    <row r="126" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A126" s="110"/>
+      <c r="B126" s="96"/>
+      <c r="C126" s="65" t="s">
         <v>286</v>
       </c>
-      <c r="D119" s="66" t="s">
+      <c r="D126" s="65" t="s">
         <v>287</v>
       </c>
-      <c r="E119" s="66"/>
-      <c r="F119" s="66" t="s">
+      <c r="E126" s="65"/>
+      <c r="F126" s="65" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A120" s="93"/>
-      <c r="B120" s="87"/>
-      <c r="C120" s="46" t="s">
+    <row r="127" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A127" s="110"/>
+      <c r="B127" s="96"/>
+      <c r="C127" s="45" t="s">
         <v>288</v>
       </c>
-      <c r="D120" s="46" t="s">
-        <v>289</v>
-      </c>
-      <c r="E120" s="46"/>
-      <c r="F120" s="46" t="s">
+      <c r="D127" s="45" t="s">
+        <v>339</v>
+      </c>
+      <c r="E127" s="45"/>
+      <c r="F127" s="45" t="s">
         <v>217</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="21">
+  <mergeCells count="22">
+    <mergeCell ref="B100:B102"/>
+    <mergeCell ref="B66:B68"/>
+    <mergeCell ref="B106:B112"/>
+    <mergeCell ref="B123:B127"/>
+    <mergeCell ref="A103:A127"/>
+    <mergeCell ref="B113:B122"/>
+    <mergeCell ref="B103:B105"/>
+    <mergeCell ref="A66:A88"/>
+    <mergeCell ref="B69:B78"/>
+    <mergeCell ref="B79:B88"/>
+    <mergeCell ref="A89:A102"/>
+    <mergeCell ref="B97:B99"/>
+    <mergeCell ref="B89:B92"/>
+    <mergeCell ref="B93:B96"/>
     <mergeCell ref="A2:A43"/>
     <mergeCell ref="B2:B11"/>
     <mergeCell ref="B12:B22"/>
@@ -4781,19 +4964,6 @@
     <mergeCell ref="B44:B53"/>
     <mergeCell ref="B54:B65"/>
     <mergeCell ref="B23:B32"/>
-    <mergeCell ref="B96:B98"/>
-    <mergeCell ref="B66:B68"/>
-    <mergeCell ref="B102:B107"/>
-    <mergeCell ref="B117:B120"/>
-    <mergeCell ref="A99:A120"/>
-    <mergeCell ref="B108:B116"/>
-    <mergeCell ref="B99:B101"/>
-    <mergeCell ref="A66:A88"/>
-    <mergeCell ref="B69:B78"/>
-    <mergeCell ref="B79:B88"/>
-    <mergeCell ref="A89:A98"/>
-    <mergeCell ref="B89:B92"/>
-    <mergeCell ref="B93:B95"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -4805,56 +4975,56 @@
   <dimension ref="B1:B31"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="11.5546875" style="67"/>
+    <col min="2" max="2" width="11.5546875" style="66"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B1" s="67" t="s">
+      <c r="B1" s="66" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="2" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B2" s="66" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="22" spans="2:2" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B22" s="69" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="24" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B24" s="66" t="s">
         <v>296</v>
       </c>
     </row>
-    <row r="2" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B2" s="67" t="s">
+    <row r="26" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B26" s="66" t="s">
         <v>290</v>
       </c>
     </row>
-    <row r="22" spans="2:2" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B22" s="70" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="24" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B24" s="67" t="s">
-        <v>297</v>
-      </c>
-    </row>
-    <row r="26" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B26" s="67" t="s">
+    <row r="27" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B27" s="66" t="s">
         <v>291</v>
       </c>
     </row>
-    <row r="27" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B27" s="67" t="s">
+    <row r="28" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B28" s="66" t="s">
         <v>292</v>
       </c>
     </row>
-    <row r="28" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B28" s="67" t="s">
+    <row r="29" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B29" s="67" t="s">
         <v>293</v>
       </c>
     </row>
-    <row r="29" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B29" s="68" t="s">
+    <row r="30" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B30" s="68" t="s">
         <v>294</v>
       </c>
     </row>
-    <row r="30" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B30" s="69" t="s">
-        <v>295</v>
-      </c>
-    </row>
     <row r="31" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B31" s="69"/>
+      <c r="B31" s="68"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
Methanol Modell Wärmespeicher eingefügt
</commit_message>
<xml_diff>
--- a/Methanol_DAC_Greenfield_Patagonien/Datenbank.xlsx
+++ b/Methanol_DAC_Greenfield_Patagonien/Datenbank.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\01-Arbeit\06-FENES\09-P2X3\FENES_P2X\Methanol_DAC_Greenfield_Patagonien\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{908D3A3D-CD06-467F-9C9A-476F00F703A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E2B28F8-FA68-4D84-8EE6-413B37AF6629}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="23520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Datenauswahl" sheetId="1" r:id="rId1"/>
@@ -46,6 +46,7 @@
     <author>tc={5F7F21A6-9267-43AB-9E2F-857C43A6B051}</author>
     <author>tc={87F94307-F9C1-413A-A184-19A69689A8AF}</author>
     <author>tc={011C4874-472E-423F-9F9E-1A44747EBF50}</author>
+    <author>tc={F7866A31-18E0-48C6-B567-67C836D4C8B7}</author>
     <author>Timon Geiß</author>
     <author>tc={24965C23-66A2-443D-B1F3-FDFF8EFF87E6}</author>
   </authors>
@@ -98,7 +99,19 @@
     ~ 40 opex/ 800 capex</t>
       </text>
     </comment>
-    <comment ref="E42" authorId="6" shapeId="0" xr:uid="{22946658-3822-4C9A-8007-CC034FA9B8AB}">
+    <comment ref="E39" authorId="6" shapeId="0" xr:uid="{F7866A31-18E0-48C6-B567-67C836D4C8B7}">
+      <text>
+        <t>[Kommentarthread]
+Ihre Version von Excel gestattet Ihnen das Lesen dieses Kommentarthreads. Jegliche Bearbeitungen daran werden jedoch entfernt, wenn die Datei in einer neueren Version von Excel geöffnet wird. Weitere Informationen: https://go.microsoft.com/fwlink/?linkid=870924.
+Kommentar:
+    Wochenfaktor 4,33 * 24h *7d = 727,44h/monat
+4,55 %/monat * 1/727,44 monat/h
+Antwort:
+    Wochenfaktor 4,33 * 24h * 7d= 727,44 h/monat
+4,55 %/monat * 1/727 monat/h</t>
+      </text>
+    </comment>
+    <comment ref="E50" authorId="7" shapeId="0" xr:uid="{22946658-3822-4C9A-8007-CC034FA9B8AB}">
       <text>
         <r>
           <rPr>
@@ -122,7 +135,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E43" authorId="6" shapeId="0" xr:uid="{426A9046-86EB-4AF9-8A2D-1FEFC7B6C4A3}">
+    <comment ref="E51" authorId="7" shapeId="0" xr:uid="{426A9046-86EB-4AF9-8A2D-1FEFC7B6C4A3}">
       <text>
         <r>
           <rPr>
@@ -146,7 +159,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E44" authorId="6" shapeId="0" xr:uid="{360FC6EE-8AD3-4EF7-B2BF-00DD1029DCAF}">
+    <comment ref="E52" authorId="7" shapeId="0" xr:uid="{360FC6EE-8AD3-4EF7-B2BF-00DD1029DCAF}">
       <text>
         <r>
           <rPr>
@@ -170,7 +183,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E65" authorId="7" shapeId="0" xr:uid="{24965C23-66A2-443D-B1F3-FDFF8EFF87E6}">
+    <comment ref="E73" authorId="8" shapeId="0" xr:uid="{24965C23-66A2-443D-B1F3-FDFF8EFF87E6}">
       <text>
         <t>[Kommentarthread]
 Ihre Version von Excel gestattet Ihnen das Lesen dieses Kommentarthreads. Jegliche Bearbeitungen daran werden jedoch entfernt, wenn die Datei in einer neueren Version von Excel geöffnet wird. Weitere Informationen: https://go.microsoft.com/fwlink/?linkid=870924.
@@ -183,7 +196,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="586" uniqueCount="346">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="644" uniqueCount="370">
   <si>
     <t>PEM Elektrolyse</t>
   </si>
@@ -721,9 +734,6 @@
     <t>calc_gesamtinvest</t>
   </si>
   <si>
-    <t>calc_verzinstinvest_annuity_gesamt</t>
-  </si>
-  <si>
     <t>calc_einnahmen_gesamt</t>
   </si>
   <si>
@@ -1223,6 +1233,81 @@
   </si>
   <si>
     <t>ct/kWh_th</t>
+  </si>
+  <si>
+    <t>Wärmespeicher</t>
+  </si>
+  <si>
+    <t>capex_qs</t>
+  </si>
+  <si>
+    <t>opex_qs</t>
+  </si>
+  <si>
+    <t>lebensdauer_qs</t>
+  </si>
+  <si>
+    <t>verlustrate_qs</t>
+  </si>
+  <si>
+    <t>eta_einspeichern_qs</t>
+  </si>
+  <si>
+    <t>eta_ausspeichern_qs</t>
+  </si>
+  <si>
+    <t>zinssatz_qs</t>
+  </si>
+  <si>
+    <t>fuellstand_qs</t>
+  </si>
+  <si>
+    <t>€/kWh_th</t>
+  </si>
+  <si>
+    <t>annuity_qs</t>
+  </si>
+  <si>
+    <t>result_qs_kapa</t>
+  </si>
+  <si>
+    <t>result_qs_flowsum_in</t>
+  </si>
+  <si>
+    <t>result_qs_flowsum_out</t>
+  </si>
+  <si>
+    <t>calc_gesamtinvest_qs</t>
+  </si>
+  <si>
+    <t>calc_opex_fix_qs</t>
+  </si>
+  <si>
+    <t>calc_annuity_qs</t>
+  </si>
+  <si>
+    <t>calc_verzinstinvest_qs</t>
+  </si>
+  <si>
+    <t>calc_cost_qs</t>
+  </si>
+  <si>
+    <t>Levelized Cost of Heatstorage</t>
+  </si>
+  <si>
+    <t>calc_lcoh_qs</t>
+  </si>
+  <si>
+    <t>Levelized Cost of Heat</t>
+  </si>
+  <si>
+    <t>calc_lcoh_q</t>
+  </si>
+  <si>
+    <t>€/ kWh_th a</t>
+  </si>
+  <si>
+    <t>kWh_th</t>
   </si>
 </sst>
 </file>
@@ -1428,7 +1513,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="113">
+  <cellXfs count="123">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -1482,7 +1567,6 @@
     <xf numFmtId="4" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -1497,7 +1581,6 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1518,6 +1601,15 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1533,13 +1625,16 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1572,20 +1667,38 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -1594,30 +1707,18 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2085,7 +2186,15 @@
   <threadedComment ref="E25" dT="2025-03-14T09:25:24.78" personId="{7B1A26D8-2D09-4CF3-BDB9-5A9185883024}" id="{011C4874-472E-423F-9F9E-1A44747EBF50}">
     <text>~ 40 opex/ 800 capex</text>
   </threadedComment>
-  <threadedComment ref="E65" dT="2025-03-18T07:43:27.70" personId="{7B1A26D8-2D09-4CF3-BDB9-5A9185883024}" id="{24965C23-66A2-443D-B1F3-FDFF8EFF87E6}">
+  <threadedComment ref="E39" dT="2025-03-26T10:22:08.04" personId="{7B1A26D8-2D09-4CF3-BDB9-5A9185883024}" id="{F7866A31-18E0-48C6-B567-67C836D4C8B7}">
+    <text>Wochenfaktor 4,33 * 24h *7d = 727,44h/monat
+4,55 %/monat * 1/727,44 monat/h</text>
+  </threadedComment>
+  <threadedComment ref="E39" dT="2025-03-26T10:28:05.27" personId="{7B1A26D8-2D09-4CF3-BDB9-5A9185883024}" id="{02E78AB9-E14B-4034-A3AB-3EF5F06F95CB}" parentId="{F7866A31-18E0-48C6-B567-67C836D4C8B7}">
+    <text>Wochenfaktor 4,33 * 24h * 7d= 727,44 h/monat
+4,55 %/monat * 1/727 monat/h</text>
+  </threadedComment>
+  <threadedComment ref="E73" dT="2025-03-18T07:43:27.70" personId="{7B1A26D8-2D09-4CF3-BDB9-5A9185883024}" id="{24965C23-66A2-443D-B1F3-FDFF8EFF87E6}">
     <text>https://de.statista.com/statistik/daten/studie/730823/umfrage/durchschnittlicher-preis-fuer-methanol-auf-dem-europaeischen-markt/</text>
     <extLst>
       <x:ext xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" uri="{F7C98A9C-CBB3-438F-8F68-D28B6AF4A901}">
@@ -2099,7 +2208,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G65"/>
+  <dimension ref="A1:G73"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.88671875" customWidth="1"/>
@@ -2137,10 +2246,10 @@
       <c r="G1" s="6"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="79" t="s">
+      <c r="A2" s="86" t="s">
         <v>71</v>
       </c>
-      <c r="B2" s="90" t="s">
+      <c r="B2" s="98" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="2" t="s">
@@ -2157,8 +2266,8 @@
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="80"/>
-      <c r="B3" s="91"/>
+      <c r="A3" s="87"/>
+      <c r="B3" s="99"/>
       <c r="C3" t="s">
         <v>85</v>
       </c>
@@ -2169,12 +2278,12 @@
         <v>50</v>
       </c>
       <c r="F3" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="80"/>
-      <c r="B4" s="91"/>
+      <c r="A4" s="87"/>
+      <c r="B4" s="99"/>
       <c r="C4" t="s">
         <v>10</v>
       </c>
@@ -2189,8 +2298,8 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="80"/>
-      <c r="B5" s="91"/>
+      <c r="A5" s="87"/>
+      <c r="B5" s="99"/>
       <c r="C5" t="s">
         <v>11</v>
       </c>
@@ -2205,8 +2314,8 @@
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="80"/>
-      <c r="B6" s="91"/>
+      <c r="A6" s="87"/>
+      <c r="B6" s="99"/>
       <c r="C6" t="s">
         <v>13</v>
       </c>
@@ -2221,8 +2330,8 @@
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="80"/>
-      <c r="B7" s="91"/>
+      <c r="A7" s="87"/>
+      <c r="B7" s="99"/>
       <c r="C7" t="s">
         <v>15</v>
       </c>
@@ -2237,33 +2346,33 @@
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="80"/>
-      <c r="B8" s="92" t="s">
-        <v>234</v>
+      <c r="A8" s="87"/>
+      <c r="B8" s="100" t="s">
+        <v>233</v>
       </c>
       <c r="C8" s="35" t="s">
         <v>85</v>
       </c>
       <c r="D8" s="35" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E8" s="36">
         <v>1.5</v>
       </c>
       <c r="F8" s="35" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="80"/>
-      <c r="B9" s="93"/>
+      <c r="A9" s="87"/>
+      <c r="B9" s="101"/>
       <c r="C9" s="45" t="s">
         <v>86</v>
       </c>
       <c r="D9" s="45" t="s">
-        <v>237</v>
-      </c>
-      <c r="E9" s="54">
+        <v>236</v>
+      </c>
+      <c r="E9" s="53">
         <v>285.39999999999998</v>
       </c>
       <c r="F9" s="45" t="s">
@@ -2271,29 +2380,29 @@
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" s="80"/>
-      <c r="B10" s="93"/>
+      <c r="A10" s="87"/>
+      <c r="B10" s="101"/>
       <c r="C10" s="13" t="s">
         <v>10</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E10" s="31">
         <v>5000</v>
       </c>
       <c r="F10" s="31" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="80"/>
-      <c r="B11" s="93"/>
+      <c r="A11" s="87"/>
+      <c r="B11" s="101"/>
       <c r="C11" s="13" t="s">
         <v>11</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E11" s="33">
         <v>0.05</v>
@@ -2303,45 +2412,45 @@
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" s="80"/>
-      <c r="B12" s="93"/>
+      <c r="A12" s="87"/>
+      <c r="B12" s="101"/>
       <c r="C12" s="13" t="s">
         <v>87</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="E12" s="31">
         <v>0.189</v>
       </c>
       <c r="F12" s="13" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A13" s="87"/>
+      <c r="B13" s="101"/>
+      <c r="C13" s="45" t="s">
+        <v>253</v>
+      </c>
+      <c r="D13" s="45" t="s">
         <v>244</v>
       </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" s="80"/>
-      <c r="B13" s="93"/>
-      <c r="C13" s="45" t="s">
-        <v>254</v>
-      </c>
-      <c r="D13" s="45" t="s">
+      <c r="E13" s="53">
+        <v>1.375</v>
+      </c>
+      <c r="F13" s="45" t="s">
         <v>245</v>
       </c>
-      <c r="E13" s="54">
-        <v>1.375</v>
-      </c>
-      <c r="F13" s="45" t="s">
-        <v>246</v>
-      </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" s="80"/>
-      <c r="B14" s="93"/>
+      <c r="A14" s="87"/>
+      <c r="B14" s="101"/>
       <c r="C14" s="13" t="s">
         <v>13</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E14" s="34">
         <v>25</v>
@@ -2351,13 +2460,13 @@
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A15" s="80"/>
-      <c r="B15" s="94"/>
+      <c r="A15" s="87"/>
+      <c r="B15" s="102"/>
       <c r="C15" s="37" t="s">
         <v>15</v>
       </c>
       <c r="D15" s="37" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="E15" s="38">
         <v>0.08</v>
@@ -2367,17 +2476,17 @@
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A16" s="80"/>
-      <c r="B16" s="92" t="s">
-        <v>299</v>
+      <c r="A16" s="87"/>
+      <c r="B16" s="100" t="s">
+        <v>298</v>
       </c>
       <c r="C16" s="35" t="s">
         <v>8</v>
       </c>
       <c r="D16" s="35" t="s">
-        <v>302</v>
-      </c>
-      <c r="E16" s="70">
+        <v>301</v>
+      </c>
+      <c r="E16" s="68">
         <v>3.7</v>
       </c>
       <c r="F16" s="35" t="s">
@@ -2385,79 +2494,79 @@
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" s="80"/>
-      <c r="B17" s="96"/>
-      <c r="C17" s="52" t="s">
+      <c r="A17" s="87"/>
+      <c r="B17" s="104"/>
+      <c r="C17" s="51" t="s">
         <v>85</v>
       </c>
-      <c r="D17" s="52" t="s">
+      <c r="D17" s="51" t="s">
+        <v>302</v>
+      </c>
+      <c r="E17" s="69">
+        <v>0.27</v>
+      </c>
+      <c r="F17" s="76" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" s="87"/>
+      <c r="B18" s="104"/>
+      <c r="C18" s="51" t="s">
+        <v>10</v>
+      </c>
+      <c r="D18" s="51" t="s">
         <v>303</v>
       </c>
-      <c r="E17" s="71">
-        <v>0.27</v>
-      </c>
-      <c r="F17" s="78" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" s="80"/>
-      <c r="B18" s="96"/>
-      <c r="C18" s="52" t="s">
-        <v>10</v>
-      </c>
-      <c r="D18" s="52" t="s">
+      <c r="E18" s="69">
+        <v>700</v>
+      </c>
+      <c r="F18" s="51" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" s="87"/>
+      <c r="B19" s="104"/>
+      <c r="C19" s="51" t="s">
+        <v>11</v>
+      </c>
+      <c r="D19" s="51" t="s">
         <v>304</v>
       </c>
-      <c r="E18" s="71">
-        <v>700</v>
-      </c>
-      <c r="F18" s="52" t="s">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" s="80"/>
-      <c r="B19" s="96"/>
-      <c r="C19" s="52" t="s">
-        <v>11</v>
-      </c>
-      <c r="D19" s="52" t="s">
+      <c r="E19" s="69">
+        <v>0.02</v>
+      </c>
+      <c r="F19" s="51" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20" s="87"/>
+      <c r="B20" s="104"/>
+      <c r="C20" s="51" t="s">
+        <v>13</v>
+      </c>
+      <c r="D20" s="51" t="s">
         <v>305</v>
       </c>
-      <c r="E19" s="71">
-        <v>0.02</v>
-      </c>
-      <c r="F19" s="52" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" s="80"/>
-      <c r="B20" s="96"/>
-      <c r="C20" s="52" t="s">
-        <v>13</v>
-      </c>
-      <c r="D20" s="52" t="s">
-        <v>306</v>
-      </c>
-      <c r="E20" s="71">
+      <c r="E20" s="69">
         <v>20</v>
       </c>
-      <c r="F20" s="52" t="s">
+      <c r="F20" s="51" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A21" s="80"/>
-      <c r="B21" s="94"/>
+      <c r="A21" s="87"/>
+      <c r="B21" s="102"/>
       <c r="C21" s="37" t="s">
         <v>15</v>
       </c>
       <c r="D21" s="37" t="s">
-        <v>307</v>
-      </c>
-      <c r="E21" s="72">
+        <v>306</v>
+      </c>
+      <c r="E21" s="70">
         <v>0.05</v>
       </c>
       <c r="F21" s="37" t="s">
@@ -2465,65 +2574,65 @@
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A22" s="80"/>
-      <c r="B22" s="95" t="s">
-        <v>233</v>
+      <c r="A22" s="87"/>
+      <c r="B22" s="103" t="s">
+        <v>232</v>
       </c>
       <c r="C22" s="45" t="s">
         <v>85</v>
       </c>
       <c r="D22" s="45" t="s">
-        <v>247</v>
-      </c>
-      <c r="E22" s="54">
+        <v>246</v>
+      </c>
+      <c r="E22" s="53">
         <v>0.5</v>
       </c>
       <c r="F22" s="45" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" s="80"/>
-      <c r="B23" s="95"/>
+      <c r="A23" s="87"/>
+      <c r="B23" s="103"/>
       <c r="C23" s="45" t="s">
+        <v>308</v>
+      </c>
+      <c r="D23" s="45" t="s">
         <v>309</v>
       </c>
-      <c r="D23" s="45" t="s">
+      <c r="E23" s="53">
+        <v>1.75</v>
+      </c>
+      <c r="F23" s="45" t="s">
         <v>310</v>
       </c>
-      <c r="E23" s="54">
-        <v>1.75</v>
-      </c>
-      <c r="F23" s="45" t="s">
-        <v>311</v>
-      </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" s="80"/>
-      <c r="B24" s="95"/>
+      <c r="A24" s="87"/>
+      <c r="B24" s="103"/>
       <c r="C24" s="45" t="s">
         <v>10</v>
       </c>
       <c r="D24" s="45" t="s">
-        <v>248</v>
-      </c>
-      <c r="E24" s="54">
+        <v>247</v>
+      </c>
+      <c r="E24" s="53">
         <v>7000</v>
       </c>
       <c r="F24" s="45" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25" s="80"/>
-      <c r="B25" s="95"/>
+      <c r="A25" s="87"/>
+      <c r="B25" s="103"/>
       <c r="C25" s="45" t="s">
         <v>11</v>
       </c>
       <c r="D25" s="45" t="s">
-        <v>249</v>
-      </c>
-      <c r="E25" s="57">
+        <v>248</v>
+      </c>
+      <c r="E25" s="56">
         <v>0.05</v>
       </c>
       <c r="F25" s="45" t="s">
@@ -2531,15 +2640,15 @@
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26" s="80"/>
-      <c r="B26" s="95"/>
+      <c r="A26" s="87"/>
+      <c r="B26" s="103"/>
       <c r="C26" s="45" t="s">
         <v>13</v>
       </c>
       <c r="D26" s="45" t="s">
-        <v>250</v>
-      </c>
-      <c r="E26" s="58">
+        <v>249</v>
+      </c>
+      <c r="E26" s="57">
         <v>15</v>
       </c>
       <c r="F26" s="45" t="s">
@@ -2547,15 +2656,15 @@
       </c>
     </row>
     <row r="27" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="80"/>
-      <c r="B27" s="95"/>
+      <c r="A27" s="87"/>
+      <c r="B27" s="103"/>
       <c r="C27" s="45" t="s">
         <v>15</v>
       </c>
       <c r="D27" s="45" t="s">
-        <v>251</v>
-      </c>
-      <c r="E27" s="57">
+        <v>250</v>
+      </c>
+      <c r="E27" s="56">
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="F27" s="45" t="s">
@@ -2563,10 +2672,10 @@
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A28" s="79" t="s">
+      <c r="A28" s="86" t="s">
         <v>72</v>
       </c>
-      <c r="B28" s="83" t="s">
+      <c r="B28" s="90" t="s">
         <v>3</v>
       </c>
       <c r="C28" s="2" t="s">
@@ -2583,632 +2692,763 @@
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A29" s="80"/>
-      <c r="B29" s="84"/>
-      <c r="C29" t="s">
+      <c r="A29" s="87"/>
+      <c r="B29" s="91"/>
+      <c r="C29" s="47" t="s">
         <v>11</v>
       </c>
-      <c r="D29" t="s">
+      <c r="D29" s="47" t="s">
         <v>40</v>
       </c>
-      <c r="E29" s="7">
+      <c r="E29" s="49">
         <v>0.01</v>
       </c>
-      <c r="F29" t="s">
+      <c r="F29" s="47" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A30" s="80"/>
-      <c r="B30" s="84"/>
-      <c r="C30" t="s">
+      <c r="A30" s="87"/>
+      <c r="B30" s="91"/>
+      <c r="C30" s="47" t="s">
         <v>13</v>
       </c>
-      <c r="D30" t="s">
+      <c r="D30" s="47" t="s">
         <v>32</v>
       </c>
-      <c r="E30" s="21">
+      <c r="E30" s="50">
         <v>20</v>
       </c>
-      <c r="F30" t="s">
+      <c r="F30" s="47" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A31" s="80"/>
-      <c r="B31" s="84"/>
-      <c r="C31" t="s">
+      <c r="A31" s="87"/>
+      <c r="B31" s="91"/>
+      <c r="C31" s="47" t="s">
         <v>20</v>
       </c>
-      <c r="D31" t="s">
+      <c r="D31" s="47" t="s">
         <v>34</v>
       </c>
-      <c r="E31" s="47">
+      <c r="E31" s="77">
         <v>1.0000000000000001E-5</v>
       </c>
-      <c r="F31" s="13" t="s">
+      <c r="F31" s="51" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A32" s="80"/>
-      <c r="B32" s="84"/>
-      <c r="C32" t="s">
+      <c r="A32" s="87"/>
+      <c r="B32" s="91"/>
+      <c r="C32" s="47" t="s">
         <v>35</v>
       </c>
-      <c r="D32" t="s">
+      <c r="D32" s="47" t="s">
         <v>37</v>
       </c>
-      <c r="E32" s="7">
+      <c r="E32" s="49">
         <v>0.83299999999999996</v>
       </c>
-      <c r="F32" t="s">
+      <c r="F32" s="47" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A33" s="80"/>
-      <c r="B33" s="84"/>
-      <c r="C33" t="s">
+      <c r="A33" s="87"/>
+      <c r="B33" s="91"/>
+      <c r="C33" s="47" t="s">
         <v>36</v>
       </c>
-      <c r="D33" t="s">
+      <c r="D33" s="47" t="s">
         <v>38</v>
       </c>
-      <c r="E33" s="7">
+      <c r="E33" s="49">
         <v>0.83299999999999996</v>
       </c>
-      <c r="F33" t="s">
+      <c r="F33" s="47" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A34" s="80"/>
-      <c r="B34" s="84"/>
-      <c r="C34" t="s">
+      <c r="A34" s="87"/>
+      <c r="B34" s="91"/>
+      <c r="C34" s="47" t="s">
         <v>15</v>
       </c>
-      <c r="D34" t="s">
+      <c r="D34" s="47" t="s">
         <v>31</v>
       </c>
-      <c r="E34" s="7">
+      <c r="E34" s="49">
         <v>0.05</v>
       </c>
-      <c r="F34" t="s">
+      <c r="F34" s="47" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A35" s="80"/>
-      <c r="B35" s="84"/>
-      <c r="C35" t="s">
+    <row r="35" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A35" s="87"/>
+      <c r="B35" s="92"/>
+      <c r="C35" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="D35" t="s">
+      <c r="D35" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="E35" s="7">
+      <c r="E35" s="10">
         <v>0</v>
       </c>
-      <c r="F35" t="s">
+      <c r="F35" s="5" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A36" s="80"/>
-      <c r="B36" s="85" t="s">
-        <v>205</v>
-      </c>
-      <c r="C36" s="4" t="s">
+      <c r="A36" s="87"/>
+      <c r="B36" s="93" t="s">
+        <v>345</v>
+      </c>
+      <c r="C36" s="78" t="s">
+        <v>88</v>
+      </c>
+      <c r="D36" s="78" t="s">
+        <v>346</v>
+      </c>
+      <c r="E36" s="79">
+        <v>2.83</v>
+      </c>
+      <c r="F36" s="78" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A37" s="87"/>
+      <c r="B37" s="94"/>
+      <c r="C37" s="63" t="s">
+        <v>11</v>
+      </c>
+      <c r="D37" s="63" t="s">
+        <v>347</v>
+      </c>
+      <c r="E37" s="80">
+        <v>0.03</v>
+      </c>
+      <c r="F37" s="63" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A38" s="87"/>
+      <c r="B38" s="94"/>
+      <c r="C38" s="63" t="s">
+        <v>13</v>
+      </c>
+      <c r="D38" s="63" t="s">
+        <v>348</v>
+      </c>
+      <c r="E38" s="81">
+        <v>30</v>
+      </c>
+      <c r="F38" s="63" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A39" s="87"/>
+      <c r="B39" s="94"/>
+      <c r="C39" s="63" t="s">
+        <v>20</v>
+      </c>
+      <c r="D39" s="63" t="s">
+        <v>349</v>
+      </c>
+      <c r="E39" s="80">
+        <v>6.2550000000000001E-3</v>
+      </c>
+      <c r="F39" s="63" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A40" s="87"/>
+      <c r="B40" s="94"/>
+      <c r="C40" s="63" t="s">
+        <v>35</v>
+      </c>
+      <c r="D40" s="63" t="s">
+        <v>350</v>
+      </c>
+      <c r="E40" s="80">
+        <v>0.98</v>
+      </c>
+      <c r="F40" s="63" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A41" s="87"/>
+      <c r="B41" s="94"/>
+      <c r="C41" s="63" t="s">
+        <v>36</v>
+      </c>
+      <c r="D41" s="63" t="s">
+        <v>351</v>
+      </c>
+      <c r="E41" s="80">
+        <v>0.98</v>
+      </c>
+      <c r="F41" s="63" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A42" s="87"/>
+      <c r="B42" s="94"/>
+      <c r="C42" s="63" t="s">
+        <v>15</v>
+      </c>
+      <c r="D42" s="63" t="s">
+        <v>352</v>
+      </c>
+      <c r="E42" s="80">
+        <v>0.05</v>
+      </c>
+      <c r="F42" s="63" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A43" s="87"/>
+      <c r="B43" s="94"/>
+      <c r="C43" s="58" t="s">
+        <v>89</v>
+      </c>
+      <c r="D43" s="58" t="s">
+        <v>353</v>
+      </c>
+      <c r="E43" s="59">
+        <v>0</v>
+      </c>
+      <c r="F43" s="58" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A44" s="87"/>
+      <c r="B44" s="93" t="s">
+        <v>204</v>
+      </c>
+      <c r="C44" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="D36" s="4" t="s">
+      <c r="D44" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="E36" s="9">
+      <c r="E44" s="9">
         <v>1.6999999999999999E-3</v>
       </c>
-      <c r="F36" s="4" t="s">
+      <c r="F44" s="4" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A37" s="80"/>
-      <c r="B37" s="88"/>
-      <c r="C37" s="48" t="s">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A45" s="87"/>
+      <c r="B45" s="96"/>
+      <c r="C45" s="47" t="s">
         <v>21</v>
       </c>
-      <c r="D37" s="48" t="s">
+      <c r="D45" s="47" t="s">
         <v>55</v>
       </c>
-      <c r="E37" s="49">
-        <f>E38*4</f>
+      <c r="E45" s="48">
+        <f>E46*4</f>
         <v>424</v>
       </c>
-      <c r="F37" s="48" t="s">
+      <c r="F45" s="47" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A38" s="80"/>
-      <c r="B38" s="88"/>
-      <c r="C38" s="48" t="s">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A46" s="87"/>
+      <c r="B46" s="96"/>
+      <c r="C46" s="47" t="s">
         <v>16</v>
       </c>
-      <c r="D38" s="48" t="s">
+      <c r="D46" s="47" t="s">
         <v>56</v>
       </c>
-      <c r="E38" s="49">
+      <c r="E46" s="48">
         <v>106</v>
       </c>
-      <c r="F38" s="48" t="s">
+      <c r="F46" s="47" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A39" s="80"/>
-      <c r="B39" s="88"/>
-      <c r="C39" s="48" t="s">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A47" s="87"/>
+      <c r="B47" s="96"/>
+      <c r="C47" s="47" t="s">
         <v>17</v>
       </c>
-      <c r="D39" s="48" t="s">
+      <c r="D47" s="47" t="s">
         <v>57</v>
       </c>
-      <c r="E39" s="50">
+      <c r="E47" s="49">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="F39" s="48" t="s">
+      <c r="F47" s="47" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A40" s="80"/>
-      <c r="B40" s="88"/>
-      <c r="C40" s="48" t="s">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A48" s="87"/>
+      <c r="B48" s="96"/>
+      <c r="C48" s="47" t="s">
         <v>18</v>
       </c>
-      <c r="D40" s="48" t="s">
+      <c r="D48" s="47" t="s">
         <v>58</v>
       </c>
-      <c r="E40" s="49">
+      <c r="E48" s="48">
         <v>0</v>
       </c>
-      <c r="F40" s="52" t="s">
+      <c r="F48" s="51" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A41" s="80"/>
-      <c r="B41" s="88"/>
-      <c r="C41" s="48" t="s">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A49" s="87"/>
+      <c r="B49" s="96"/>
+      <c r="C49" s="47" t="s">
         <v>35</v>
       </c>
-      <c r="D41" s="48" t="s">
+      <c r="D49" s="47" t="s">
         <v>60</v>
       </c>
-      <c r="E41" s="50">
+      <c r="E49" s="49">
         <v>0.93500000000000005</v>
       </c>
-      <c r="F41" s="48" t="s">
+      <c r="F49" s="47" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A42" s="80"/>
-      <c r="B42" s="88"/>
-      <c r="C42" s="48" t="s">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A50" s="87"/>
+      <c r="B50" s="96"/>
+      <c r="C50" s="47" t="s">
         <v>36</v>
       </c>
-      <c r="D42" s="48" t="s">
+      <c r="D50" s="47" t="s">
         <v>61</v>
       </c>
-      <c r="E42" s="50">
+      <c r="E50" s="49">
         <v>0.93500000000000005</v>
       </c>
-      <c r="F42" s="48" t="s">
+      <c r="F50" s="47" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A43" s="80"/>
-      <c r="B43" s="88"/>
-      <c r="C43" s="48" t="s">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A51" s="87"/>
+      <c r="B51" s="96"/>
+      <c r="C51" s="47" t="s">
         <v>90</v>
       </c>
-      <c r="D43" s="48" t="s">
+      <c r="D51" s="47" t="s">
         <v>59</v>
       </c>
-      <c r="E43" s="49">
+      <c r="E51" s="48">
         <v>0.25</v>
       </c>
-      <c r="F43" s="48" t="s">
+      <c r="F51" s="47" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A44" s="80"/>
-      <c r="B44" s="88"/>
-      <c r="C44" s="48" t="s">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A52" s="87"/>
+      <c r="B52" s="96"/>
+      <c r="C52" s="47" t="s">
         <v>89</v>
       </c>
-      <c r="D44" s="48" t="s">
+      <c r="D52" s="47" t="s">
         <v>62</v>
       </c>
-      <c r="E44" s="50">
+      <c r="E52" s="49">
         <v>0</v>
       </c>
-      <c r="F44" s="48" t="s">
+      <c r="F52" s="47" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A45" s="80"/>
-      <c r="B45" s="88"/>
-      <c r="C45" s="48" t="s">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A53" s="87"/>
+      <c r="B53" s="96"/>
+      <c r="C53" s="47" t="s">
         <v>13</v>
       </c>
-      <c r="D45" s="48" t="s">
+      <c r="D53" s="47" t="s">
         <v>54</v>
       </c>
-      <c r="E45" s="51">
+      <c r="E53" s="50">
         <v>15</v>
       </c>
-      <c r="F45" s="48" t="s">
+      <c r="F53" s="47" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="46" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A46" s="81"/>
-      <c r="B46" s="89"/>
-      <c r="C46" s="15" t="s">
+    <row r="54" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A54" s="88"/>
+      <c r="B54" s="97"/>
+      <c r="C54" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="D46" s="15" t="s">
+      <c r="D54" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="E46" s="16">
+      <c r="E54" s="16">
         <v>0.1</v>
       </c>
-      <c r="F46" s="15" t="s">
+      <c r="F54" s="15" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A47" s="79" t="s">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A55" s="86" t="s">
         <v>73</v>
       </c>
-      <c r="B47" s="11" t="s">
+      <c r="B55" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="C47" s="2" t="s">
+      <c r="C55" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="D47" s="2" t="s">
+      <c r="D55" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="E47" s="22">
+      <c r="E55" s="22">
         <v>2000</v>
       </c>
-      <c r="F47" s="2" t="s">
+      <c r="F55" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A48" s="80"/>
-      <c r="B48" s="85" t="s">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A56" s="87"/>
+      <c r="B56" s="93" t="s">
         <v>4</v>
       </c>
-      <c r="C48" s="4" t="s">
+      <c r="C56" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D48" s="4" t="s">
+      <c r="D56" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="E48" s="9">
+      <c r="E56" s="9">
         <v>0.99</v>
       </c>
-      <c r="F48" s="4" t="s">
+      <c r="F56" s="4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A49" s="80"/>
-      <c r="B49" s="84"/>
-      <c r="C49" t="s">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A57" s="87"/>
+      <c r="B57" s="94"/>
+      <c r="C57" t="s">
         <v>10</v>
       </c>
-      <c r="D49" t="s">
+      <c r="D57" t="s">
         <v>43</v>
       </c>
-      <c r="E49" s="23">
+      <c r="E57" s="23">
         <v>1100</v>
       </c>
-      <c r="F49" t="s">
+      <c r="F57" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A50" s="80"/>
-      <c r="B50" s="84"/>
-      <c r="C50" t="s">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A58" s="87"/>
+      <c r="B58" s="94"/>
+      <c r="C58" t="s">
         <v>17</v>
       </c>
-      <c r="D50" t="s">
+      <c r="D58" t="s">
         <v>44</v>
       </c>
-      <c r="E50" s="23">
+      <c r="E58" s="23">
         <v>17.84</v>
       </c>
-      <c r="F50" t="s">
+      <c r="F58" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A51" s="80"/>
-      <c r="B51" s="84"/>
-      <c r="C51" t="s">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A59" s="87"/>
+      <c r="B59" s="94"/>
+      <c r="C59" t="s">
         <v>18</v>
       </c>
-      <c r="D51" t="s">
+      <c r="D59" t="s">
         <v>45</v>
       </c>
-      <c r="E51" s="14">
+      <c r="E59" s="14">
         <v>0</v>
       </c>
-      <c r="F51" t="s">
+      <c r="F59" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A52" s="80"/>
-      <c r="B52" s="84"/>
-      <c r="C52" t="s">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A60" s="87"/>
+      <c r="B60" s="94"/>
+      <c r="C60" t="s">
         <v>13</v>
       </c>
-      <c r="D52" t="s">
+      <c r="D60" t="s">
         <v>42</v>
       </c>
-      <c r="E52" s="21">
+      <c r="E60" s="21">
         <v>25</v>
       </c>
-      <c r="F52" t="s">
+      <c r="F60" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A53" s="80"/>
-      <c r="B53" s="84"/>
-      <c r="C53" t="s">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A61" s="87"/>
+      <c r="B61" s="94"/>
+      <c r="C61" t="s">
         <v>69</v>
       </c>
-      <c r="D53" t="s">
+      <c r="D61" t="s">
         <v>68</v>
       </c>
-      <c r="E53" s="14">
+      <c r="E61" s="14">
         <v>1000000</v>
       </c>
-      <c r="F53" t="s">
+      <c r="F61" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A54" s="80"/>
-      <c r="B54" s="86"/>
-      <c r="C54" s="5" t="s">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A62" s="87"/>
+      <c r="B62" s="92"/>
+      <c r="C62" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="D54" s="5" t="s">
+      <c r="D62" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="E54" s="10">
+      <c r="E62" s="10">
         <v>5.2999999999999999E-2</v>
       </c>
-      <c r="F54" s="5" t="s">
+      <c r="F62" s="5" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A55" s="80"/>
-      <c r="B55" s="85" t="s">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A63" s="87"/>
+      <c r="B63" s="93" t="s">
         <v>5</v>
       </c>
-      <c r="C55" s="4" t="s">
+      <c r="C63" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D55" s="4" t="s">
+      <c r="D63" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="E55" s="9">
+      <c r="E63" s="9">
         <v>0.997</v>
       </c>
-      <c r="F55" s="4" t="s">
+      <c r="F63" s="4" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A56" s="80"/>
-      <c r="B56" s="84"/>
-      <c r="C56" t="s">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A64" s="87"/>
+      <c r="B64" s="94"/>
+      <c r="C64" t="s">
         <v>10</v>
       </c>
-      <c r="D56" t="s">
+      <c r="D64" t="s">
         <v>48</v>
       </c>
-      <c r="E56" s="23">
+      <c r="E64" s="23">
         <v>1080</v>
       </c>
-      <c r="F56" t="s">
+      <c r="F64" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A57" s="80"/>
-      <c r="B57" s="84"/>
-      <c r="C57" t="s">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A65" s="87"/>
+      <c r="B65" s="94"/>
+      <c r="C65" t="s">
         <v>17</v>
       </c>
-      <c r="D57" t="s">
+      <c r="D65" t="s">
         <v>52</v>
       </c>
-      <c r="E57" s="43">
+      <c r="E65" s="43">
         <v>12.68</v>
       </c>
-      <c r="F57" s="24" t="s">
+      <c r="F65" s="24" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A58" s="80"/>
-      <c r="B58" s="84"/>
-      <c r="C58" t="s">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A66" s="87"/>
+      <c r="B66" s="94"/>
+      <c r="C66" t="s">
         <v>18</v>
       </c>
-      <c r="D58" t="s">
+      <c r="D66" t="s">
         <v>49</v>
       </c>
-      <c r="E58" s="46">
+      <c r="E66" s="46">
         <v>5.0000000000000001E-3</v>
       </c>
-      <c r="F58" t="s">
+      <c r="F66" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A59" s="80"/>
-      <c r="B59" s="84"/>
-      <c r="C59" t="s">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A67" s="87"/>
+      <c r="B67" s="94"/>
+      <c r="C67" t="s">
         <v>13</v>
       </c>
-      <c r="D59" t="s">
+      <c r="D67" t="s">
         <v>50</v>
       </c>
-      <c r="E59" s="21">
+      <c r="E67" s="21">
         <v>25</v>
       </c>
-      <c r="F59" t="s">
+      <c r="F67" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A60" s="80"/>
-      <c r="B60" s="84"/>
-      <c r="C60" t="s">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A68" s="87"/>
+      <c r="B68" s="94"/>
+      <c r="C68" t="s">
         <v>69</v>
       </c>
-      <c r="D60" t="s">
+      <c r="D68" t="s">
         <v>66</v>
       </c>
-      <c r="E60" s="25">
+      <c r="E68" s="25">
         <v>1000000</v>
       </c>
-      <c r="F60" t="s">
+      <c r="F68" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A61" s="81"/>
-      <c r="B61" s="87"/>
-      <c r="C61" s="15" t="s">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A69" s="88"/>
+      <c r="B69" s="95"/>
+      <c r="C69" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="D61" s="15" t="s">
+      <c r="D69" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="E61" s="16">
+      <c r="E69" s="16">
         <v>5.8000000000000003E-2</v>
       </c>
-      <c r="F61" s="15" t="s">
+      <c r="F69" s="15" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A62" s="79" t="s">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A70" s="86" t="s">
         <v>77</v>
       </c>
-      <c r="B62" s="74" t="s">
+      <c r="B70" s="72" t="s">
         <v>74</v>
       </c>
-      <c r="C62" s="75" t="s">
+      <c r="C70" s="73" t="s">
         <v>78</v>
       </c>
-      <c r="D62" s="75" t="s">
+      <c r="D70" s="73" t="s">
         <v>79</v>
       </c>
-      <c r="E62" s="76">
+      <c r="E70" s="74">
         <v>-1E-4</v>
       </c>
-      <c r="F62" s="75" t="s">
+      <c r="F70" s="73" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A63" s="82"/>
-      <c r="B63" s="73" t="s">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A71" s="89"/>
+      <c r="B71" s="71" t="s">
+        <v>327</v>
+      </c>
+      <c r="C71" s="75" t="s">
         <v>328</v>
       </c>
-      <c r="C63" s="77" t="s">
+      <c r="D71" s="75" t="s">
         <v>329</v>
       </c>
-      <c r="D63" s="77" t="s">
-        <v>330</v>
-      </c>
-      <c r="E63" s="50">
+      <c r="E71" s="49">
         <v>-1E-4</v>
       </c>
-      <c r="F63" s="77" t="s">
+      <c r="F71" s="75" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A64" s="80"/>
-      <c r="B64" s="17" t="s">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A72" s="87"/>
+      <c r="B72" s="17" t="s">
         <v>80</v>
       </c>
-      <c r="C64" s="18" t="s">
+      <c r="C72" s="18" t="s">
         <v>81</v>
       </c>
-      <c r="D64" s="18" t="s">
+      <c r="D72" s="18" t="s">
         <v>82</v>
       </c>
-      <c r="E64" s="19">
+      <c r="E72" s="19">
         <v>-1.5</v>
       </c>
-      <c r="F64" s="18" t="s">
+      <c r="F72" s="18" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A65" s="81"/>
-      <c r="B65" s="1" t="s">
-        <v>278</v>
-      </c>
-      <c r="C65" s="15" t="s">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A73" s="88"/>
+      <c r="B73" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="C73" s="15" t="s">
+        <v>299</v>
+      </c>
+      <c r="D73" s="15" t="s">
+        <v>297</v>
+      </c>
+      <c r="E73" s="16">
+        <v>-0.6</v>
+      </c>
+      <c r="F73" s="15" t="s">
         <v>300</v>
       </c>
-      <c r="D65" s="15" t="s">
-        <v>298</v>
-      </c>
-      <c r="E65" s="16">
-        <v>-0.6</v>
-      </c>
-      <c r="F65" s="15" t="s">
-        <v>301</v>
-      </c>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="13">
     <mergeCell ref="A2:A27"/>
-    <mergeCell ref="A28:A46"/>
-    <mergeCell ref="A47:A61"/>
-    <mergeCell ref="A62:A65"/>
+    <mergeCell ref="A28:A54"/>
+    <mergeCell ref="A55:A69"/>
+    <mergeCell ref="A70:A73"/>
     <mergeCell ref="B28:B35"/>
-    <mergeCell ref="B48:B54"/>
-    <mergeCell ref="B55:B61"/>
-    <mergeCell ref="B36:B46"/>
+    <mergeCell ref="B56:B62"/>
+    <mergeCell ref="B63:B69"/>
+    <mergeCell ref="B44:B54"/>
     <mergeCell ref="B2:B7"/>
     <mergeCell ref="B8:B15"/>
     <mergeCell ref="B22:B27"/>
     <mergeCell ref="B16:B21"/>
+    <mergeCell ref="B36:B43"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -3218,7 +3458,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83AB2E79-6F94-41B5-A552-C40EC4890194}">
-  <dimension ref="A1:F127"/>
+  <dimension ref="A1:F140"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.5546875" style="13" customWidth="1"/>
@@ -3251,10 +3491,10 @@
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="97" t="s">
+      <c r="A2" s="109" t="s">
         <v>71</v>
       </c>
-      <c r="B2" s="99" t="s">
+      <c r="B2" s="108" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="26" t="s">
@@ -3269,8 +3509,8 @@
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="98"/>
-      <c r="B3" s="93"/>
+      <c r="A3" s="111"/>
+      <c r="B3" s="101"/>
       <c r="C3" s="13" t="s">
         <v>109</v>
       </c>
@@ -3283,8 +3523,8 @@
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="98"/>
-      <c r="B4" s="93"/>
+      <c r="A4" s="111"/>
+      <c r="B4" s="101"/>
       <c r="C4" s="13" t="s">
         <v>85</v>
       </c>
@@ -3297,8 +3537,8 @@
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="98"/>
-      <c r="B5" s="93"/>
+      <c r="A5" s="111"/>
+      <c r="B5" s="101"/>
       <c r="C5" s="13" t="s">
         <v>140</v>
       </c>
@@ -3311,8 +3551,8 @@
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="98"/>
-      <c r="B6" s="93"/>
+      <c r="A6" s="111"/>
+      <c r="B6" s="101"/>
       <c r="C6" s="13" t="s">
         <v>143</v>
       </c>
@@ -3325,8 +3565,8 @@
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="98"/>
-      <c r="B7" s="93"/>
+      <c r="A7" s="111"/>
+      <c r="B7" s="101"/>
       <c r="C7" s="13" t="s">
         <v>157</v>
       </c>
@@ -3339,13 +3579,13 @@
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="98"/>
-      <c r="B8" s="93"/>
+      <c r="A8" s="111"/>
+      <c r="B8" s="101"/>
       <c r="C8" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E8" s="34"/>
       <c r="F8" s="13" t="s">
@@ -3353,8 +3593,8 @@
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="98"/>
-      <c r="B9" s="93"/>
+      <c r="A9" s="111"/>
+      <c r="B9" s="101"/>
       <c r="C9" s="13" t="s">
         <v>169</v>
       </c>
@@ -3367,13 +3607,13 @@
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="98"/>
-      <c r="B10" s="93"/>
+      <c r="A10" s="111"/>
+      <c r="B10" s="101"/>
       <c r="C10" s="13" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E10" s="34"/>
       <c r="F10" s="13" t="s">
@@ -3381,451 +3621,451 @@
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" s="98"/>
-      <c r="B11" s="93"/>
+      <c r="A11" s="111"/>
+      <c r="B11" s="101"/>
       <c r="E11" s="33"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="98"/>
-      <c r="B12" s="100" t="s">
-        <v>234</v>
-      </c>
-      <c r="C12" s="55" t="s">
+      <c r="A12" s="111"/>
+      <c r="B12" s="105" t="s">
+        <v>233</v>
+      </c>
+      <c r="C12" s="54" t="s">
         <v>98</v>
       </c>
-      <c r="D12" s="55" t="s">
-        <v>255</v>
-      </c>
-      <c r="E12" s="56"/>
-      <c r="F12" s="55" t="s">
+      <c r="D12" s="54" t="s">
+        <v>254</v>
+      </c>
+      <c r="E12" s="55"/>
+      <c r="F12" s="54" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="98"/>
-      <c r="B13" s="101"/>
+      <c r="A13" s="111"/>
+      <c r="B13" s="106"/>
       <c r="C13" s="45" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="D13" s="45" t="s">
-        <v>327</v>
-      </c>
-      <c r="E13" s="54"/>
+        <v>326</v>
+      </c>
+      <c r="E13" s="53"/>
       <c r="F13" s="45" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" s="98"/>
-      <c r="B14" s="101"/>
+      <c r="A14" s="111"/>
+      <c r="B14" s="106"/>
       <c r="C14" s="45" t="s">
         <v>141</v>
       </c>
       <c r="D14" s="45" t="s">
-        <v>256</v>
-      </c>
-      <c r="E14" s="54"/>
-      <c r="F14" s="54" t="s">
+        <v>255</v>
+      </c>
+      <c r="E14" s="53"/>
+      <c r="F14" s="53" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" s="98"/>
-      <c r="B15" s="101"/>
+      <c r="A15" s="111"/>
+      <c r="B15" s="106"/>
       <c r="C15" s="45" t="s">
+        <v>263</v>
+      </c>
+      <c r="D15" s="45" t="s">
         <v>264</v>
       </c>
-      <c r="D15" s="45" t="s">
-        <v>265</v>
-      </c>
-      <c r="E15" s="57"/>
+      <c r="E15" s="56"/>
       <c r="F15" s="45" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" s="98"/>
-      <c r="B16" s="101"/>
+      <c r="A16" s="111"/>
+      <c r="B16" s="106"/>
       <c r="C16" s="45" t="s">
         <v>85</v>
       </c>
       <c r="D16" s="45" t="s">
-        <v>257</v>
-      </c>
-      <c r="E16" s="54"/>
+        <v>256</v>
+      </c>
+      <c r="E16" s="53"/>
       <c r="F16" s="45" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" s="98"/>
-      <c r="B17" s="101"/>
+      <c r="A17" s="111"/>
+      <c r="B17" s="106"/>
       <c r="C17" s="45" t="s">
         <v>143</v>
       </c>
       <c r="D17" s="45" t="s">
-        <v>258</v>
-      </c>
-      <c r="E17" s="54"/>
+        <v>257</v>
+      </c>
+      <c r="E17" s="53"/>
       <c r="F17" s="45" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" s="98"/>
-      <c r="B18" s="101"/>
+      <c r="A18" s="111"/>
+      <c r="B18" s="106"/>
       <c r="C18" s="45" t="s">
         <v>157</v>
       </c>
       <c r="D18" s="45" t="s">
-        <v>259</v>
-      </c>
-      <c r="E18" s="58"/>
+        <v>258</v>
+      </c>
+      <c r="E18" s="57"/>
       <c r="F18" s="45" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" s="98"/>
-      <c r="B19" s="101"/>
+      <c r="A19" s="111"/>
+      <c r="B19" s="106"/>
       <c r="C19" s="45" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="D19" s="45" t="s">
-        <v>260</v>
-      </c>
-      <c r="E19" s="58"/>
+        <v>259</v>
+      </c>
+      <c r="E19" s="57"/>
       <c r="F19" s="45" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" s="98"/>
-      <c r="B20" s="101"/>
+      <c r="A20" s="111"/>
+      <c r="B20" s="106"/>
       <c r="C20" s="45" t="s">
         <v>169</v>
       </c>
       <c r="D20" s="45" t="s">
-        <v>261</v>
-      </c>
-      <c r="E20" s="58"/>
+        <v>260</v>
+      </c>
+      <c r="E20" s="57"/>
       <c r="F20" s="45" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A21" s="98"/>
-      <c r="B21" s="101"/>
+      <c r="A21" s="111"/>
+      <c r="B21" s="106"/>
       <c r="C21" s="45" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D21" s="45" t="s">
-        <v>262</v>
-      </c>
-      <c r="E21" s="58"/>
+        <v>261</v>
+      </c>
+      <c r="E21" s="57"/>
       <c r="F21" s="45" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A22" s="98"/>
-      <c r="B22" s="102"/>
-      <c r="C22" s="59"/>
-      <c r="D22" s="59"/>
-      <c r="E22" s="60"/>
-      <c r="F22" s="59"/>
+      <c r="A22" s="111"/>
+      <c r="B22" s="116"/>
+      <c r="C22" s="58"/>
+      <c r="D22" s="58"/>
+      <c r="E22" s="59"/>
+      <c r="F22" s="58"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" s="98"/>
-      <c r="B23" s="100" t="s">
-        <v>299</v>
+      <c r="A23" s="111"/>
+      <c r="B23" s="105" t="s">
+        <v>298</v>
       </c>
       <c r="C23" s="45" t="s">
         <v>98</v>
       </c>
       <c r="D23" s="45" t="s">
-        <v>312</v>
-      </c>
-      <c r="E23" s="54"/>
+        <v>311</v>
+      </c>
+      <c r="E23" s="53"/>
       <c r="F23" s="45" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" s="98"/>
-      <c r="B24" s="108"/>
+      <c r="A24" s="111"/>
+      <c r="B24" s="119"/>
       <c r="C24" s="45" t="s">
         <v>109</v>
       </c>
       <c r="D24" s="45" t="s">
-        <v>313</v>
-      </c>
-      <c r="E24" s="54"/>
+        <v>312</v>
+      </c>
+      <c r="E24" s="53"/>
       <c r="F24" s="45" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25" s="98"/>
-      <c r="B25" s="108"/>
+      <c r="A25" s="111"/>
+      <c r="B25" s="119"/>
       <c r="C25" s="45" t="s">
         <v>85</v>
       </c>
       <c r="D25" s="45" t="s">
-        <v>314</v>
-      </c>
-      <c r="E25" s="57"/>
+        <v>313</v>
+      </c>
+      <c r="E25" s="56"/>
       <c r="F25" s="45" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26" s="98"/>
-      <c r="B26" s="108"/>
+      <c r="A26" s="111"/>
+      <c r="B26" s="119"/>
       <c r="C26" s="45" t="s">
+        <v>321</v>
+      </c>
+      <c r="D26" s="45" t="s">
         <v>322</v>
       </c>
-      <c r="D26" s="45" t="s">
-        <v>323</v>
-      </c>
-      <c r="E26" s="58"/>
+      <c r="E26" s="57"/>
       <c r="F26" s="45" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A27" s="98"/>
-      <c r="B27" s="108"/>
+      <c r="A27" s="111"/>
+      <c r="B27" s="119"/>
       <c r="C27" s="45" t="s">
         <v>143</v>
       </c>
       <c r="D27" s="45" t="s">
-        <v>315</v>
-      </c>
-      <c r="E27" s="58"/>
+        <v>314</v>
+      </c>
+      <c r="E27" s="57"/>
       <c r="F27" s="45" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A28" s="98"/>
-      <c r="B28" s="108"/>
+      <c r="A28" s="111"/>
+      <c r="B28" s="119"/>
       <c r="C28" s="45" t="s">
         <v>157</v>
       </c>
       <c r="D28" s="45" t="s">
-        <v>316</v>
-      </c>
-      <c r="E28" s="58"/>
+        <v>315</v>
+      </c>
+      <c r="E28" s="57"/>
       <c r="F28" s="45" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A29" s="98"/>
-      <c r="B29" s="108"/>
+      <c r="A29" s="111"/>
+      <c r="B29" s="119"/>
       <c r="C29" s="45" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="D29" s="45" t="s">
-        <v>317</v>
-      </c>
-      <c r="E29" s="58"/>
+        <v>316</v>
+      </c>
+      <c r="E29" s="57"/>
       <c r="F29" s="45" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A30" s="98"/>
-      <c r="B30" s="108"/>
+      <c r="A30" s="111"/>
+      <c r="B30" s="119"/>
       <c r="C30" s="45" t="s">
         <v>169</v>
       </c>
       <c r="D30" s="45" t="s">
-        <v>318</v>
-      </c>
-      <c r="E30" s="57"/>
+        <v>317</v>
+      </c>
+      <c r="E30" s="56"/>
       <c r="F30" s="45" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A31" s="98"/>
-      <c r="B31" s="108"/>
+      <c r="A31" s="111"/>
+      <c r="B31" s="119"/>
       <c r="C31" s="45" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D31" s="45" t="s">
-        <v>319</v>
-      </c>
-      <c r="E31" s="57"/>
+        <v>318</v>
+      </c>
+      <c r="E31" s="56"/>
       <c r="F31" s="45" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A32" s="98"/>
-      <c r="B32" s="102"/>
-      <c r="C32" s="59"/>
-      <c r="D32" s="59"/>
-      <c r="E32" s="60"/>
-      <c r="F32" s="59"/>
+      <c r="A32" s="111"/>
+      <c r="B32" s="116"/>
+      <c r="C32" s="58"/>
+      <c r="D32" s="58"/>
+      <c r="E32" s="59"/>
+      <c r="F32" s="58"/>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A33" s="98"/>
-      <c r="B33" s="103" t="s">
-        <v>233</v>
+      <c r="A33" s="111"/>
+      <c r="B33" s="117" t="s">
+        <v>232</v>
       </c>
       <c r="C33" s="45" t="s">
         <v>98</v>
       </c>
       <c r="D33" s="45" t="s">
-        <v>268</v>
-      </c>
-      <c r="E33" s="54"/>
+        <v>267</v>
+      </c>
+      <c r="E33" s="53"/>
       <c r="F33" s="45" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A34" s="98"/>
-      <c r="B34" s="103"/>
+      <c r="A34" s="111"/>
+      <c r="B34" s="117"/>
       <c r="C34" s="45" t="s">
         <v>109</v>
       </c>
       <c r="D34" s="45" t="s">
-        <v>269</v>
-      </c>
-      <c r="E34" s="54"/>
+        <v>268</v>
+      </c>
+      <c r="E34" s="53"/>
       <c r="F34" s="45" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A35" s="98"/>
-      <c r="B35" s="103"/>
+      <c r="A35" s="111"/>
+      <c r="B35" s="117"/>
       <c r="C35" s="45" t="s">
         <v>85</v>
       </c>
       <c r="D35" s="45" t="s">
-        <v>270</v>
-      </c>
-      <c r="E35" s="57"/>
+        <v>269</v>
+      </c>
+      <c r="E35" s="56"/>
       <c r="F35" s="45" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A36" s="98"/>
-      <c r="B36" s="103"/>
+      <c r="A36" s="111"/>
+      <c r="B36" s="117"/>
       <c r="C36" s="45" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="D36" s="45" t="s">
-        <v>326</v>
-      </c>
-      <c r="E36" s="57"/>
+        <v>325</v>
+      </c>
+      <c r="E36" s="56"/>
       <c r="F36" s="45" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A37" s="98"/>
-      <c r="B37" s="103"/>
+      <c r="A37" s="111"/>
+      <c r="B37" s="117"/>
       <c r="C37" s="45" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="D37" s="45" t="s">
-        <v>325</v>
-      </c>
-      <c r="E37" s="58"/>
+        <v>324</v>
+      </c>
+      <c r="E37" s="57"/>
       <c r="F37" s="45" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A38" s="98"/>
-      <c r="B38" s="103"/>
+      <c r="A38" s="111"/>
+      <c r="B38" s="117"/>
       <c r="C38" s="45" t="s">
         <v>143</v>
       </c>
       <c r="D38" s="45" t="s">
-        <v>271</v>
-      </c>
-      <c r="E38" s="58"/>
+        <v>270</v>
+      </c>
+      <c r="E38" s="57"/>
       <c r="F38" s="45" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A39" s="98"/>
-      <c r="B39" s="103"/>
+      <c r="A39" s="111"/>
+      <c r="B39" s="117"/>
       <c r="C39" s="45" t="s">
         <v>157</v>
       </c>
       <c r="D39" s="45" t="s">
-        <v>272</v>
-      </c>
-      <c r="E39" s="58"/>
+        <v>271</v>
+      </c>
+      <c r="E39" s="57"/>
       <c r="F39" s="45" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A40" s="98"/>
-      <c r="B40" s="103"/>
+      <c r="A40" s="111"/>
+      <c r="B40" s="117"/>
       <c r="C40" s="45" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="D40" s="45" t="s">
-        <v>273</v>
-      </c>
-      <c r="E40" s="58"/>
+        <v>272</v>
+      </c>
+      <c r="E40" s="57"/>
       <c r="F40" s="45" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A41" s="98"/>
-      <c r="B41" s="103"/>
+      <c r="A41" s="111"/>
+      <c r="B41" s="117"/>
       <c r="C41" s="45" t="s">
         <v>169</v>
       </c>
       <c r="D41" s="45" t="s">
-        <v>274</v>
-      </c>
-      <c r="E41" s="57"/>
+        <v>273</v>
+      </c>
+      <c r="E41" s="56"/>
       <c r="F41" s="45" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A42" s="98"/>
-      <c r="B42" s="103"/>
+      <c r="A42" s="111"/>
+      <c r="B42" s="117"/>
       <c r="C42" s="45" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D42" s="45" t="s">
-        <v>275</v>
-      </c>
-      <c r="E42" s="57"/>
+        <v>274</v>
+      </c>
+      <c r="E42" s="56"/>
       <c r="F42" s="45" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="43" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="98"/>
-      <c r="B43" s="103"/>
+      <c r="A43" s="111"/>
+      <c r="B43" s="117"/>
       <c r="C43" s="45"/>
       <c r="D43" s="45"/>
-      <c r="E43" s="57"/>
+      <c r="E43" s="56"/>
       <c r="F43" s="45"/>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A44" s="97" t="s">
+    <row r="44" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="109" t="s">
         <v>72</v>
       </c>
-      <c r="B44" s="105" t="s">
+      <c r="B44" s="120" t="s">
         <v>3</v>
       </c>
       <c r="C44" s="26" t="s">
@@ -3835,470 +4075,477 @@
         <v>105</v>
       </c>
       <c r="E44" s="39"/>
-      <c r="F44" s="61" t="s">
-        <v>190</v>
+      <c r="F44" s="60" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A45" s="98"/>
-      <c r="B45" s="95"/>
-      <c r="C45" s="13" t="s">
+      <c r="A45" s="111"/>
+      <c r="B45" s="121"/>
+      <c r="C45" s="51" t="s">
         <v>113</v>
       </c>
-      <c r="D45" s="13" t="s">
+      <c r="D45" s="51" t="s">
         <v>112</v>
       </c>
-      <c r="E45" s="33"/>
-      <c r="F45" s="62" t="s">
+      <c r="E45" s="52"/>
+      <c r="F45" s="82" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A46" s="98"/>
-      <c r="B46" s="95"/>
-      <c r="C46" s="13" t="s">
+      <c r="A46" s="111"/>
+      <c r="B46" s="121"/>
+      <c r="C46" s="51" t="s">
         <v>137</v>
       </c>
-      <c r="D46" s="13" t="s">
+      <c r="D46" s="51" t="s">
         <v>135</v>
       </c>
-      <c r="E46" s="34"/>
-      <c r="F46" s="13" t="s">
+      <c r="E46" s="83"/>
+      <c r="F46" s="51" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A47" s="98"/>
-      <c r="B47" s="95"/>
-      <c r="C47" s="13" t="s">
+      <c r="A47" s="111"/>
+      <c r="B47" s="121"/>
+      <c r="C47" s="51" t="s">
         <v>138</v>
       </c>
-      <c r="D47" s="13" t="s">
+      <c r="D47" s="51" t="s">
         <v>136</v>
       </c>
-      <c r="E47" s="33"/>
-      <c r="F47" s="13" t="s">
+      <c r="E47" s="52"/>
+      <c r="F47" s="51" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A48" s="98"/>
-      <c r="B48" s="95"/>
-      <c r="C48" s="13" t="s">
+      <c r="A48" s="111"/>
+      <c r="B48" s="121"/>
+      <c r="C48" s="51" t="s">
         <v>143</v>
       </c>
-      <c r="D48" s="13" t="s">
+      <c r="D48" s="51" t="s">
         <v>148</v>
       </c>
-      <c r="E48" s="33"/>
-      <c r="F48" s="13" t="s">
+      <c r="E48" s="52"/>
+      <c r="F48" s="51" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A49" s="98"/>
-      <c r="B49" s="95"/>
-      <c r="C49" s="13" t="s">
+      <c r="A49" s="111"/>
+      <c r="B49" s="121"/>
+      <c r="C49" s="51" t="s">
         <v>157</v>
       </c>
-      <c r="D49" s="13" t="s">
+      <c r="D49" s="51" t="s">
         <v>161</v>
       </c>
-      <c r="E49" s="33"/>
-      <c r="F49" s="13" t="s">
+      <c r="E49" s="52"/>
+      <c r="F49" s="51" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A50" s="98"/>
-      <c r="B50" s="95"/>
-      <c r="C50" s="13" t="s">
-        <v>200</v>
-      </c>
-      <c r="D50" s="13" t="s">
-        <v>203</v>
-      </c>
-      <c r="E50" s="33"/>
-      <c r="F50" s="13" t="s">
+      <c r="A50" s="111"/>
+      <c r="B50" s="121"/>
+      <c r="C50" s="51" t="s">
+        <v>199</v>
+      </c>
+      <c r="D50" s="51" t="s">
+        <v>202</v>
+      </c>
+      <c r="E50" s="52"/>
+      <c r="F50" s="51" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A51" s="98"/>
-      <c r="B51" s="95"/>
-      <c r="C51" s="13" t="s">
+      <c r="A51" s="111"/>
+      <c r="B51" s="121"/>
+      <c r="C51" s="51" t="s">
         <v>169</v>
       </c>
-      <c r="D51" s="13" t="s">
+      <c r="D51" s="51" t="s">
         <v>173</v>
       </c>
-      <c r="E51" s="33"/>
-      <c r="F51" s="13" t="s">
+      <c r="E51" s="52"/>
+      <c r="F51" s="51" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A52" s="98"/>
-      <c r="B52" s="95"/>
-      <c r="C52" s="13" t="s">
-        <v>192</v>
-      </c>
-      <c r="D52" s="13" t="s">
-        <v>197</v>
-      </c>
-      <c r="E52" s="33"/>
-      <c r="F52" s="13" t="s">
+      <c r="A52" s="111"/>
+      <c r="B52" s="121"/>
+      <c r="C52" s="51" t="s">
+        <v>191</v>
+      </c>
+      <c r="D52" s="51" t="s">
+        <v>196</v>
+      </c>
+      <c r="E52" s="52"/>
+      <c r="F52" s="51" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A53" s="98"/>
-      <c r="B53" s="95"/>
-      <c r="E53" s="33"/>
+      <c r="A53" s="111"/>
+      <c r="B53" s="114"/>
+      <c r="C53" s="37"/>
+      <c r="D53" s="37"/>
+      <c r="E53" s="38"/>
+      <c r="F53" s="37"/>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A54" s="98"/>
-      <c r="B54" s="106" t="s">
+      <c r="A54" s="111"/>
+      <c r="B54" s="117" t="s">
+        <v>345</v>
+      </c>
+      <c r="C54" s="63" t="s">
+        <v>115</v>
+      </c>
+      <c r="D54" s="63" t="s">
+        <v>355</v>
+      </c>
+      <c r="E54" s="84"/>
+      <c r="F54" s="63" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A55" s="111"/>
+      <c r="B55" s="117"/>
+      <c r="C55" s="45" t="s">
+        <v>113</v>
+      </c>
+      <c r="D55" s="45" t="s">
+        <v>356</v>
+      </c>
+      <c r="E55" s="56"/>
+      <c r="F55" s="45" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A56" s="111"/>
+      <c r="B56" s="117"/>
+      <c r="C56" s="45" t="s">
+        <v>137</v>
+      </c>
+      <c r="D56" s="45" t="s">
+        <v>357</v>
+      </c>
+      <c r="E56" s="57"/>
+      <c r="F56" s="85" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A57" s="111"/>
+      <c r="B57" s="117"/>
+      <c r="C57" s="45" t="s">
+        <v>138</v>
+      </c>
+      <c r="D57" s="45" t="s">
+        <v>358</v>
+      </c>
+      <c r="E57" s="56"/>
+      <c r="F57" s="85" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A58" s="111"/>
+      <c r="B58" s="117"/>
+      <c r="C58" s="45" t="s">
+        <v>143</v>
+      </c>
+      <c r="D58" s="45" t="s">
+        <v>359</v>
+      </c>
+      <c r="E58" s="56"/>
+      <c r="F58" s="85" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A59" s="111"/>
+      <c r="B59" s="117"/>
+      <c r="C59" s="45" t="s">
+        <v>157</v>
+      </c>
+      <c r="D59" s="45" t="s">
+        <v>360</v>
+      </c>
+      <c r="E59" s="56"/>
+      <c r="F59" s="85" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A60" s="111"/>
+      <c r="B60" s="117"/>
+      <c r="C60" s="45" t="s">
+        <v>199</v>
+      </c>
+      <c r="D60" s="45" t="s">
+        <v>361</v>
+      </c>
+      <c r="E60" s="56"/>
+      <c r="F60" s="85" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A61" s="111"/>
+      <c r="B61" s="117"/>
+      <c r="C61" s="45" t="s">
+        <v>169</v>
+      </c>
+      <c r="D61" s="45" t="s">
+        <v>362</v>
+      </c>
+      <c r="E61" s="56"/>
+      <c r="F61" s="85" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A62" s="111"/>
+      <c r="B62" s="117"/>
+      <c r="C62" s="45" t="s">
+        <v>191</v>
+      </c>
+      <c r="D62" s="45" t="s">
+        <v>363</v>
+      </c>
+      <c r="E62" s="56"/>
+      <c r="F62" s="85" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A63" s="111"/>
+      <c r="B63" s="122"/>
+      <c r="C63" s="45"/>
+      <c r="D63" s="45"/>
+      <c r="E63" s="56"/>
+      <c r="F63" s="45"/>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A64" s="111"/>
+      <c r="B64" s="113" t="s">
         <v>6</v>
       </c>
-      <c r="C54" s="35" t="s">
+      <c r="C64" s="35" t="s">
         <v>98</v>
       </c>
-      <c r="D54" s="35" t="s">
+      <c r="D64" s="35" t="s">
         <v>102</v>
       </c>
-      <c r="E54" s="40"/>
-      <c r="F54" s="35" t="s">
+      <c r="E64" s="40"/>
+      <c r="F64" s="35" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A55" s="98"/>
-      <c r="B55" s="95"/>
-      <c r="C55" s="13" t="s">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A65" s="111"/>
+      <c r="B65" s="103"/>
+      <c r="C65" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="D55" s="13" t="s">
+      <c r="D65" s="13" t="s">
         <v>104</v>
       </c>
-      <c r="E55" s="33"/>
-      <c r="F55" s="13" t="s">
+      <c r="E65" s="33"/>
+      <c r="F65" s="13" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A56" s="98"/>
-      <c r="B56" s="93"/>
-      <c r="C56" s="13" t="s">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A66" s="111"/>
+      <c r="B66" s="101"/>
+      <c r="C66" s="13" t="s">
         <v>113</v>
       </c>
-      <c r="D56" s="13" t="s">
+      <c r="D66" s="13" t="s">
         <v>114</v>
       </c>
-      <c r="E56" s="31"/>
-      <c r="F56" s="13" t="s">
+      <c r="E66" s="31"/>
+      <c r="F66" s="13" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A57" s="98"/>
-      <c r="B57" s="93"/>
-      <c r="C57" s="13" t="s">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A67" s="111"/>
+      <c r="B67" s="101"/>
+      <c r="C67" s="13" t="s">
         <v>109</v>
       </c>
-      <c r="D57" s="13" t="s">
-        <v>188</v>
-      </c>
-      <c r="E57" s="31"/>
-      <c r="F57" s="13" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A58" s="98"/>
-      <c r="B58" s="93"/>
-      <c r="C58" s="13" t="s">
-        <v>128</v>
-      </c>
-      <c r="D58" s="13" t="s">
-        <v>126</v>
-      </c>
-      <c r="E58" s="31"/>
-      <c r="F58" s="13" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A59" s="98"/>
-      <c r="B59" s="93"/>
-      <c r="C59" s="13" t="s">
-        <v>129</v>
-      </c>
-      <c r="D59" s="13" t="s">
-        <v>127</v>
-      </c>
-      <c r="E59" s="33"/>
-      <c r="F59" s="13" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A60" s="98"/>
-      <c r="B60" s="93"/>
-      <c r="C60" s="13" t="s">
-        <v>143</v>
-      </c>
-      <c r="D60" s="13" t="s">
-        <v>147</v>
-      </c>
-      <c r="E60" s="31"/>
-      <c r="F60" s="13" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A61" s="98"/>
-      <c r="B61" s="93"/>
-      <c r="C61" s="13" t="s">
-        <v>157</v>
-      </c>
-      <c r="D61" s="13" t="s">
-        <v>159</v>
-      </c>
-      <c r="E61" s="33"/>
-      <c r="F61" s="13" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A62" s="98"/>
-      <c r="B62" s="93"/>
-      <c r="C62" s="13" t="s">
-        <v>200</v>
-      </c>
-      <c r="D62" s="13" t="s">
-        <v>204</v>
-      </c>
-      <c r="E62" s="33"/>
-      <c r="F62" s="13" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A63" s="98"/>
-      <c r="B63" s="93"/>
-      <c r="C63" s="13" t="s">
-        <v>169</v>
-      </c>
-      <c r="D63" s="13" t="s">
-        <v>172</v>
-      </c>
-      <c r="E63" s="33"/>
-      <c r="F63" s="13" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A64" s="98"/>
-      <c r="B64" s="93"/>
-      <c r="C64" s="13" t="s">
-        <v>192</v>
-      </c>
-      <c r="D64" s="13" t="s">
-        <v>196</v>
-      </c>
-      <c r="E64" s="33"/>
-      <c r="F64" s="13" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="65" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A65" s="104"/>
-      <c r="B65" s="107"/>
-      <c r="C65" s="41"/>
-      <c r="D65" s="41"/>
-      <c r="E65" s="42"/>
-      <c r="F65" s="41"/>
-    </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A66" s="97" t="s">
-        <v>73</v>
-      </c>
-      <c r="B66" s="99" t="s">
-        <v>74</v>
-      </c>
-      <c r="C66" s="26" t="s">
-        <v>119</v>
-      </c>
-      <c r="D66" s="26" t="s">
-        <v>118</v>
-      </c>
-      <c r="E66" s="39"/>
-      <c r="F66" s="26" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A67" s="98"/>
-      <c r="B67" s="93"/>
-      <c r="C67" s="13" t="s">
-        <v>155</v>
-      </c>
       <c r="D67" s="13" t="s">
-        <v>154</v>
+        <v>187</v>
       </c>
       <c r="E67" s="31"/>
       <c r="F67" s="13" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A68" s="111"/>
+      <c r="B68" s="101"/>
+      <c r="C68" s="13" t="s">
+        <v>128</v>
+      </c>
+      <c r="D68" s="13" t="s">
+        <v>126</v>
+      </c>
+      <c r="E68" s="31"/>
+      <c r="F68" s="13" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A69" s="111"/>
+      <c r="B69" s="101"/>
+      <c r="C69" s="13" t="s">
+        <v>129</v>
+      </c>
+      <c r="D69" s="13" t="s">
+        <v>127</v>
+      </c>
+      <c r="E69" s="33"/>
+      <c r="F69" s="13" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A70" s="111"/>
+      <c r="B70" s="101"/>
+      <c r="C70" s="13" t="s">
+        <v>143</v>
+      </c>
+      <c r="D70" s="13" t="s">
+        <v>147</v>
+      </c>
+      <c r="E70" s="31"/>
+      <c r="F70" s="13" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A71" s="111"/>
+      <c r="B71" s="101"/>
+      <c r="C71" s="13" t="s">
+        <v>157</v>
+      </c>
+      <c r="D71" s="13" t="s">
+        <v>159</v>
+      </c>
+      <c r="E71" s="33"/>
+      <c r="F71" s="13" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A68" s="98"/>
-      <c r="B68" s="94"/>
-      <c r="E68" s="31"/>
-    </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A69" s="98"/>
-      <c r="B69" s="106" t="s">
-        <v>4</v>
-      </c>
-      <c r="C69" s="35" t="s">
-        <v>98</v>
-      </c>
-      <c r="D69" s="35" t="s">
-        <v>101</v>
-      </c>
-      <c r="E69" s="40"/>
-      <c r="F69" s="35" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A70" s="98"/>
-      <c r="B70" s="95"/>
-      <c r="C70" s="13" t="s">
-        <v>109</v>
-      </c>
-      <c r="D70" s="13" t="s">
-        <v>111</v>
-      </c>
-      <c r="E70" s="43"/>
-      <c r="F70" s="13" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A71" s="98"/>
-      <c r="B71" s="95"/>
-      <c r="C71" s="13" t="s">
-        <v>124</v>
-      </c>
-      <c r="D71" s="13" t="s">
-        <v>123</v>
-      </c>
-      <c r="E71" s="43"/>
-      <c r="F71" s="13" t="s">
-        <v>120</v>
-      </c>
-    </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A72" s="98"/>
-      <c r="B72" s="95"/>
+      <c r="A72" s="111"/>
+      <c r="B72" s="101"/>
       <c r="C72" s="13" t="s">
-        <v>143</v>
+        <v>199</v>
       </c>
       <c r="D72" s="13" t="s">
-        <v>146</v>
-      </c>
-      <c r="E72" s="31"/>
+        <v>203</v>
+      </c>
+      <c r="E72" s="33"/>
       <c r="F72" s="13" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A73" s="111"/>
+      <c r="B73" s="101"/>
+      <c r="C73" s="13" t="s">
+        <v>169</v>
+      </c>
+      <c r="D73" s="13" t="s">
+        <v>172</v>
+      </c>
+      <c r="E73" s="33"/>
+      <c r="F73" s="13" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A73" s="98"/>
-      <c r="B73" s="95"/>
-      <c r="C73" s="13" t="s">
-        <v>157</v>
-      </c>
-      <c r="D73" s="13" t="s">
-        <v>158</v>
-      </c>
-      <c r="E73" s="34"/>
-      <c r="F73" s="13" t="s">
-        <v>151</v>
-      </c>
-    </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A74" s="98"/>
-      <c r="B74" s="95"/>
+      <c r="A74" s="111"/>
+      <c r="B74" s="101"/>
       <c r="C74" s="13" t="s">
-        <v>163</v>
+        <v>191</v>
       </c>
       <c r="D74" s="13" t="s">
-        <v>164</v>
-      </c>
-      <c r="E74" s="31"/>
+        <v>195</v>
+      </c>
+      <c r="E74" s="33"/>
       <c r="F74" s="13" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A75" s="98"/>
-      <c r="B75" s="95"/>
-      <c r="C75" s="13" t="s">
-        <v>200</v>
-      </c>
-      <c r="D75" s="13" t="s">
-        <v>202</v>
-      </c>
-      <c r="E75" s="31"/>
-      <c r="F75" s="13" t="s">
-        <v>151</v>
-      </c>
+    <row r="75" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A75" s="112"/>
+      <c r="B75" s="118"/>
+      <c r="C75" s="41"/>
+      <c r="D75" s="41"/>
+      <c r="E75" s="42"/>
+      <c r="F75" s="41"/>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A76" s="98"/>
-      <c r="B76" s="95"/>
-      <c r="C76" s="13" t="s">
-        <v>169</v>
-      </c>
-      <c r="D76" s="13" t="s">
-        <v>171</v>
-      </c>
-      <c r="E76" s="33"/>
-      <c r="F76" s="13" t="s">
-        <v>142</v>
+      <c r="A76" s="109" t="s">
+        <v>73</v>
+      </c>
+      <c r="B76" s="108" t="s">
+        <v>74</v>
+      </c>
+      <c r="C76" s="26" t="s">
+        <v>119</v>
+      </c>
+      <c r="D76" s="26" t="s">
+        <v>118</v>
+      </c>
+      <c r="E76" s="39"/>
+      <c r="F76" s="26" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A77" s="98"/>
-      <c r="B77" s="95"/>
+      <c r="A77" s="111"/>
+      <c r="B77" s="101"/>
       <c r="C77" s="13" t="s">
-        <v>192</v>
+        <v>155</v>
       </c>
       <c r="D77" s="13" t="s">
-        <v>194</v>
-      </c>
-      <c r="E77" s="33"/>
+        <v>154</v>
+      </c>
+      <c r="E77" s="31"/>
       <c r="F77" s="13" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A78" s="98"/>
-      <c r="B78" s="111"/>
+      <c r="A78" s="111"/>
+      <c r="B78" s="102"/>
+      <c r="E78" s="31"/>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A79" s="98"/>
-      <c r="B79" s="106" t="s">
-        <v>5</v>
+      <c r="A79" s="111"/>
+      <c r="B79" s="113" t="s">
+        <v>4</v>
       </c>
       <c r="C79" s="35" t="s">
         <v>98</v>
       </c>
       <c r="D79" s="35" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="E79" s="40"/>
       <c r="F79" s="35" t="s">
@@ -4306,13 +4553,13 @@
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A80" s="98"/>
-      <c r="B80" s="95"/>
+      <c r="A80" s="111"/>
+      <c r="B80" s="103"/>
       <c r="C80" s="13" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D80" s="13" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="E80" s="43"/>
       <c r="F80" s="13" t="s">
@@ -4320,13 +4567,13 @@
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A81" s="98"/>
-      <c r="B81" s="95"/>
+      <c r="A81" s="111"/>
+      <c r="B81" s="103"/>
       <c r="C81" s="13" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D81" s="13" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="E81" s="43"/>
       <c r="F81" s="13" t="s">
@@ -4334,27 +4581,27 @@
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A82" s="98"/>
-      <c r="B82" s="95"/>
+      <c r="A82" s="111"/>
+      <c r="B82" s="103"/>
       <c r="C82" s="13" t="s">
         <v>143</v>
       </c>
       <c r="D82" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="E82" s="43"/>
+        <v>146</v>
+      </c>
+      <c r="E82" s="31"/>
       <c r="F82" s="13" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A83" s="98"/>
-      <c r="B83" s="95"/>
+      <c r="A83" s="111"/>
+      <c r="B83" s="103"/>
       <c r="C83" s="13" t="s">
         <v>157</v>
       </c>
       <c r="D83" s="13" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="E83" s="34"/>
       <c r="F83" s="13" t="s">
@@ -4362,41 +4609,41 @@
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A84" s="98"/>
-      <c r="B84" s="95"/>
+      <c r="A84" s="111"/>
+      <c r="B84" s="103"/>
       <c r="C84" s="13" t="s">
         <v>163</v>
       </c>
       <c r="D84" s="13" t="s">
-        <v>162</v>
-      </c>
-      <c r="E84" s="44"/>
+        <v>164</v>
+      </c>
+      <c r="E84" s="31"/>
       <c r="F84" s="13" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A85" s="98"/>
-      <c r="B85" s="95"/>
+      <c r="A85" s="111"/>
+      <c r="B85" s="103"/>
       <c r="C85" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="D85" s="13" t="s">
         <v>201</v>
       </c>
-      <c r="E85" s="44"/>
+      <c r="E85" s="31"/>
       <c r="F85" s="13" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A86" s="98"/>
-      <c r="B86" s="95"/>
+      <c r="A86" s="111"/>
+      <c r="B86" s="103"/>
       <c r="C86" s="13" t="s">
         <v>169</v>
       </c>
       <c r="D86" s="13" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="E86" s="33"/>
       <c r="F86" s="13" t="s">
@@ -4404,10 +4651,10 @@
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A87" s="98"/>
-      <c r="B87" s="95"/>
+      <c r="A87" s="111"/>
+      <c r="B87" s="103"/>
       <c r="C87" s="13" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D87" s="13" t="s">
         <v>193</v>
@@ -4417,553 +4664,719 @@
         <v>151</v>
       </c>
     </row>
-    <row r="88" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A88" s="104"/>
-      <c r="B88" s="112"/>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A88" s="111"/>
+      <c r="B88" s="114"/>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A89" s="97" t="s">
-        <v>77</v>
-      </c>
-      <c r="B89" s="99" t="s">
-        <v>74</v>
-      </c>
-      <c r="C89" s="26" t="s">
-        <v>131</v>
-      </c>
-      <c r="D89" s="26" t="s">
-        <v>130</v>
-      </c>
-      <c r="E89" s="30"/>
-      <c r="F89" s="26" t="s">
+      <c r="A89" s="111"/>
+      <c r="B89" s="113" t="s">
+        <v>5</v>
+      </c>
+      <c r="C89" s="35" t="s">
+        <v>98</v>
+      </c>
+      <c r="D89" s="35" t="s">
+        <v>103</v>
+      </c>
+      <c r="E89" s="40"/>
+      <c r="F89" s="35" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A90" s="111"/>
+      <c r="B90" s="103"/>
+      <c r="C90" s="13" t="s">
+        <v>110</v>
+      </c>
+      <c r="D90" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="E90" s="43"/>
+      <c r="F90" s="13" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A91" s="111"/>
+      <c r="B91" s="103"/>
+      <c r="C91" s="13" t="s">
+        <v>122</v>
+      </c>
+      <c r="D91" s="13" t="s">
+        <v>121</v>
+      </c>
+      <c r="E91" s="43"/>
+      <c r="F91" s="13" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A90" s="110"/>
-      <c r="B90" s="96"/>
-      <c r="C90" s="52" t="s">
-        <v>232</v>
-      </c>
-      <c r="D90" s="52" t="s">
-        <v>231</v>
-      </c>
-      <c r="E90" s="53"/>
-      <c r="F90" s="52" t="s">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A92" s="111"/>
+      <c r="B92" s="103"/>
+      <c r="C92" s="13" t="s">
+        <v>143</v>
+      </c>
+      <c r="D92" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E92" s="43"/>
+      <c r="F92" s="13" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A93" s="111"/>
+      <c r="B93" s="103"/>
+      <c r="C93" s="13" t="s">
+        <v>157</v>
+      </c>
+      <c r="D93" s="13" t="s">
+        <v>156</v>
+      </c>
+      <c r="E93" s="34"/>
+      <c r="F93" s="13" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A91" s="98"/>
-      <c r="B91" s="96"/>
-      <c r="C91" s="52" t="s">
-        <v>152</v>
-      </c>
-      <c r="D91" s="52" t="s">
-        <v>149</v>
-      </c>
-      <c r="E91" s="53"/>
-      <c r="F91" s="52" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A92" s="98"/>
-      <c r="B92" s="94"/>
-      <c r="C92" s="37"/>
-      <c r="D92" s="37"/>
-      <c r="E92" s="38"/>
-      <c r="F92" s="37"/>
-    </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A93" s="98"/>
-      <c r="B93" s="92" t="s">
-        <v>332</v>
-      </c>
-      <c r="C93" s="13" t="s">
-        <v>333</v>
-      </c>
-      <c r="D93" s="13" t="s">
-        <v>334</v>
-      </c>
-      <c r="E93" s="33"/>
-      <c r="F93" s="13" t="s">
-        <v>321</v>
-      </c>
-    </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A94" s="98"/>
-      <c r="B94" s="93"/>
+      <c r="A94" s="111"/>
+      <c r="B94" s="103"/>
       <c r="C94" s="13" t="s">
-        <v>337</v>
+        <v>163</v>
       </c>
       <c r="D94" s="13" t="s">
-        <v>335</v>
-      </c>
-      <c r="E94" s="33"/>
+        <v>162</v>
+      </c>
+      <c r="E94" s="44"/>
       <c r="F94" s="13" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A95" s="98"/>
-      <c r="B95" s="93"/>
+      <c r="A95" s="111"/>
+      <c r="B95" s="103"/>
       <c r="C95" s="13" t="s">
-        <v>338</v>
+        <v>199</v>
       </c>
       <c r="D95" s="13" t="s">
-        <v>336</v>
-      </c>
-      <c r="E95" s="33"/>
+        <v>200</v>
+      </c>
+      <c r="E95" s="44"/>
       <c r="F95" s="13" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A96" s="98"/>
-      <c r="B96" s="94"/>
+      <c r="A96" s="111"/>
+      <c r="B96" s="103"/>
+      <c r="C96" s="13" t="s">
+        <v>169</v>
+      </c>
+      <c r="D96" s="13" t="s">
+        <v>170</v>
+      </c>
       <c r="E96" s="33"/>
+      <c r="F96" s="13" t="s">
+        <v>142</v>
+      </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A97" s="98"/>
-      <c r="B97" s="92" t="s">
+      <c r="A97" s="111"/>
+      <c r="B97" s="103"/>
+      <c r="C97" s="13" t="s">
+        <v>191</v>
+      </c>
+      <c r="D97" s="13" t="s">
+        <v>192</v>
+      </c>
+      <c r="E97" s="33"/>
+      <c r="F97" s="13" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A98" s="112"/>
+      <c r="B98" s="115"/>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A99" s="109" t="s">
+        <v>77</v>
+      </c>
+      <c r="B99" s="108" t="s">
+        <v>74</v>
+      </c>
+      <c r="C99" s="26" t="s">
+        <v>131</v>
+      </c>
+      <c r="D99" s="26" t="s">
+        <v>130</v>
+      </c>
+      <c r="E99" s="30"/>
+      <c r="F99" s="26" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A100" s="110"/>
+      <c r="B100" s="104"/>
+      <c r="C100" s="51" t="s">
+        <v>231</v>
+      </c>
+      <c r="D100" s="51" t="s">
+        <v>230</v>
+      </c>
+      <c r="E100" s="52"/>
+      <c r="F100" s="51" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A101" s="111"/>
+      <c r="B101" s="104"/>
+      <c r="C101" s="51" t="s">
+        <v>152</v>
+      </c>
+      <c r="D101" s="51" t="s">
+        <v>149</v>
+      </c>
+      <c r="E101" s="52"/>
+      <c r="F101" s="51" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A102" s="111"/>
+      <c r="B102" s="102"/>
+      <c r="C102" s="37"/>
+      <c r="D102" s="37"/>
+      <c r="E102" s="38"/>
+      <c r="F102" s="37"/>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A103" s="111"/>
+      <c r="B103" s="100" t="s">
+        <v>331</v>
+      </c>
+      <c r="C103" s="13" t="s">
+        <v>332</v>
+      </c>
+      <c r="D103" s="13" t="s">
+        <v>333</v>
+      </c>
+      <c r="E103" s="33"/>
+      <c r="F103" s="13" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A104" s="111"/>
+      <c r="B104" s="101"/>
+      <c r="C104" s="13" t="s">
+        <v>336</v>
+      </c>
+      <c r="D104" s="13" t="s">
+        <v>334</v>
+      </c>
+      <c r="E104" s="33"/>
+      <c r="F104" s="13" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A105" s="111"/>
+      <c r="B105" s="101"/>
+      <c r="C105" s="13" t="s">
+        <v>337</v>
+      </c>
+      <c r="D105" s="13" t="s">
+        <v>335</v>
+      </c>
+      <c r="E105" s="33"/>
+      <c r="F105" s="13" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A106" s="111"/>
+      <c r="B106" s="102"/>
+      <c r="E106" s="33"/>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A107" s="111"/>
+      <c r="B107" s="100" t="s">
         <v>80</v>
       </c>
-      <c r="C97" s="35" t="s">
+      <c r="C107" s="35" t="s">
         <v>133</v>
       </c>
-      <c r="D97" s="35" t="s">
+      <c r="D107" s="35" t="s">
         <v>132</v>
       </c>
-      <c r="E97" s="40"/>
-      <c r="F97" s="35" t="s">
+      <c r="E107" s="40"/>
+      <c r="F107" s="35" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A98" s="98"/>
-      <c r="B98" s="93"/>
-      <c r="C98" s="13" t="s">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A108" s="111"/>
+      <c r="B108" s="101"/>
+      <c r="C108" s="13" t="s">
         <v>153</v>
       </c>
-      <c r="D98" s="13" t="s">
+      <c r="D108" s="13" t="s">
         <v>150</v>
       </c>
-      <c r="E98" s="33"/>
-      <c r="F98" s="13" t="s">
+      <c r="E108" s="33"/>
+      <c r="F108" s="13" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A99" s="98"/>
-      <c r="B99" s="94"/>
-      <c r="C99" s="37"/>
-      <c r="D99" s="37"/>
-      <c r="E99" s="38"/>
-      <c r="F99" s="37"/>
-    </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A100" s="98"/>
-      <c r="B100" s="100" t="s">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A109" s="111"/>
+      <c r="B109" s="102"/>
+      <c r="C109" s="37"/>
+      <c r="D109" s="37"/>
+      <c r="E109" s="38"/>
+      <c r="F109" s="37"/>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A110" s="111"/>
+      <c r="B110" s="105" t="s">
+        <v>277</v>
+      </c>
+      <c r="C110" s="45" t="s">
+        <v>276</v>
+      </c>
+      <c r="D110" s="45" t="s">
+        <v>279</v>
+      </c>
+      <c r="E110" s="56"/>
+      <c r="F110" s="45" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A111" s="111"/>
+      <c r="B111" s="106"/>
+      <c r="C111" s="45" t="s">
         <v>278</v>
       </c>
-      <c r="C100" s="45" t="s">
-        <v>277</v>
-      </c>
-      <c r="D100" s="45" t="s">
+      <c r="D111" s="45" t="s">
         <v>280</v>
       </c>
-      <c r="E100" s="57"/>
-      <c r="F100" s="45" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A101" s="98"/>
-      <c r="B101" s="101"/>
-      <c r="C101" s="45" t="s">
-        <v>279</v>
-      </c>
-      <c r="D101" s="45" t="s">
-        <v>281</v>
-      </c>
-      <c r="E101" s="57"/>
-      <c r="F101" s="45" t="s">
+      <c r="E111" s="56"/>
+      <c r="F111" s="45" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="102" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A102" s="104"/>
-      <c r="B102" s="109"/>
-      <c r="C102" s="63"/>
-      <c r="D102" s="63"/>
-      <c r="E102" s="64"/>
-      <c r="F102" s="63"/>
-    </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A103" s="97" t="s">
+    <row r="112" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A112" s="112"/>
+      <c r="B112" s="107"/>
+      <c r="C112" s="61"/>
+      <c r="D112" s="61"/>
+      <c r="E112" s="62"/>
+      <c r="F112" s="61"/>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A113" s="109" t="s">
         <v>165</v>
       </c>
-      <c r="B103" s="99" t="s">
+      <c r="B113" s="108" t="s">
         <v>13</v>
       </c>
-      <c r="C103" s="26" t="s">
+      <c r="C113" s="26" t="s">
         <v>175</v>
       </c>
-      <c r="D103" s="26" t="s">
+      <c r="D113" s="26" t="s">
         <v>174</v>
       </c>
-      <c r="E103" s="26"/>
-      <c r="F103" s="26" t="s">
+      <c r="E113" s="26"/>
+      <c r="F113" s="26" t="s">
         <v>142</v>
-      </c>
-    </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A104" s="110"/>
-      <c r="B104" s="93"/>
-      <c r="C104" s="13" t="s">
-        <v>176</v>
-      </c>
-      <c r="D104" s="13" t="s">
-        <v>177</v>
-      </c>
-      <c r="F104" s="13" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A105" s="110"/>
-      <c r="B105" s="94"/>
-      <c r="C105" s="37"/>
-      <c r="D105" s="37"/>
-      <c r="E105" s="37"/>
-      <c r="F105" s="37"/>
-    </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A106" s="110"/>
-      <c r="B106" s="92" t="s">
-        <v>186</v>
-      </c>
-      <c r="C106" s="13" t="s">
-        <v>167</v>
-      </c>
-      <c r="D106" s="13" t="s">
-        <v>166</v>
-      </c>
-      <c r="F106" s="13" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A107" s="110"/>
-      <c r="B107" s="93"/>
-      <c r="C107" s="13" t="s">
-        <v>184</v>
-      </c>
-      <c r="D107" s="13" t="s">
-        <v>178</v>
-      </c>
-      <c r="F107" s="13" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A108" s="110"/>
-      <c r="B108" s="93"/>
-      <c r="D108" s="13" t="s">
-        <v>340</v>
-      </c>
-    </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A109" s="110"/>
-      <c r="B109" s="93"/>
-      <c r="C109" s="13" t="s">
-        <v>180</v>
-      </c>
-      <c r="D109" s="13" t="s">
-        <v>179</v>
-      </c>
-      <c r="F109" s="13" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A110" s="110"/>
-      <c r="B110" s="93"/>
-      <c r="C110" s="13" t="s">
-        <v>182</v>
-      </c>
-      <c r="D110" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="F110" s="13" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A111" s="110"/>
-      <c r="B111" s="93"/>
-      <c r="C111" s="13" t="s">
-        <v>185</v>
-      </c>
-      <c r="D111" s="13" t="s">
-        <v>183</v>
-      </c>
-      <c r="F111" s="13" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A112" s="110"/>
-      <c r="B112" s="93"/>
-      <c r="C112" s="13" t="s">
-        <v>195</v>
-      </c>
-      <c r="D112" s="13" t="s">
-        <v>191</v>
-      </c>
-      <c r="F112" s="13" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A113" s="110"/>
-      <c r="B113" s="92" t="s">
-        <v>210</v>
-      </c>
-      <c r="C113" s="35" t="s">
-        <v>207</v>
-      </c>
-      <c r="D113" s="35" t="s">
-        <v>211</v>
-      </c>
-      <c r="E113" s="35"/>
-      <c r="F113" s="35" t="s">
-        <v>212</v>
       </c>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A114" s="110"/>
-      <c r="B114" s="96"/>
-      <c r="C114" s="52" t="s">
-        <v>208</v>
-      </c>
-      <c r="D114" s="52" t="s">
-        <v>214</v>
-      </c>
-      <c r="E114" s="52"/>
-      <c r="F114" s="52" t="s">
-        <v>212</v>
+      <c r="B114" s="101"/>
+      <c r="C114" s="13" t="s">
+        <v>176</v>
+      </c>
+      <c r="D114" s="13" t="s">
+        <v>177</v>
+      </c>
+      <c r="F114" s="13" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A115" s="110"/>
-      <c r="B115" s="96"/>
-      <c r="C115" s="52" t="s">
-        <v>219</v>
-      </c>
-      <c r="D115" s="52" t="s">
-        <v>218</v>
-      </c>
-      <c r="E115" s="52"/>
-      <c r="F115" s="52" t="s">
-        <v>223</v>
-      </c>
+      <c r="B115" s="102"/>
+      <c r="C115" s="37"/>
+      <c r="D115" s="37"/>
+      <c r="E115" s="37"/>
+      <c r="F115" s="37"/>
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A116" s="110"/>
-      <c r="B116" s="96"/>
-      <c r="C116" s="52" t="s">
-        <v>209</v>
-      </c>
-      <c r="D116" s="52" t="s">
-        <v>213</v>
-      </c>
-      <c r="E116" s="52"/>
-      <c r="F116" s="52" t="s">
-        <v>212</v>
+      <c r="B116" s="100" t="s">
+        <v>185</v>
+      </c>
+      <c r="C116" s="13" t="s">
+        <v>167</v>
+      </c>
+      <c r="D116" s="13" t="s">
+        <v>166</v>
+      </c>
+      <c r="F116" s="13" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A117" s="110"/>
-      <c r="B117" s="96"/>
-      <c r="C117" s="52" t="s">
-        <v>341</v>
-      </c>
-      <c r="D117" s="52" t="s">
-        <v>342</v>
-      </c>
-      <c r="E117" s="52"/>
-      <c r="F117" s="52" t="s">
-        <v>345</v>
+      <c r="B117" s="101"/>
+      <c r="C117" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="D117" s="13" t="s">
+        <v>339</v>
+      </c>
+      <c r="F117" s="13" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A118" s="110"/>
-      <c r="B118" s="96"/>
-      <c r="C118" s="52" t="s">
-        <v>221</v>
-      </c>
-      <c r="D118" s="52" t="s">
-        <v>220</v>
-      </c>
-      <c r="E118" s="52"/>
-      <c r="F118" s="52" t="s">
-        <v>222</v>
+      <c r="B118" s="101"/>
+      <c r="C118" s="13" t="s">
+        <v>179</v>
+      </c>
+      <c r="D118" s="13" t="s">
+        <v>178</v>
+      </c>
+      <c r="F118" s="13" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A119" s="110"/>
-      <c r="B119" s="96"/>
-      <c r="C119" s="52" t="s">
-        <v>225</v>
-      </c>
-      <c r="D119" s="52" t="s">
-        <v>215</v>
-      </c>
-      <c r="E119" s="52"/>
-      <c r="F119" s="52" t="s">
-        <v>216</v>
+      <c r="B119" s="101"/>
+      <c r="C119" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="D119" s="13" t="s">
+        <v>180</v>
+      </c>
+      <c r="F119" s="13" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A120" s="110"/>
-      <c r="B120" s="96"/>
-      <c r="C120" s="52" t="s">
-        <v>206</v>
+      <c r="B120" s="101"/>
+      <c r="C120" s="13" t="s">
+        <v>184</v>
       </c>
       <c r="D120" s="13" t="s">
-        <v>224</v>
-      </c>
-      <c r="E120" s="52"/>
-      <c r="F120" s="52" t="s">
-        <v>216</v>
+        <v>182</v>
+      </c>
+      <c r="F120" s="13" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A121" s="110"/>
-      <c r="B121" s="96"/>
-      <c r="C121" s="65" t="s">
-        <v>282</v>
-      </c>
-      <c r="D121" s="65" t="s">
-        <v>283</v>
-      </c>
-      <c r="E121" s="65"/>
-      <c r="F121" s="45" t="s">
-        <v>216</v>
+      <c r="B121" s="101"/>
+      <c r="C121" s="13" t="s">
+        <v>194</v>
+      </c>
+      <c r="D121" s="13" t="s">
+        <v>190</v>
+      </c>
+      <c r="F121" s="13" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A122" s="110"/>
-      <c r="B122" s="96"/>
-      <c r="C122" s="65" t="s">
-        <v>285</v>
-      </c>
-      <c r="D122" s="65" t="s">
-        <v>284</v>
-      </c>
-      <c r="E122" s="65"/>
-      <c r="F122" s="65" t="s">
-        <v>217</v>
-      </c>
+      <c r="B122" s="101"/>
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A123" s="110"/>
-      <c r="B123" s="92" t="s">
-        <v>226</v>
+      <c r="B123" s="100" t="s">
+        <v>209</v>
       </c>
       <c r="C123" s="35" t="s">
-        <v>228</v>
+        <v>206</v>
       </c>
       <c r="D123" s="35" t="s">
-        <v>227</v>
+        <v>210</v>
       </c>
       <c r="E123" s="35"/>
       <c r="F123" s="35" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A124" s="110"/>
-      <c r="B124" s="96"/>
-      <c r="C124" s="52" t="s">
-        <v>343</v>
-      </c>
-      <c r="D124" s="52" t="s">
-        <v>344</v>
-      </c>
-      <c r="E124" s="52"/>
-      <c r="F124" s="52" t="s">
-        <v>345</v>
+      <c r="B124" s="104"/>
+      <c r="C124" s="51" t="s">
+        <v>207</v>
+      </c>
+      <c r="D124" s="51" t="s">
+        <v>213</v>
+      </c>
+      <c r="E124" s="51"/>
+      <c r="F124" s="51" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A125" s="110"/>
-      <c r="B125" s="96"/>
-      <c r="C125" s="52" t="s">
-        <v>229</v>
-      </c>
-      <c r="D125" s="52" t="s">
-        <v>230</v>
-      </c>
-      <c r="E125" s="52"/>
-      <c r="F125" s="52" t="s">
-        <v>216</v>
+      <c r="B125" s="104"/>
+      <c r="C125" s="51" t="s">
+        <v>218</v>
+      </c>
+      <c r="D125" s="51" t="s">
+        <v>217</v>
+      </c>
+      <c r="E125" s="51"/>
+      <c r="F125" s="51" t="s">
+        <v>222</v>
       </c>
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A126" s="110"/>
-      <c r="B126" s="96"/>
-      <c r="C126" s="65" t="s">
-        <v>286</v>
-      </c>
-      <c r="D126" s="65" t="s">
-        <v>287</v>
-      </c>
-      <c r="E126" s="65"/>
-      <c r="F126" s="65" t="s">
-        <v>216</v>
+      <c r="B126" s="104"/>
+      <c r="C126" s="51" t="s">
+        <v>208</v>
+      </c>
+      <c r="D126" s="51" t="s">
+        <v>212</v>
+      </c>
+      <c r="E126" s="51"/>
+      <c r="F126" s="51" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A127" s="110"/>
-      <c r="B127" s="96"/>
-      <c r="C127" s="45" t="s">
-        <v>288</v>
-      </c>
-      <c r="D127" s="45" t="s">
-        <v>339</v>
-      </c>
-      <c r="E127" s="45"/>
-      <c r="F127" s="45" t="s">
-        <v>217</v>
+      <c r="B127" s="104"/>
+      <c r="C127" s="51" t="s">
+        <v>340</v>
+      </c>
+      <c r="D127" s="51" t="s">
+        <v>341</v>
+      </c>
+      <c r="E127" s="51"/>
+      <c r="F127" s="51" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="128" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A128" s="110"/>
+      <c r="B128" s="104"/>
+      <c r="C128" s="63" t="s">
+        <v>364</v>
+      </c>
+      <c r="D128" s="63" t="s">
+        <v>365</v>
+      </c>
+      <c r="E128" s="63"/>
+      <c r="F128" s="51" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="129" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A129" s="110"/>
+      <c r="B129" s="104"/>
+      <c r="C129" s="45" t="s">
+        <v>366</v>
+      </c>
+      <c r="D129" s="45" t="s">
+        <v>367</v>
+      </c>
+      <c r="E129" s="45"/>
+      <c r="F129" s="51" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="130" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A130" s="110"/>
+      <c r="B130" s="104"/>
+      <c r="C130" s="51" t="s">
+        <v>220</v>
+      </c>
+      <c r="D130" s="51" t="s">
+        <v>219</v>
+      </c>
+      <c r="E130" s="51"/>
+      <c r="F130" s="51" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="131" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A131" s="110"/>
+      <c r="B131" s="104"/>
+      <c r="C131" s="51" t="s">
+        <v>224</v>
+      </c>
+      <c r="D131" s="51" t="s">
+        <v>214</v>
+      </c>
+      <c r="E131" s="51"/>
+      <c r="F131" s="51" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="132" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A132" s="110"/>
+      <c r="B132" s="104"/>
+      <c r="C132" s="51" t="s">
+        <v>205</v>
+      </c>
+      <c r="D132" s="13" t="s">
+        <v>223</v>
+      </c>
+      <c r="E132" s="51"/>
+      <c r="F132" s="51" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="133" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A133" s="110"/>
+      <c r="B133" s="104"/>
+      <c r="C133" s="63" t="s">
+        <v>281</v>
+      </c>
+      <c r="D133" s="63" t="s">
+        <v>282</v>
+      </c>
+      <c r="E133" s="63"/>
+      <c r="F133" s="45" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="134" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A134" s="110"/>
+      <c r="B134" s="104"/>
+      <c r="C134" s="63" t="s">
+        <v>284</v>
+      </c>
+      <c r="D134" s="63" t="s">
+        <v>283</v>
+      </c>
+      <c r="E134" s="63"/>
+      <c r="F134" s="63" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="135" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A135" s="110"/>
+      <c r="B135" s="104"/>
+      <c r="C135" s="63"/>
+      <c r="D135" s="63"/>
+      <c r="E135" s="63"/>
+      <c r="F135" s="63"/>
+    </row>
+    <row r="136" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A136" s="110"/>
+      <c r="B136" s="100" t="s">
+        <v>225</v>
+      </c>
+      <c r="C136" s="35" t="s">
+        <v>227</v>
+      </c>
+      <c r="D136" s="35" t="s">
+        <v>226</v>
+      </c>
+      <c r="E136" s="35"/>
+      <c r="F136" s="35" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="137" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A137" s="110"/>
+      <c r="B137" s="104"/>
+      <c r="C137" s="51" t="s">
+        <v>342</v>
+      </c>
+      <c r="D137" s="51" t="s">
+        <v>343</v>
+      </c>
+      <c r="E137" s="51"/>
+      <c r="F137" s="51" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="138" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A138" s="110"/>
+      <c r="B138" s="104"/>
+      <c r="C138" s="51" t="s">
+        <v>228</v>
+      </c>
+      <c r="D138" s="51" t="s">
+        <v>229</v>
+      </c>
+      <c r="E138" s="51"/>
+      <c r="F138" s="51" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="139" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A139" s="110"/>
+      <c r="B139" s="104"/>
+      <c r="C139" s="63" t="s">
+        <v>285</v>
+      </c>
+      <c r="D139" s="63" t="s">
+        <v>286</v>
+      </c>
+      <c r="E139" s="63"/>
+      <c r="F139" s="63" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="140" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A140" s="110"/>
+      <c r="B140" s="104"/>
+      <c r="C140" s="45" t="s">
+        <v>287</v>
+      </c>
+      <c r="D140" s="45" t="s">
+        <v>338</v>
+      </c>
+      <c r="E140" s="45"/>
+      <c r="F140" s="45" t="s">
+        <v>216</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="22">
-    <mergeCell ref="B100:B102"/>
-    <mergeCell ref="B66:B68"/>
-    <mergeCell ref="B106:B112"/>
-    <mergeCell ref="B123:B127"/>
-    <mergeCell ref="A103:A127"/>
-    <mergeCell ref="B113:B122"/>
-    <mergeCell ref="B103:B105"/>
-    <mergeCell ref="A66:A88"/>
-    <mergeCell ref="B69:B78"/>
-    <mergeCell ref="B79:B88"/>
-    <mergeCell ref="A89:A102"/>
-    <mergeCell ref="B97:B99"/>
-    <mergeCell ref="B89:B92"/>
-    <mergeCell ref="B93:B96"/>
+  <mergeCells count="23">
     <mergeCell ref="A2:A43"/>
     <mergeCell ref="B2:B11"/>
     <mergeCell ref="B12:B22"/>
     <mergeCell ref="B33:B43"/>
-    <mergeCell ref="A44:A65"/>
+    <mergeCell ref="A44:A75"/>
+    <mergeCell ref="B64:B75"/>
+    <mergeCell ref="B23:B32"/>
     <mergeCell ref="B44:B53"/>
-    <mergeCell ref="B54:B65"/>
-    <mergeCell ref="B23:B32"/>
+    <mergeCell ref="B54:B63"/>
+    <mergeCell ref="B110:B112"/>
+    <mergeCell ref="B76:B78"/>
+    <mergeCell ref="B116:B122"/>
+    <mergeCell ref="B136:B140"/>
+    <mergeCell ref="A113:A140"/>
+    <mergeCell ref="B123:B135"/>
+    <mergeCell ref="B113:B115"/>
+    <mergeCell ref="A76:A98"/>
+    <mergeCell ref="B79:B88"/>
+    <mergeCell ref="B89:B98"/>
+    <mergeCell ref="A99:A112"/>
+    <mergeCell ref="B107:B109"/>
+    <mergeCell ref="B99:B102"/>
+    <mergeCell ref="B103:B106"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -4975,56 +5388,56 @@
   <dimension ref="B1:B31"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="11.5546875" style="66"/>
+    <col min="2" max="2" width="11.5546875" style="64"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B1" s="66" t="s">
+      <c r="B1" s="64" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="2" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B2" s="64" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="22" spans="2:2" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B22" s="67" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="24" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B24" s="64" t="s">
         <v>295</v>
       </c>
     </row>
-    <row r="2" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B2" s="66" t="s">
+    <row r="26" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B26" s="64" t="s">
         <v>289</v>
       </c>
     </row>
-    <row r="22" spans="2:2" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="B22" s="69" t="s">
-        <v>297</v>
-      </c>
-    </row>
-    <row r="24" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B24" s="66" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="26" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B26" s="66" t="s">
+    <row r="27" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B27" s="64" t="s">
         <v>290</v>
       </c>
     </row>
-    <row r="27" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B27" s="66" t="s">
+    <row r="28" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B28" s="64" t="s">
         <v>291</v>
       </c>
     </row>
-    <row r="28" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B28" s="66" t="s">
+    <row r="29" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B29" s="65" t="s">
         <v>292</v>
       </c>
     </row>
-    <row r="29" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B29" s="67" t="s">
+    <row r="30" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B30" s="66" t="s">
         <v>293</v>
       </c>
     </row>
-    <row r="30" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B30" s="68" t="s">
-        <v>294</v>
-      </c>
-    </row>
     <row r="31" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B31" s="68"/>
+      <c r="B31" s="66"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>